<commit_message>
state: 2026-10-11 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5122,7 +5122,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6506,7 +6506,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6678,7 +6678,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6742,7 +6742,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6806,7 +6806,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -7242,7 +7242,7 @@
       </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K127" s="2" t="inlineStr"/>
@@ -8010,7 +8010,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8074,12 +8074,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8090,7 +8090,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>826b577fecaf22bbf65c9544168d1dd82dd44e910b60182e7014015b6c62f6e3</t>
+          <t>611b74bda6c4acf7864b7d92bcaeec9665e1422d7ed8589359065885a625d774</t>
         </is>
       </c>
     </row>
@@ -8142,7 +8142,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8210,7 +8210,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8610,7 +8610,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8750,7 +8750,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8878,7 +8878,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8946,7 +8946,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10710,7 +10710,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10890,7 +10890,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10958,7 +10958,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11030,7 +11030,7 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
@@ -11102,7 +11102,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11174,7 +11174,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11246,7 +11246,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11318,7 +11318,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11390,7 +11390,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11458,7 +11458,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11526,7 +11526,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11594,7 +11594,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11666,7 +11666,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11734,7 +11734,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11806,7 +11806,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11878,7 +11878,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12010,12 +12010,12 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -12030,7 +12030,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>abdcb5c9c9ba2fec3bbc78a104a53261117b2fc19cc2510708187da1cc60737f</t>
+          <t>b2a60b2bda13220281b4129225034a4c70848f134bae8af314dc185d5619e5f6</t>
         </is>
       </c>
     </row>
@@ -12082,7 +12082,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12150,7 +12150,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12222,7 +12222,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12518,7 +12518,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12766,7 +12766,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12834,7 +12834,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12902,7 +12902,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13094,7 +13094,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr"/>
@@ -13162,7 +13162,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr"/>
@@ -13230,7 +13230,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13298,7 +13298,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13366,7 +13366,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13434,7 +13434,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13558,7 +13558,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13630,7 +13630,7 @@
       </c>
       <c r="J232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K232" s="2" t="inlineStr"/>
@@ -13870,10 +13870,14 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
-        </is>
-      </c>
-      <c r="K236" s="2" t="inlineStr"/>
+          <t>2026-10-11T14:09:30+00:00</t>
+        </is>
+      </c>
+      <c r="K236" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T14:09:30+00:00</t>
+        </is>
+      </c>
       <c r="L236" s="2" t="inlineStr">
         <is>
           <t>2026-09-30</t>
@@ -13886,7 +13890,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>dcdb120dbe3f7a669c69db40787e656451bfafc441a9b3e2b65cd88b960058d8</t>
+          <t>708caf90f6e18492618bc604fecfe3d9257dc624b5a0383d9fb227fa57469373</t>
         </is>
       </c>
     </row>
@@ -18138,7 +18142,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18210,12 +18214,12 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="L313" s="2" t="inlineStr">
@@ -18230,7 +18234,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>13ddb9df9d2cc52fea3f018ba916c3df659388776543d7a21e93141cc8810e77</t>
+          <t>fbef424e915e377aa42c556b18f21302c7c0a69b6585a47749bd0503a124425a</t>
         </is>
       </c>
     </row>
@@ -18282,7 +18286,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18354,7 +18358,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18422,7 +18426,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18490,7 +18494,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18614,7 +18618,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19042,7 +19046,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19110,7 +19114,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19178,7 +19182,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19246,12 +19250,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19266,7 +19270,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>689ff0a10ae8a53468c66dd085c3c06b3e1b65ddcbafd123f1d16236198a2d97</t>
+          <t>02dae79631178666e17934312cf80a28afc58e5f9bc29a15f9c41670b370c71e</t>
         </is>
       </c>
     </row>
@@ -19318,12 +19322,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19338,7 +19342,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>65ecd7c7d703437fcf068b759971925488a3d670b656c1377a2a8bb6da1e33f6</t>
+          <t>fe579b85e1dd26ca58ab1b28bc046809a8c7cd3ec72d1481390704526b112c4c</t>
         </is>
       </c>
     </row>
@@ -19390,12 +19394,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19410,7 +19414,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>37efc8c16173ea0352bc660d406f5c88a1553f458978f2f841e0d7e647eff8c8</t>
+          <t>0e62dc4897689d4f776fe2a65c0b64f93d67582b65c775547de481bba8c28168</t>
         </is>
       </c>
     </row>
@@ -19462,7 +19466,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr"/>
@@ -19586,7 +19590,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19654,7 +19658,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19722,7 +19726,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19790,7 +19794,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr"/>
@@ -19858,7 +19862,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr"/>
@@ -19926,7 +19930,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -19994,7 +19998,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20062,7 +20066,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20130,12 +20134,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20150,7 +20154,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>9b6c8fad2b0c95f685bac8bf6d888e13b5d47c583146a86af8b847c5d3f17d6a</t>
+          <t>4f99673d3cb28d104bb2c867f58203f1b2458a39cdf9cc3173660c919091c63e</t>
         </is>
       </c>
     </row>
@@ -20318,7 +20322,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr"/>
@@ -20386,7 +20390,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20454,7 +20458,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20522,7 +20526,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20590,7 +20594,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20658,7 +20662,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20726,7 +20730,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20794,7 +20798,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -21253,7 +21257,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -21291,7 +21295,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -21333,7 +21337,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -21371,7 +21375,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -21409,7 +21413,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -21447,7 +21451,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -21485,7 +21489,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -21527,7 +21531,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -21565,7 +21569,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -21607,7 +21611,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -21649,7 +21653,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -21691,7 +21695,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -21733,7 +21737,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -21775,7 +21779,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -21817,7 +21821,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -21859,7 +21863,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -21901,7 +21905,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -21943,7 +21947,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -21985,7 +21989,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -22027,7 +22031,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -22069,7 +22073,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -22111,7 +22115,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -22149,7 +22153,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -22191,7 +22195,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -22229,7 +22233,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -22271,7 +22275,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -22313,7 +22317,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -22355,7 +22359,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -22397,7 +22401,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -22439,7 +22443,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -22477,7 +22481,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -22515,7 +22519,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -22553,7 +22557,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -22595,7 +22599,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -22637,7 +22641,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -22675,7 +22679,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -22713,7 +22717,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -22755,7 +22759,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -22793,7 +22797,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -22835,7 +22839,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -22873,7 +22877,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -22911,7 +22915,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -22953,7 +22957,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -22991,7 +22995,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -23029,7 +23033,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -23067,7 +23071,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -23109,7 +23113,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -23147,7 +23151,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -23189,7 +23193,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -23231,7 +23235,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -23273,7 +23277,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -23315,7 +23319,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -23353,7 +23357,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -23391,7 +23395,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -23429,7 +23433,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -23471,7 +23475,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -23509,7 +23513,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -23551,7 +23555,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -23593,7 +23597,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -23631,7 +23635,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -23673,7 +23677,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -23715,7 +23719,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -23753,7 +23757,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -23795,7 +23799,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -23833,7 +23837,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -23875,7 +23879,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -23917,7 +23921,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -23959,7 +23963,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -23997,7 +24001,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -24035,7 +24039,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -24073,7 +24077,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -24111,7 +24115,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -24149,7 +24153,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -24191,7 +24195,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -24229,7 +24233,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -24267,7 +24271,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -24309,7 +24313,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -24347,7 +24351,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -24389,7 +24393,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -24427,7 +24431,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -24469,7 +24473,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -24507,7 +24511,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -24545,7 +24549,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -24587,7 +24591,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -24933,7 +24937,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -24975,7 +24979,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -25017,7 +25021,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -25059,7 +25063,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -25101,7 +25105,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -25143,7 +25147,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -25185,7 +25189,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -25227,7 +25231,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -25269,7 +25273,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -25311,7 +25315,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -25353,7 +25357,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -25395,7 +25399,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -25437,7 +25441,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -25479,7 +25483,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -25521,7 +25525,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -25563,7 +25567,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -25605,7 +25609,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -25647,7 +25651,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -25689,7 +25693,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -25731,7 +25735,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -25773,7 +25777,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -25815,7 +25819,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -25857,7 +25861,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -25899,7 +25903,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -25941,7 +25945,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -25983,7 +25987,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -26025,12 +26029,12 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
@@ -26067,7 +26071,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -26109,7 +26113,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -26151,7 +26155,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -26193,7 +26197,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -26235,7 +26239,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -26277,7 +26281,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -26320,7 +26324,7 @@
       <c r="F127" s="2" t="inlineStr"/>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
@@ -26357,7 +26361,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -26399,7 +26403,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -26441,7 +26445,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -26479,7 +26483,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -26521,7 +26525,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -26563,7 +26567,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -26605,7 +26609,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -26647,7 +26651,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -26689,7 +26693,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -26731,7 +26735,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -26773,7 +26777,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -26815,7 +26819,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -26857,12 +26861,12 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
@@ -26899,7 +26903,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -26941,7 +26945,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -26983,7 +26987,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -27025,7 +27029,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -27067,7 +27071,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -27109,7 +27113,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -27151,7 +27155,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -27193,7 +27197,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -27235,7 +27239,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -27277,7 +27281,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -27319,7 +27323,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -27361,7 +27365,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -27403,7 +27407,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -27445,7 +27449,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -27487,7 +27491,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -27529,7 +27533,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -27571,7 +27575,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -27613,7 +27617,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -27655,7 +27659,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -27697,7 +27701,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -27739,7 +27743,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -27781,7 +27785,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -27823,7 +27827,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -27865,7 +27869,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -27907,7 +27911,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -27949,12 +27953,12 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -27991,7 +27995,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -28033,7 +28037,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -28075,7 +28079,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -28117,7 +28121,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -28159,7 +28163,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -28201,7 +28205,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -28243,7 +28247,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -28285,7 +28289,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -28327,7 +28331,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -28369,7 +28373,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -28411,7 +28415,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -28453,7 +28457,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -28495,7 +28499,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -28537,7 +28541,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -28579,7 +28583,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -28621,7 +28625,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -28663,7 +28667,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -28705,7 +28709,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -28747,7 +28751,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -28789,7 +28793,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -28831,7 +28835,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -28873,7 +28877,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -28915,7 +28919,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -28957,7 +28961,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -28999,7 +29003,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -29041,7 +29045,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -29083,7 +29087,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -29125,7 +29129,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -29167,7 +29171,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -29209,7 +29213,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -29251,7 +29255,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -29293,7 +29297,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -29335,7 +29339,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -29377,7 +29381,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -29419,7 +29423,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -29461,7 +29465,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -29503,7 +29507,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -29545,7 +29549,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -29587,7 +29591,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -29630,7 +29634,7 @@
       <c r="F206" s="2" t="inlineStr"/>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
@@ -29667,7 +29671,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -29709,7 +29713,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -29751,7 +29755,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -29793,7 +29797,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -29835,7 +29839,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -29877,7 +29881,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -29919,7 +29923,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -29961,7 +29965,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -30003,7 +30007,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -30045,7 +30049,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -30087,7 +30091,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -30129,7 +30133,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -30171,7 +30175,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -30213,7 +30217,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -30255,7 +30259,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -30297,7 +30301,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -30339,7 +30343,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -30381,7 +30385,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -30423,7 +30427,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -30465,7 +30469,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -30507,7 +30511,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -30549,7 +30553,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -30591,7 +30595,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -30633,7 +30637,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -30675,7 +30679,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -30713,7 +30717,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -30755,7 +30759,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -30793,7 +30797,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -30835,7 +30839,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -30877,7 +30881,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -30915,7 +30919,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -30953,7 +30957,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -30991,7 +30995,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -31029,7 +31033,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -31067,7 +31071,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -31105,7 +31109,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -31143,7 +31147,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -31181,7 +31185,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -31223,7 +31227,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -31265,7 +31269,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -31303,7 +31307,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -31341,7 +31345,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -31379,7 +31383,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -31417,7 +31421,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -31455,7 +31459,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-11T14:09:30+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-13 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6510,7 +6510,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7030,7 +7030,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8078,12 +8078,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8094,7 +8094,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>e492967bfb72eb22c8c1db69edfa298b7696624fddd1531b943f22f84691b3e8</t>
+          <t>4fdb256a902dd5e365bbc5b17e1926ae002b72c41495f4174aa01ba95bfe6833</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8614,7 +8614,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8754,7 +8754,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8882,7 +8882,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10714,7 +10714,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10894,7 +10894,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10962,7 +10962,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11034,12 +11034,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11054,7 +11054,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>ac2f317cab483dc04f68f84604495049bdecc47a3d9f8e0893b1e6101ac3557f</t>
+          <t>6f258b6021da8deb3fd5673a7960b1decf7b68e60298e9551a0cd7d0d283823f</t>
         </is>
       </c>
     </row>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11178,12 +11178,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11198,7 +11198,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>a6203a118f5d6b8de9a15576e2f23a74872d781f1b202bd343e05c7c1dbe03cf</t>
+          <t>51081ff037091c08cec9c71a7550226d330f194712f7b732041cc7a53d7bd7ce</t>
         </is>
       </c>
     </row>
@@ -11250,7 +11250,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11462,7 +11462,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11530,7 +11530,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11670,7 +11670,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11738,7 +11738,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11810,7 +11810,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11882,7 +11882,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12014,7 +12014,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>e86c3556d34454e09cb752a904458e89943d5351b97a0ac4a3e015313909eb86</t>
+          <t>abdcb5c9c9ba2fec3bbc78a104a53261117b2fc19cc2510708187da1cc60737f</t>
         </is>
       </c>
     </row>
@@ -12086,7 +12086,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12154,7 +12154,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12174,7 +12174,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
+          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
         </is>
       </c>
     </row>
@@ -12226,7 +12226,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12522,7 +12522,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12770,7 +12770,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12838,7 +12838,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12906,7 +12906,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13098,7 +13098,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr"/>
@@ -13166,7 +13166,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr"/>
@@ -13234,7 +13234,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13302,7 +13302,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13370,7 +13370,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13438,7 +13438,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13562,7 +13562,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13582,7 +13582,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>139bf427923549ed8ee73443000c2ff683bd8d774d550aaee03ba043d2fe6ab4</t>
+          <t>7aac9d9c52a684d194f84c75ea15e8b14fb3a13a5f54f735261a8d39b6d4af67</t>
         </is>
       </c>
     </row>
@@ -13874,12 +13874,12 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11T14:09:30+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>6c91e9807e3b838c1f2d6e61f9207e30013193c8dd6764a026f5a36f5df5e60b</t>
+          <t>507024c4db7ade4ea8ad7eaa8a06520b997f4a551b2c4cb24aa9e27f1ec72a6b</t>
         </is>
       </c>
     </row>
@@ -18146,12 +18146,12 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="L312" s="2" t="inlineStr">
@@ -18166,7 +18166,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>54f57f8f73ad40662374dbfec960a34fd4666e285a941647a51880f38dd2f712</t>
+          <t>698da8062ce0ed7aa726791fe92d7aac4fad77a93b2f894b4a171f512744718d</t>
         </is>
       </c>
     </row>
@@ -18218,12 +18218,12 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11T14:09:30+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="L313" s="2" t="inlineStr">
@@ -18238,7 +18238,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>663dc63dbdd5dca71f6527acca68e18b9f82fc4d762cd1a3d3ae909b4e227631</t>
+          <t>5c737e3ede2a24bb547f6775237cb24a80ca2bb02e8422470ecadb7fb8592a49</t>
         </is>
       </c>
     </row>
@@ -18290,7 +18290,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18362,7 +18362,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18430,7 +18430,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18498,7 +18498,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18622,7 +18622,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19118,7 +19118,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19186,7 +19186,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19254,12 +19254,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19274,7 +19274,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>a11b386bd400a8872f1d78db81bdaf73266475cac91da84bd79f08601ba020a7</t>
+          <t>c590a678e5a4416ad7174591e81c284aa75e9d40f63a7f4879338b6c803d5434</t>
         </is>
       </c>
     </row>
@@ -19326,7 +19326,7 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
@@ -19346,7 +19346,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>0a1124ba8eacbbc839d35494262ea8220cb56d23229e0061fb6f70d21b92b424</t>
+          <t>af79caf88b2de905250c356b07f541452519c0fcf4a9cdea3e413105ed1b1aee</t>
         </is>
       </c>
     </row>
@@ -19398,12 +19398,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11T14:09:30+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19418,7 +19418,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>0bc7fa42e926e70da9eeaa656c202eca7cf31bb798f50c9628c90010b32a602f</t>
+          <t>24be046587768f330df02db27a76008b96240019bee1260aee250963db00bf59</t>
         </is>
       </c>
     </row>
@@ -19470,7 +19470,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr"/>
@@ -19594,7 +19594,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19662,7 +19662,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19730,7 +19730,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19798,7 +19798,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr"/>
@@ -19866,7 +19866,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr"/>
@@ -19882,7 +19882,7 @@
       </c>
       <c r="N338" s="2" t="inlineStr">
         <is>
-          <t>ea06a46b11320bd57b751172369cfcc31f17024123cbd88ddcaf6a325a9e091c</t>
+          <t>ba5bcc9dd80ede24167a05bf5130fb145446ad9de08dd47d522337562778b3d0</t>
         </is>
       </c>
     </row>
@@ -19934,7 +19934,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20002,7 +20002,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20070,7 +20070,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20138,12 +20138,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20158,7 +20158,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>7b14c4c6b5c41ea0a4553a469be7e12de7890fd3bf1280f792bc5b2a484ba159</t>
+          <t>f8ac95507a65afa444f76667fd44a5fba200a679d712ce015335f64d1f02c156</t>
         </is>
       </c>
     </row>
@@ -20326,7 +20326,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr"/>
@@ -20394,7 +20394,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20462,7 +20462,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20530,7 +20530,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20598,7 +20598,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20666,7 +20666,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20734,7 +20734,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20802,7 +20802,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20870,7 +20870,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20938,7 +20938,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr"/>
@@ -20998,7 +20998,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21058,10 +21058,14 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
-        </is>
-      </c>
-      <c r="K356" s="2" t="inlineStr"/>
+          <t>2026-10-13T15:17:55+00:00</t>
+        </is>
+      </c>
+      <c r="K356" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13T15:17:55+00:00</t>
+        </is>
+      </c>
       <c r="L356" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21074,7 +21078,7 @@
       </c>
       <c r="N356" s="2" t="inlineStr">
         <is>
-          <t>e3f6bf0b545ddea1862c8277793d4eca876630f816d8d21c156797435acfcbc6</t>
+          <t>c2074ff35e64cdfcef8257d127e1212cf8dfb576ae7ba58e2ce955aa28ee9d1f</t>
         </is>
       </c>
     </row>
@@ -21126,7 +21130,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr"/>
@@ -21186,7 +21190,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr"/>
@@ -21254,7 +21258,7 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr"/>
@@ -21318,7 +21322,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr"/>
@@ -21386,7 +21390,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21446,7 +21450,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21510,7 +21514,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr"/>
@@ -21570,7 +21574,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21638,7 +21642,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr"/>
@@ -21654,7 +21658,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>8049b9cb808bea700e35a8bee24f12d16bb2dd58117c934564c2e16aa7b998b2</t>
+          <t>c3f4bcae147fd2f8de1141fc7f1e682062f2d13176a121382a9bb7fbde256f22</t>
         </is>
       </c>
     </row>
@@ -21706,7 +21710,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr"/>
@@ -21722,7 +21726,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>83bbd3747858fd5777527acdb233a2bda546fe8984b911e1aebd1127ff0440d6</t>
+          <t>ae1fa3de99e70d0637da41397f89dafacb36f23270601d02e4cd3fcbaeadf2ed</t>
         </is>
       </c>
     </row>
@@ -21774,7 +21778,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr"/>
@@ -21842,7 +21846,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -21906,7 +21910,7 @@
       </c>
       <c r="J369" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K369" s="2" t="inlineStr"/>
@@ -21970,7 +21974,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22447,7 +22451,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22489,7 +22493,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22523,7 +22527,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22565,7 +22569,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22603,7 +22607,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22641,7 +22645,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22679,7 +22683,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22717,7 +22721,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22759,7 +22763,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22797,7 +22801,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22839,7 +22843,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22881,7 +22885,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -22923,7 +22927,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -22965,7 +22969,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23007,7 +23011,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -23049,7 +23053,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23091,7 +23095,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23133,7 +23137,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23175,7 +23179,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23217,7 +23221,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23259,7 +23263,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23301,7 +23305,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23343,7 +23347,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23381,7 +23385,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23423,7 +23427,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23461,7 +23465,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23503,7 +23507,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23545,7 +23549,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23587,7 +23591,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23629,7 +23633,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -23671,7 +23675,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23709,7 +23713,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23747,7 +23751,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23785,7 +23789,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23827,7 +23831,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23869,7 +23873,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -23907,7 +23911,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -23945,7 +23949,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -23987,7 +23991,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24029,7 +24033,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24063,7 +24067,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24105,7 +24109,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24143,7 +24147,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24181,7 +24185,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24223,7 +24227,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24261,7 +24265,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24299,7 +24303,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24337,7 +24341,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24379,7 +24383,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24417,7 +24421,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24459,7 +24463,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24501,7 +24505,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24539,7 +24543,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24581,7 +24585,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24623,7 +24627,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24661,7 +24665,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24699,7 +24703,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24737,7 +24741,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24779,7 +24783,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24817,7 +24821,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24859,7 +24863,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -24901,7 +24905,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -24939,7 +24943,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -24981,7 +24985,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25023,7 +25027,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25061,7 +25065,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25103,7 +25107,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25141,7 +25145,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25183,7 +25187,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25225,7 +25229,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25267,7 +25271,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25305,7 +25309,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25343,7 +25347,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25381,7 +25385,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25419,7 +25423,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25457,7 +25461,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25499,7 +25503,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25537,7 +25541,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25575,7 +25579,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25617,7 +25621,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25655,7 +25659,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25697,7 +25701,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25735,7 +25739,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25777,7 +25781,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25815,7 +25819,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25853,7 +25857,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25895,7 +25899,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26317,7 +26321,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -26359,7 +26363,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26401,7 +26405,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26443,7 +26447,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26485,7 +26489,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26527,7 +26531,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26569,7 +26573,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26611,7 +26615,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26653,7 +26657,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26695,7 +26699,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26737,7 +26741,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26779,7 +26783,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26821,7 +26825,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26863,7 +26867,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -26905,7 +26909,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -26947,7 +26951,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -26989,7 +26993,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27031,7 +27035,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27073,7 +27077,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27115,7 +27119,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27157,7 +27161,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27199,7 +27203,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27241,7 +27245,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27283,7 +27287,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27325,7 +27329,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27367,7 +27371,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27409,7 +27413,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27451,7 +27455,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27493,7 +27497,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27535,7 +27539,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27577,7 +27581,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27619,7 +27623,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27661,7 +27665,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -27703,7 +27707,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27745,7 +27749,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27787,7 +27791,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27829,7 +27833,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27871,7 +27875,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -27909,7 +27913,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -27951,7 +27955,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -27993,7 +27997,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28035,7 +28039,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28077,7 +28081,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28119,7 +28123,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28161,7 +28165,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28203,7 +28207,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28245,7 +28249,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28287,7 +28291,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28329,7 +28333,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28371,7 +28375,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28413,7 +28417,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28455,7 +28459,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28497,7 +28501,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28539,7 +28543,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28581,7 +28585,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28623,7 +28627,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28665,7 +28669,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28707,7 +28711,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28749,7 +28753,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28791,7 +28795,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28833,7 +28837,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28875,7 +28879,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -28917,7 +28921,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -28959,7 +28963,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29001,7 +29005,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29043,7 +29047,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29085,7 +29089,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29127,7 +29131,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29169,7 +29173,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29211,7 +29215,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29253,7 +29257,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29295,7 +29299,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29337,7 +29341,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29379,7 +29383,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29421,7 +29425,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29463,7 +29467,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29505,7 +29509,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29547,7 +29551,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29589,7 +29593,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29631,7 +29635,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29673,7 +29677,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29715,7 +29719,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29757,7 +29761,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29799,7 +29803,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29841,7 +29845,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29883,7 +29887,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -29925,7 +29929,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -29967,7 +29971,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30009,7 +30013,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30051,7 +30055,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30093,7 +30097,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30135,7 +30139,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30177,7 +30181,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30219,7 +30223,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30261,7 +30265,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30303,7 +30307,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30345,7 +30349,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30387,7 +30391,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30429,7 +30433,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30471,7 +30475,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30513,7 +30517,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30555,7 +30559,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30597,7 +30601,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30639,7 +30643,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30681,7 +30685,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30723,7 +30727,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30766,7 +30770,7 @@
       <c r="F205" s="2" t="inlineStr"/>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
@@ -30803,7 +30807,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30845,7 +30849,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -30887,7 +30891,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -30929,7 +30933,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -30971,7 +30975,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31013,7 +31017,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31055,7 +31059,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31097,7 +31101,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31139,7 +31143,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31181,7 +31185,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31223,7 +31227,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31265,7 +31269,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31307,7 +31311,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31349,7 +31353,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31391,7 +31395,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31433,7 +31437,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31475,7 +31479,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31517,7 +31521,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31559,7 +31563,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31601,7 +31605,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31643,7 +31647,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31685,7 +31689,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31727,7 +31731,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31769,7 +31773,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31811,7 +31815,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31853,7 +31857,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31895,7 +31899,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -31937,7 +31941,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -31979,7 +31983,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32021,7 +32025,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32063,7 +32067,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32105,7 +32109,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32147,7 +32151,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32189,7 +32193,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32231,7 +32235,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32273,7 +32277,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32315,7 +32319,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32357,7 +32361,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32395,7 +32399,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32437,7 +32441,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32475,7 +32479,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32509,7 +32513,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32551,7 +32555,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32589,7 +32593,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32631,7 +32635,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32673,7 +32677,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32711,7 +32715,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32749,7 +32753,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32787,7 +32791,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32825,7 +32829,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32867,7 +32871,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -32905,7 +32909,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -32939,7 +32943,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -32977,7 +32981,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33015,7 +33019,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33053,7 +33057,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33095,7 +33099,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33137,7 +33141,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33175,7 +33179,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33217,7 +33221,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33251,7 +33255,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33289,7 +33293,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33327,7 +33331,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33365,7 +33369,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-14 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6510,7 +6510,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7030,7 +7030,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8078,12 +8078,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8094,7 +8094,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>4fdb256a902dd5e365bbc5b17e1926ae002b72c41495f4174aa01ba95bfe6833</t>
+          <t>456531634f4bc163b8a8736bba7a8a5c30ae9a1d5b2de0b83bc23c569e890b01</t>
         </is>
       </c>
     </row>
@@ -8146,12 +8146,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8162,7 +8162,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>f03899a65bfc9087b21f14dc6d978e77d4fd3f574fd84dc081406af5ac8f5f3b</t>
+          <t>56cb7c6399cf6d5ed94f4a41148a3e3459123817a4437ec66d442b23be62ae19</t>
         </is>
       </c>
     </row>
@@ -8214,7 +8214,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8614,7 +8614,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8754,7 +8754,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8882,7 +8882,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10714,7 +10714,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10894,7 +10894,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10962,7 +10962,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11034,12 +11034,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11054,7 +11054,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>6f258b6021da8deb3fd5673a7960b1decf7b68e60298e9551a0cd7d0d283823f</t>
+          <t>563eef56108235bcc4fce2a837685c8ead866713d307af3b46987f59a5666ae3</t>
         </is>
       </c>
     </row>
@@ -11106,12 +11106,12 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
@@ -11126,7 +11126,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>eb6c71808c83546daa05541541be631063ae1c3125608d710c8796264c76afae</t>
+          <t>ad1cde1a1f4304f55ffba748ff785af1c412a7f672d1d798f7f48eaa379afdfe</t>
         </is>
       </c>
     </row>
@@ -11178,7 +11178,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11250,7 +11250,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11462,10 +11462,14 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
-        </is>
-      </c>
-      <c r="K199" s="2" t="inlineStr"/>
+          <t>2026-10-14T13:09:42+00:00</t>
+        </is>
+      </c>
+      <c r="K199" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T13:09:42+00:00</t>
+        </is>
+      </c>
       <c r="L199" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11478,7 +11482,7 @@
       </c>
       <c r="N199" s="2" t="inlineStr">
         <is>
-          <t>a6d6271efcfe395f03a4aff9fb76aeab50a662024ce46e25c9415caab60cf91e</t>
+          <t>bd5aee8a847f7ce1d2926cdfee0b83462cabdfb514363f93a5434af2da5f4048</t>
         </is>
       </c>
     </row>
@@ -11530,10 +11534,14 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
-        </is>
-      </c>
-      <c r="K200" s="2" t="inlineStr"/>
+          <t>2026-10-14T13:09:42+00:00</t>
+        </is>
+      </c>
+      <c r="K200" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T13:09:42+00:00</t>
+        </is>
+      </c>
       <c r="L200" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11546,7 +11554,7 @@
       </c>
       <c r="N200" s="2" t="inlineStr">
         <is>
-          <t>ddc9f99d2c78fc06635a68f693af7f2329f3044fb475438b931e0d5c9efabebb</t>
+          <t>27251f7c8e29eb152f14ab15abc2da94023143c398b45c67ac3b1c188942f930</t>
         </is>
       </c>
     </row>
@@ -11598,7 +11606,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11670,7 +11678,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11738,7 +11746,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11810,7 +11818,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11882,7 +11890,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12014,7 +12022,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12034,7 +12042,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>abdcb5c9c9ba2fec3bbc78a104a53261117b2fc19cc2510708187da1cc60737f</t>
+          <t>0398a8b2f44e87e35cebc2bc39be0125946115179470248ee01cc1b367a10e6a</t>
         </is>
       </c>
     </row>
@@ -12086,7 +12094,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12154,12 +12162,12 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
@@ -12174,7 +12182,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
+          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
         </is>
       </c>
     </row>
@@ -12226,7 +12234,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12522,7 +12530,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12770,7 +12778,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12838,7 +12846,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12906,7 +12914,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13098,7 +13106,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr"/>
@@ -13166,7 +13174,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr"/>
@@ -13234,7 +13242,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13302,7 +13310,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13370,7 +13378,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13438,7 +13446,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13562,7 +13570,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13582,7 +13590,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>7aac9d9c52a684d194f84c75ea15e8b14fb3a13a5f54f735261a8d39b6d4af67</t>
+          <t>48e81c8b31547c08652044290e37ba96ce52798aff926af59882658059ac2b6b</t>
         </is>
       </c>
     </row>
@@ -13874,12 +13882,12 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
@@ -13894,7 +13902,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>507024c4db7ade4ea8ad7eaa8a06520b997f4a551b2c4cb24aa9e27f1ec72a6b</t>
+          <t>24548a00c47e1ebeab67613a87172acba0b8950e67008391d0a496042d8052c5</t>
         </is>
       </c>
     </row>
@@ -18146,14 +18154,14 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
+          <t>2026-10-14T13:09:42+00:00</t>
+        </is>
+      </c>
+      <c r="K312" s="2" t="inlineStr">
+        <is>
           <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
-      <c r="K312" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13T15:17:55+00:00</t>
-        </is>
-      </c>
       <c r="L312" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -18166,7 +18174,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>698da8062ce0ed7aa726791fe92d7aac4fad77a93b2f894b4a171f512744718d</t>
+          <t>35faef9fae846e990fab57f24c2da1aa1dbbaca7cd66ec0c677871c020c6d346</t>
         </is>
       </c>
     </row>
@@ -18218,14 +18226,14 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
+          <t>2026-10-14T13:09:42+00:00</t>
+        </is>
+      </c>
+      <c r="K313" s="2" t="inlineStr">
+        <is>
           <t>2026-10-13T15:17:55+00:00</t>
         </is>
       </c>
-      <c r="K313" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13T15:17:55+00:00</t>
-        </is>
-      </c>
       <c r="L313" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -18238,7 +18246,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>5c737e3ede2a24bb547f6775237cb24a80ca2bb02e8422470ecadb7fb8592a49</t>
+          <t>bf60eedd5a6d4b2673f957f99530091212ff775573d2583056c3097b0ae9e07f</t>
         </is>
       </c>
     </row>
@@ -18290,7 +18298,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18362,7 +18370,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18430,7 +18438,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18498,7 +18506,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18622,7 +18630,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19050,7 +19058,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19118,7 +19126,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19186,7 +19194,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19254,12 +19262,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19274,7 +19282,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>c590a678e5a4416ad7174591e81c284aa75e9d40f63a7f4879338b6c803d5434</t>
+          <t>39a760671c47da8e16ca0f808d7a21c2a4a8bcd34ced81052e9e718cf16ed612</t>
         </is>
       </c>
     </row>
@@ -19326,7 +19334,7 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
@@ -19346,7 +19354,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>af79caf88b2de905250c356b07f541452519c0fcf4a9cdea3e413105ed1b1aee</t>
+          <t>22672cfdfb82c3b6c9e1fc6b9b73e9ba4bfeaced08a486d3569ed28fabcd3136</t>
         </is>
       </c>
     </row>
@@ -19398,12 +19406,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19418,7 +19426,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>24be046587768f330df02db27a76008b96240019bee1260aee250963db00bf59</t>
+          <t>15655045c0e6dfe33623e088ad4cd44bbf3592d63fb1029223145dcd5622f58e</t>
         </is>
       </c>
     </row>
@@ -19470,7 +19478,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr"/>
@@ -19594,7 +19602,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19662,7 +19670,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19730,7 +19738,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19798,7 +19806,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr"/>
@@ -19866,7 +19874,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr"/>
@@ -19934,7 +19942,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20002,7 +20010,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20070,7 +20078,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20138,12 +20146,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20158,7 +20166,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>f8ac95507a65afa444f76667fd44a5fba200a679d712ce015335f64d1f02c156</t>
+          <t>5a5c9818896af21e16a86bd45ba7673f8e0e076cb10b8d2835b93925b81652e1</t>
         </is>
       </c>
     </row>
@@ -20326,7 +20334,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr"/>
@@ -20394,7 +20402,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20462,7 +20470,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20530,7 +20538,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20598,7 +20606,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20666,7 +20674,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20734,7 +20742,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20802,7 +20810,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20870,7 +20878,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20938,7 +20946,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr"/>
@@ -20998,7 +21006,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21058,7 +21066,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21130,10 +21138,14 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
-        </is>
-      </c>
-      <c r="K357" s="2" t="inlineStr"/>
+          <t>2026-10-14T13:09:42+00:00</t>
+        </is>
+      </c>
+      <c r="K357" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T13:09:42+00:00</t>
+        </is>
+      </c>
       <c r="L357" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21146,7 +21158,7 @@
       </c>
       <c r="N357" s="2" t="inlineStr">
         <is>
-          <t>03f07d51151650af40df39198da49d45abc478d517e2da1cafd54fcdad799aa7</t>
+          <t>390dd9e09404b50f97a439e68120f52880697d102557905eb05bfeefb3b67f2a</t>
         </is>
       </c>
     </row>
@@ -21190,7 +21202,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr"/>
@@ -21258,7 +21270,7 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr"/>
@@ -21322,7 +21334,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr"/>
@@ -21390,7 +21402,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21450,7 +21462,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21514,7 +21526,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr"/>
@@ -21574,7 +21586,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21642,7 +21654,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr"/>
@@ -21658,7 +21670,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>c3f4bcae147fd2f8de1141fc7f1e682062f2d13176a121382a9bb7fbde256f22</t>
+          <t>de14fb9bf5387df6ed19b8c24388e0e31757eec548e3c570fc62750276ca0742</t>
         </is>
       </c>
     </row>
@@ -21710,7 +21722,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr"/>
@@ -21726,7 +21738,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>ae1fa3de99e70d0637da41397f89dafacb36f23270601d02e4cd3fcbaeadf2ed</t>
+          <t>947cf57ca3946089cd14824384b8fd7329038b280f46850bea3dc873dacb6b95</t>
         </is>
       </c>
     </row>
@@ -21778,10 +21790,14 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
-        </is>
-      </c>
-      <c r="K367" s="2" t="inlineStr"/>
+          <t>2026-10-14T13:09:42+00:00</t>
+        </is>
+      </c>
+      <c r="K367" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T13:09:42+00:00</t>
+        </is>
+      </c>
       <c r="L367" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21794,7 +21810,7 @@
       </c>
       <c r="N367" s="2" t="inlineStr">
         <is>
-          <t>be8dee3fad1f5ebe96951f5be14b13b5f3bb68b76f67f0dfbdc2b2cbcb407bf7</t>
+          <t>748b02860fb388344d9f9ecf1fca221a7e9645000e2c57095e7b94ffe080c5c4</t>
         </is>
       </c>
     </row>
@@ -21846,7 +21862,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -21910,7 +21926,7 @@
       </c>
       <c r="J369" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K369" s="2" t="inlineStr"/>
@@ -21974,7 +21990,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22451,7 +22467,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22493,7 +22509,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22527,7 +22543,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22569,7 +22585,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22607,7 +22623,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22645,7 +22661,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22683,7 +22699,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22721,7 +22737,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22763,7 +22779,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22801,7 +22817,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22843,7 +22859,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22885,7 +22901,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -22927,7 +22943,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -22969,7 +22985,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23011,7 +23027,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -23053,7 +23069,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23095,7 +23111,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23137,7 +23153,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23179,7 +23195,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23221,7 +23237,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23263,7 +23279,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23305,7 +23321,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23347,7 +23363,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23385,7 +23401,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23427,7 +23443,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23465,7 +23481,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23507,7 +23523,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23549,7 +23565,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23591,7 +23607,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23633,7 +23649,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -23675,7 +23691,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23713,7 +23729,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23751,7 +23767,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23789,7 +23805,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23831,7 +23847,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23873,7 +23889,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -23911,7 +23927,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -23949,7 +23965,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -23991,7 +24007,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24033,7 +24049,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24067,7 +24083,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24109,7 +24125,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24147,7 +24163,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24185,7 +24201,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24227,7 +24243,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24265,7 +24281,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24303,7 +24319,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24341,7 +24357,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24383,7 +24399,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24421,7 +24437,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24463,7 +24479,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24505,7 +24521,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24543,7 +24559,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24585,7 +24601,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24627,7 +24643,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24665,7 +24681,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24703,7 +24719,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24741,7 +24757,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24783,7 +24799,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24821,7 +24837,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24863,7 +24879,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -24905,7 +24921,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -24943,7 +24959,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -24985,7 +25001,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25027,7 +25043,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25065,7 +25081,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25107,7 +25123,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25145,7 +25161,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25187,7 +25203,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25229,7 +25245,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25271,7 +25287,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25309,7 +25325,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25347,7 +25363,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25385,7 +25401,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25423,7 +25439,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25461,7 +25477,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25503,7 +25519,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25541,7 +25557,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25579,7 +25595,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25621,7 +25637,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25659,7 +25675,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25701,7 +25717,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25739,7 +25755,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25781,7 +25797,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25819,7 +25835,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25857,7 +25873,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25899,7 +25915,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26321,7 +26337,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -26363,7 +26379,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26405,7 +26421,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26447,7 +26463,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26489,7 +26505,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26531,7 +26547,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26573,7 +26589,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26615,7 +26631,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26657,7 +26673,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26699,7 +26715,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26741,7 +26757,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26783,7 +26799,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26825,7 +26841,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26867,7 +26883,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -26909,7 +26925,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -26951,7 +26967,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -26993,7 +27009,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27035,7 +27051,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27077,7 +27093,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27119,7 +27135,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27161,7 +27177,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27203,7 +27219,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27245,7 +27261,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27287,7 +27303,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27329,7 +27345,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27371,7 +27387,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27413,7 +27429,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27455,7 +27471,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27497,7 +27513,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27539,7 +27555,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27581,7 +27597,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27623,7 +27639,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27665,7 +27681,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -27707,7 +27723,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27749,7 +27765,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27791,7 +27807,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27833,7 +27849,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27875,7 +27891,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -27913,7 +27929,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -27955,7 +27971,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -27997,7 +28013,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28039,7 +28055,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28081,7 +28097,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28123,7 +28139,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28165,7 +28181,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28207,7 +28223,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28249,7 +28265,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28291,7 +28307,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28333,7 +28349,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28375,7 +28391,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28417,7 +28433,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28459,7 +28475,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28501,7 +28517,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28543,7 +28559,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28585,7 +28601,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28627,7 +28643,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28669,7 +28685,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28711,7 +28727,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28753,7 +28769,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28795,7 +28811,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28837,7 +28853,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28879,7 +28895,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -28921,7 +28937,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -28963,7 +28979,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29005,7 +29021,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29047,7 +29063,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29089,7 +29105,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29131,7 +29147,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29173,7 +29189,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29215,7 +29231,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29257,7 +29273,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29299,7 +29315,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29341,7 +29357,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29383,7 +29399,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29425,7 +29441,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29467,7 +29483,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29509,7 +29525,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29551,7 +29567,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29593,7 +29609,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29635,7 +29651,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29677,7 +29693,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29719,7 +29735,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29766,7 +29782,7 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H181" s="2" t="inlineStr">
@@ -29803,7 +29819,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29845,7 +29861,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29887,7 +29903,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -29929,7 +29945,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -29971,7 +29987,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30013,7 +30029,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30055,7 +30071,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30097,7 +30113,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30139,7 +30155,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30181,7 +30197,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30223,7 +30239,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30265,7 +30281,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30307,7 +30323,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30349,7 +30365,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30391,7 +30407,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30433,7 +30449,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30475,7 +30491,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30517,7 +30533,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30559,7 +30575,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30601,7 +30617,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30643,7 +30659,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30685,7 +30701,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30727,7 +30743,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30770,7 +30786,7 @@
       <c r="F205" s="2" t="inlineStr"/>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
@@ -30807,7 +30823,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30849,7 +30865,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -30891,7 +30907,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -30933,7 +30949,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -30975,7 +30991,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31017,7 +31033,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31059,7 +31075,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31101,7 +31117,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31143,7 +31159,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31185,7 +31201,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31227,7 +31243,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31269,7 +31285,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31311,7 +31327,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31353,7 +31369,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31395,7 +31411,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31437,7 +31453,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31479,7 +31495,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31521,7 +31537,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31563,7 +31579,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31605,7 +31621,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31647,7 +31663,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31689,7 +31705,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31731,7 +31747,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31773,7 +31789,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31815,7 +31831,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31857,7 +31873,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31899,7 +31915,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -31941,7 +31957,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -31983,7 +31999,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32025,7 +32041,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32067,7 +32083,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32109,7 +32125,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32151,7 +32167,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32193,7 +32209,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32235,7 +32251,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32277,7 +32293,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32319,7 +32335,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32361,7 +32377,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32399,7 +32415,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32441,7 +32457,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32479,7 +32495,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32513,7 +32529,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32555,7 +32571,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32593,7 +32609,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32635,7 +32651,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32677,7 +32693,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32715,7 +32731,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32753,7 +32769,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32791,7 +32807,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32829,7 +32845,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32871,7 +32887,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -32909,7 +32925,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -32943,7 +32959,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -32981,7 +32997,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33019,7 +33035,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33057,7 +33073,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33099,7 +33115,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33141,7 +33157,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33179,7 +33195,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33221,7 +33237,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33255,7 +33271,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33293,7 +33309,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33331,7 +33347,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33369,7 +33385,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-14T13:09:42+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-15 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6510,7 +6510,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7030,7 +7030,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8078,12 +8078,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8094,7 +8094,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>456531634f4bc163b8a8736bba7a8a5c30ae9a1d5b2de0b83bc23c569e890b01</t>
+          <t>4e71e98e68febda1c52c6c5a943bdd50a727b86f031d9ea8e5d1c890fca412c0</t>
         </is>
       </c>
     </row>
@@ -8146,12 +8146,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8162,7 +8162,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>56cb7c6399cf6d5ed94f4a41148a3e3459123817a4437ec66d442b23be62ae19</t>
+          <t>c732c383f5ed63dcd0bf2c6e61ae542a09988681e3baa9fdbd4492912902b817</t>
         </is>
       </c>
     </row>
@@ -8214,7 +8214,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8614,7 +8614,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8754,7 +8754,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8882,7 +8882,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10714,7 +10714,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10894,7 +10894,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10962,7 +10962,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11034,12 +11034,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11054,7 +11054,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>563eef56108235bcc4fce2a837685c8ead866713d307af3b46987f59a5666ae3</t>
+          <t>bb4610b9f408f10095804bb1fb1b8faa669753631bc0ccefad083f1de0662342</t>
         </is>
       </c>
     </row>
@@ -11106,7 +11106,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11178,7 +11178,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11250,7 +11250,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11462,7 +11462,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11534,7 +11534,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11606,7 +11606,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11678,7 +11678,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11746,7 +11746,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11818,7 +11818,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11890,7 +11890,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12022,7 +12022,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12042,7 +12042,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>0398a8b2f44e87e35cebc2bc39be0125946115179470248ee01cc1b367a10e6a</t>
+          <t>b2a60b2bda13220281b4129225034a4c70848f134bae8af314dc185d5619e5f6</t>
         </is>
       </c>
     </row>
@@ -12094,7 +12094,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12162,7 +12162,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12530,7 +12530,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12778,10 +12778,14 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
-        </is>
-      </c>
-      <c r="K219" s="2" t="inlineStr"/>
+          <t>2026-10-15T12:54:41+00:00</t>
+        </is>
+      </c>
+      <c r="K219" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T12:54:41+00:00</t>
+        </is>
+      </c>
       <c r="L219" s="2" t="inlineStr">
         <is>
           <t>2026-09-30</t>
@@ -12794,7 +12798,7 @@
       </c>
       <c r="N219" s="2" t="inlineStr">
         <is>
-          <t>ed25df8df719b00e7c8b065ffff68395992cf4e1dde158b1213ced16889c3965</t>
+          <t>7d213556641924980cf256ce1311f268027b171bf8a2169f1823bfa973743e3b</t>
         </is>
       </c>
     </row>
@@ -12846,7 +12850,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12914,7 +12918,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13106,7 +13110,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr"/>
@@ -13174,7 +13178,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr"/>
@@ -13242,7 +13246,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13310,7 +13314,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13378,7 +13382,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13446,7 +13450,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13570,7 +13574,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13590,7 +13594,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>48e81c8b31547c08652044290e37ba96ce52798aff926af59882658059ac2b6b</t>
+          <t>a55a21f9c39028df1294608bfa4eea59bcb8dbf9cd3fc8ac33b197e038e27e34</t>
         </is>
       </c>
     </row>
@@ -13882,12 +13886,12 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
@@ -13902,7 +13906,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>24548a00c47e1ebeab67613a87172acba0b8950e67008391d0a496042d8052c5</t>
+          <t>533f92c08eec0fd3ccb24e56ba54cc7d7e61059afb842afe9ddf783522de2b15</t>
         </is>
       </c>
     </row>
@@ -18154,12 +18158,12 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="L312" s="2" t="inlineStr">
@@ -18174,7 +18178,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>35faef9fae846e990fab57f24c2da1aa1dbbaca7cd66ec0c677871c020c6d346</t>
+          <t>0d0903557b20b250d77fe4717ab0e84fd0e6cf11f2c019013fb01d38eac5720f</t>
         </is>
       </c>
     </row>
@@ -18226,12 +18230,12 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="L313" s="2" t="inlineStr">
@@ -18246,7 +18250,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>bf60eedd5a6d4b2673f957f99530091212ff775573d2583056c3097b0ae9e07f</t>
+          <t>821a1acbe9420ae8a533bedd964c0ef5a4b96fa2fbb081579c896e633b3718d0</t>
         </is>
       </c>
     </row>
@@ -18298,7 +18302,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18370,7 +18374,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18438,7 +18442,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18506,7 +18510,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18630,7 +18634,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19058,7 +19062,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19126,7 +19130,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19194,7 +19198,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19262,12 +19266,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19282,7 +19286,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>39a760671c47da8e16ca0f808d7a21c2a4a8bcd34ced81052e9e718cf16ed612</t>
+          <t>60e8dc1c9d9cc07425e96139c042e55ad8b86b70d9e9a3f7cede3dbf305f5732</t>
         </is>
       </c>
     </row>
@@ -19334,7 +19338,7 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
@@ -19354,7 +19358,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>22672cfdfb82c3b6c9e1fc6b9b73e9ba4bfeaced08a486d3569ed28fabcd3136</t>
+          <t>0b1bc468b3e3f3504928bed6a886789d7e4e40ae8fd5d09da1e8acccbe129ecc</t>
         </is>
       </c>
     </row>
@@ -19406,12 +19410,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19426,7 +19430,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>15655045c0e6dfe33623e088ad4cd44bbf3592d63fb1029223145dcd5622f58e</t>
+          <t>0b7346c86b3c0ef98c8b8e1f5d30ac20943f7a48fdba5c5607f0eeabae56fcfa</t>
         </is>
       </c>
     </row>
@@ -19478,7 +19482,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr"/>
@@ -19602,7 +19606,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19670,7 +19674,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19738,7 +19742,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19806,7 +19810,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr"/>
@@ -19874,7 +19878,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr"/>
@@ -19942,7 +19946,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20010,7 +20014,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20078,7 +20082,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20146,12 +20150,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20166,7 +20170,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>5a5c9818896af21e16a86bd45ba7673f8e0e076cb10b8d2835b93925b81652e1</t>
+          <t>b07298093de43aa133c0fef2b61ca00824fe69e097becc9f88c2b12e578533b3</t>
         </is>
       </c>
     </row>
@@ -20334,7 +20338,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr"/>
@@ -20402,7 +20406,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20470,7 +20474,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20538,7 +20542,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20606,7 +20610,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20674,7 +20678,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20742,7 +20746,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20810,7 +20814,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20878,7 +20882,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20946,7 +20950,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr"/>
@@ -21006,7 +21010,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21066,7 +21070,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21138,7 +21142,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21202,7 +21206,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr"/>
@@ -21270,10 +21274,14 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
-        </is>
-      </c>
-      <c r="K359" s="2" t="inlineStr"/>
+          <t>2026-10-15T12:54:41+00:00</t>
+        </is>
+      </c>
+      <c r="K359" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T12:54:41+00:00</t>
+        </is>
+      </c>
       <c r="L359" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21286,7 +21294,7 @@
       </c>
       <c r="N359" s="2" t="inlineStr">
         <is>
-          <t>9c26992a5e779f3b88432ec580f2ab762aace0d4682af88b770390e75c06cbc1</t>
+          <t>2aad17d7261e53631df4ef311d46bdb9d37b2fbc79969f32c0689f65bf163b96</t>
         </is>
       </c>
     </row>
@@ -21334,7 +21342,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr"/>
@@ -21402,7 +21410,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21462,7 +21470,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21526,7 +21534,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr"/>
@@ -21586,7 +21594,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21654,7 +21662,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr"/>
@@ -21670,7 +21678,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>de14fb9bf5387df6ed19b8c24388e0e31757eec548e3c570fc62750276ca0742</t>
+          <t>32eec940ea46c6891a7a967f0f01f66d9e102f7974586199538b2f0169258064</t>
         </is>
       </c>
     </row>
@@ -21722,7 +21730,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr"/>
@@ -21738,7 +21746,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>947cf57ca3946089cd14824384b8fd7329038b280f46850bea3dc873dacb6b95</t>
+          <t>67dd9cee38bbc411028eeeb8a9c51d415c5a1db92bb27eb50ac66bd36cd0409b</t>
         </is>
       </c>
     </row>
@@ -21790,7 +21798,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21862,7 +21870,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -21926,7 +21934,7 @@
       </c>
       <c r="J369" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K369" s="2" t="inlineStr"/>
@@ -21990,7 +21998,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22467,7 +22475,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22509,7 +22517,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22543,7 +22551,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22585,7 +22593,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22623,7 +22631,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22661,7 +22669,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22699,7 +22707,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22737,7 +22745,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22779,7 +22787,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22817,7 +22825,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22859,7 +22867,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22901,7 +22909,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -22943,7 +22951,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -22985,7 +22993,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23027,7 +23035,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -23069,7 +23077,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23111,7 +23119,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23153,7 +23161,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23195,7 +23203,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23237,7 +23245,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23279,7 +23287,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23321,7 +23329,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23363,7 +23371,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23401,7 +23409,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23443,7 +23451,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23481,7 +23489,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23523,7 +23531,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23565,7 +23573,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23607,7 +23615,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23649,7 +23657,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -23691,7 +23699,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23729,7 +23737,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23767,7 +23775,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23805,7 +23813,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23847,7 +23855,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23889,7 +23897,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -23927,7 +23935,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -23965,7 +23973,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24007,7 +24015,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24049,7 +24057,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24083,7 +24091,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24125,7 +24133,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24163,7 +24171,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24201,7 +24209,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24243,7 +24251,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24281,7 +24289,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24319,7 +24327,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24357,7 +24365,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24399,7 +24407,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24437,7 +24445,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24479,7 +24487,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24521,7 +24529,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24559,7 +24567,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24601,7 +24609,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24643,7 +24651,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24681,7 +24689,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24719,7 +24727,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24757,7 +24765,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24799,7 +24807,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24837,7 +24845,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24879,7 +24887,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -24921,7 +24929,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -24959,7 +24967,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25001,7 +25009,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25043,7 +25051,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25081,7 +25089,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25123,7 +25131,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25161,7 +25169,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25203,7 +25211,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25245,7 +25253,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25287,7 +25295,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25325,7 +25333,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25363,7 +25371,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25401,7 +25409,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25439,7 +25447,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25477,7 +25485,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25519,7 +25527,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25557,7 +25565,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25595,7 +25603,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25637,7 +25645,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25675,7 +25683,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25717,7 +25725,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25755,7 +25763,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25797,7 +25805,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25835,7 +25843,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25873,7 +25881,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25915,7 +25923,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26337,7 +26345,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -26379,7 +26387,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26421,7 +26429,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26463,7 +26471,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26505,7 +26513,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26547,7 +26555,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26589,7 +26597,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26631,7 +26639,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26673,7 +26681,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26715,7 +26723,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26757,7 +26765,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26799,7 +26807,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26841,7 +26849,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26883,7 +26891,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -26925,7 +26933,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -26967,7 +26975,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27009,7 +27017,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27051,7 +27059,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27093,7 +27101,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27135,7 +27143,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27177,7 +27185,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27219,7 +27227,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27261,7 +27269,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27303,7 +27311,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27345,7 +27353,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27387,7 +27395,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27429,7 +27437,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27471,7 +27479,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27513,7 +27521,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27555,7 +27563,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27597,7 +27605,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27639,7 +27647,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27681,7 +27689,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -27723,7 +27731,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27765,7 +27773,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27807,7 +27815,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27849,7 +27857,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27891,7 +27899,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -27929,7 +27937,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -27971,7 +27979,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28013,7 +28021,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28055,7 +28063,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28097,7 +28105,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28139,7 +28147,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28181,7 +28189,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28223,7 +28231,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28265,7 +28273,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28307,7 +28315,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28349,7 +28357,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28391,7 +28399,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28433,7 +28441,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28475,7 +28483,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28517,7 +28525,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28559,7 +28567,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28601,7 +28609,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28643,7 +28651,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28685,7 +28693,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28727,7 +28735,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28769,7 +28777,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28811,7 +28819,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28853,7 +28861,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28895,7 +28903,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -28937,7 +28945,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -28979,7 +28987,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29021,7 +29029,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29063,7 +29071,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29105,7 +29113,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29147,7 +29155,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29189,7 +29197,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29231,7 +29239,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29273,7 +29281,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29315,7 +29323,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29357,7 +29365,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29399,7 +29407,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29441,7 +29449,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29483,7 +29491,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29525,7 +29533,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29567,7 +29575,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29609,7 +29617,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29651,7 +29659,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29693,7 +29701,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29735,7 +29743,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29777,12 +29785,12 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H181" s="2" t="inlineStr">
@@ -29819,7 +29827,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29861,7 +29869,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29903,7 +29911,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -29950,7 +29958,7 @@
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H185" s="2" t="inlineStr">
@@ -29987,7 +29995,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30029,7 +30037,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30071,7 +30079,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30113,7 +30121,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30155,7 +30163,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30197,7 +30205,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30239,7 +30247,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30281,7 +30289,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30323,7 +30331,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30365,7 +30373,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30407,7 +30415,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30449,7 +30457,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30491,7 +30499,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30533,7 +30541,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30575,7 +30583,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30617,7 +30625,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30659,7 +30667,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30701,7 +30709,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30743,7 +30751,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30786,7 +30794,7 @@
       <c r="F205" s="2" t="inlineStr"/>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
@@ -30823,7 +30831,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30865,7 +30873,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -30907,7 +30915,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -30949,7 +30957,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -30991,7 +30999,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31033,7 +31041,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31075,7 +31083,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31117,7 +31125,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31159,7 +31167,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31201,7 +31209,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31243,7 +31251,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31285,7 +31293,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31327,7 +31335,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31369,7 +31377,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31411,7 +31419,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31453,7 +31461,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31495,7 +31503,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31537,7 +31545,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31579,7 +31587,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31621,7 +31629,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31663,7 +31671,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31705,7 +31713,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31747,7 +31755,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31789,7 +31797,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31831,7 +31839,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31873,7 +31881,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31915,7 +31923,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -31957,7 +31965,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -31999,7 +32007,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32041,7 +32049,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32083,7 +32091,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32125,7 +32133,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32167,7 +32175,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32209,7 +32217,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32251,7 +32259,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32293,7 +32301,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32335,7 +32343,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32377,7 +32385,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32415,7 +32423,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32457,7 +32465,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32495,7 +32503,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32529,7 +32537,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32571,7 +32579,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32609,7 +32617,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32651,7 +32659,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32693,7 +32701,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32731,7 +32739,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32769,7 +32777,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32807,7 +32815,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32845,7 +32853,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32887,7 +32895,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -32925,7 +32933,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -32959,7 +32967,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -32997,7 +33005,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33035,7 +33043,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33073,7 +33081,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33115,7 +33123,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33157,7 +33165,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33195,7 +33203,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33237,7 +33245,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33271,7 +33279,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33309,7 +33317,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33347,7 +33355,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33385,7 +33393,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-16 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6510,7 +6510,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7030,7 +7030,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8078,12 +8078,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8094,7 +8094,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>4e71e98e68febda1c52c6c5a943bdd50a727b86f031d9ea8e5d1c890fca412c0</t>
+          <t>36cba3959afa1ebd074f0091369259c7a27b47ad1d3a48458e1dc9addc73cd58</t>
         </is>
       </c>
     </row>
@@ -8146,12 +8146,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8162,7 +8162,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>c732c383f5ed63dcd0bf2c6e61ae542a09988681e3baa9fdbd4492912902b817</t>
+          <t>312937aeef7a59572980b7056eb17f932d193ed21fc77219b6fde9baec9335d9</t>
         </is>
       </c>
     </row>
@@ -8214,7 +8214,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8614,7 +8614,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8754,7 +8754,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8882,7 +8882,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9022,10 +9022,14 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
-        </is>
-      </c>
-      <c r="K158" s="2" t="inlineStr"/>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
+      <c r="K158" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
           <t>2026-09-06</t>
@@ -9038,7 +9042,7 @@
       </c>
       <c r="N158" s="2" t="inlineStr">
         <is>
-          <t>a3e05e05353a3351797d1cb622c95e6275066b2d13ceb9b48d17a9f2faac0bfc</t>
+          <t>ebd4a50c230f3ff69b874327f44329938fddbf9151dc852013ec26611f075520</t>
         </is>
       </c>
     </row>
@@ -10714,7 +10718,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10894,7 +10898,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10962,7 +10966,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11034,12 +11038,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11054,7 +11058,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>bb4610b9f408f10095804bb1fb1b8faa669753631bc0ccefad083f1de0662342</t>
+          <t>ca07f195765ce5464ebbb41ee48bc696c3d6bfcd55ca6935963cac3f0eb33fba</t>
         </is>
       </c>
     </row>
@@ -11106,7 +11110,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11126,7 +11130,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>ad1cde1a1f4304f55ffba748ff785af1c412a7f672d1d798f7f48eaa379afdfe</t>
+          <t>70e86499b9258eabdfa7947c036fab6c14abca885b2175748569ffa5ab7f8669</t>
         </is>
       </c>
     </row>
@@ -11178,12 +11182,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11198,7 +11202,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>51081ff037091c08cec9c71a7550226d330f194712f7b732041cc7a53d7bd7ce</t>
+          <t>32df9e260ab4093d0d9b60083b627784f3c48080b194b85688f06449dfc22f37</t>
         </is>
       </c>
     </row>
@@ -11250,12 +11254,12 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10T13:51:10+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
@@ -11270,7 +11274,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>5d3931b51d7fb11073b8907fc7cfa1e20083c39adf7a2ed8ff67d00713e6ba95</t>
+          <t>b6b27a7efe1d73b642f07e8f2ffa02beea94d20c7ba545b0d8ec777beb02589c</t>
         </is>
       </c>
     </row>
@@ -11322,7 +11326,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11394,7 +11398,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11462,7 +11466,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11534,7 +11538,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11606,7 +11610,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11678,7 +11682,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11746,7 +11750,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11818,7 +11822,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11890,7 +11894,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12022,7 +12026,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12094,7 +12098,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12162,7 +12166,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12182,7 +12186,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
+          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
         </is>
       </c>
     </row>
@@ -12234,7 +12238,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12530,7 +12534,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12778,7 +12782,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12850,10 +12854,14 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
-        </is>
-      </c>
-      <c r="K220" s="2" t="inlineStr"/>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
+      <c r="K220" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
       <c r="L220" s="2" t="inlineStr">
         <is>
           <t>2026-09-30</t>
@@ -12866,7 +12874,7 @@
       </c>
       <c r="N220" s="2" t="inlineStr">
         <is>
-          <t>19fab800776b7c2cb44522f479ef68fc38d89692f4288a4f9a96b46ab7cdee96</t>
+          <t>cfffc1773d5fcbeefc5f1f05d3996da8400db2f4c889dbe4c70b1df9730cffb1</t>
         </is>
       </c>
     </row>
@@ -12918,7 +12926,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13110,10 +13118,14 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
-        </is>
-      </c>
-      <c r="K224" s="2" t="inlineStr"/>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
+      <c r="K224" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
       <c r="L224" s="2" t="inlineStr">
         <is>
           <t>2026-09-30</t>
@@ -13126,7 +13138,7 @@
       </c>
       <c r="N224" s="2" t="inlineStr">
         <is>
-          <t>86c7e948b3264fe37a0c5409975f8fec1eea4f0ff8f9c01b11bb08ebada1876d</t>
+          <t>51216777fbb4726211a885940169761b21a52d18b6357fa744629970d16f9f68</t>
         </is>
       </c>
     </row>
@@ -13178,10 +13190,14 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
-        </is>
-      </c>
-      <c r="K225" s="2" t="inlineStr"/>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
+      <c r="K225" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
       <c r="L225" s="2" t="inlineStr">
         <is>
           <t>2026-10-08</t>
@@ -13194,7 +13210,7 @@
       </c>
       <c r="N225" s="2" t="inlineStr">
         <is>
-          <t>66a0661a0966c676dd7d1d601a9d41ac34dadac9991081817d728bef6a5ab33e</t>
+          <t>b085021fb3874f27b526face8ac99466487c72a05b9c9f31af36c937a015c7d2</t>
         </is>
       </c>
     </row>
@@ -13246,7 +13262,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13314,7 +13330,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13382,7 +13398,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13450,7 +13466,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13574,7 +13590,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13594,7 +13610,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>a55a21f9c39028df1294608bfa4eea59bcb8dbf9cd3fc8ac33b197e038e27e34</t>
+          <t>84f5926aa0671dc0e4638c60833270b8caa5aed5ad58bf2a48a22437637be9e2</t>
         </is>
       </c>
     </row>
@@ -13886,12 +13902,12 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
@@ -13906,7 +13922,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>533f92c08eec0fd3ccb24e56ba54cc7d7e61059afb842afe9ddf783522de2b15</t>
+          <t>20731603a546316575d8e7b09a41dce5926d79d4e84fbf3566de18f902cd83a7</t>
         </is>
       </c>
     </row>
@@ -18158,7 +18174,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18230,14 +18246,14 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
+      <c r="K313" s="2" t="inlineStr">
+        <is>
           <t>2026-10-15T12:54:41+00:00</t>
         </is>
       </c>
-      <c r="K313" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-15T12:54:41+00:00</t>
-        </is>
-      </c>
       <c r="L313" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -18250,7 +18266,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>821a1acbe9420ae8a533bedd964c0ef5a4b96fa2fbb081579c896e633b3718d0</t>
+          <t>50316d07b996d21720b7a8379e686ec76f0db2ccb316579fa9a2f5a564972f69</t>
         </is>
       </c>
     </row>
@@ -18302,7 +18318,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18374,7 +18390,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18442,7 +18458,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18510,7 +18526,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18634,7 +18650,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19062,7 +19078,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19130,7 +19146,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19198,7 +19214,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19266,12 +19282,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19286,7 +19302,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>60e8dc1c9d9cc07425e96139c042e55ad8b86b70d9e9a3f7cede3dbf305f5732</t>
+          <t>2e591b0c09df4e353760136ded8ef7f8d8812f4758686f6c12ab2c679ce6bb86</t>
         </is>
       </c>
     </row>
@@ -19338,12 +19354,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11T14:09:30+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19358,7 +19374,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>0b1bc468b3e3f3504928bed6a886789d7e4e40ae8fd5d09da1e8acccbe129ecc</t>
+          <t>4a488d1ace17372fa512e68d9b22e710519ce4d9070faa8938f2a68e93c10252</t>
         </is>
       </c>
     </row>
@@ -19410,12 +19426,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19430,7 +19446,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>0b7346c86b3c0ef98c8b8e1f5d30ac20943f7a48fdba5c5607f0eeabae56fcfa</t>
+          <t>7944c275492ab2f1fea7287aa95c4e42d6b85ce22036152bcf526a5f46161816</t>
         </is>
       </c>
     </row>
@@ -19482,7 +19498,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr"/>
@@ -19606,7 +19622,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19674,7 +19690,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19742,7 +19758,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19810,7 +19826,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr"/>
@@ -19878,7 +19894,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr"/>
@@ -19946,7 +19962,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20014,7 +20030,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20082,7 +20098,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20150,12 +20166,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20170,7 +20186,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>b07298093de43aa133c0fef2b61ca00824fe69e097becc9f88c2b12e578533b3</t>
+          <t>0e91c37168f822ae6a127d93eda2e34af04d9fac70a4b1b8bf3321e2709eb87f</t>
         </is>
       </c>
     </row>
@@ -20338,7 +20354,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr"/>
@@ -20406,7 +20422,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20474,7 +20490,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20542,7 +20558,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20610,7 +20626,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20678,7 +20694,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20746,7 +20762,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20814,7 +20830,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20882,7 +20898,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20950,10 +20966,14 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
-        </is>
-      </c>
-      <c r="K354" s="2" t="inlineStr"/>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
+      <c r="K354" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
       <c r="L354" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -20966,7 +20986,7 @@
       </c>
       <c r="N354" s="2" t="inlineStr">
         <is>
-          <t>5b7e4e654380babb1d10413abe45de88b8649abf8ce4739adc379144db916509</t>
+          <t>f895be4e380ab8a4c3339c53fe500183b00334cc64259a2dacd7b6a6997d1bb3</t>
         </is>
       </c>
     </row>
@@ -21010,7 +21030,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21070,12 +21090,12 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T15:17:55+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L356" s="2" t="inlineStr">
@@ -21090,7 +21110,7 @@
       </c>
       <c r="N356" s="2" t="inlineStr">
         <is>
-          <t>c2074ff35e64cdfcef8257d127e1212cf8dfb576ae7ba58e2ce955aa28ee9d1f</t>
+          <t>c721347f59d4f0e22b59a19a86cd2a180bed800457aa9cf248f70a8c3328317e</t>
         </is>
       </c>
     </row>
@@ -21142,7 +21162,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21206,10 +21226,14 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
-        </is>
-      </c>
-      <c r="K358" s="2" t="inlineStr"/>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
+      <c r="K358" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:34:03+00:00</t>
+        </is>
+      </c>
       <c r="L358" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21222,7 +21246,7 @@
       </c>
       <c r="N358" s="2" t="inlineStr">
         <is>
-          <t>91c199983a848bc7c28834e4b7797feec051d6f4353c7ff91e9e54b56e402708</t>
+          <t>b67a9ed80b45878e9eaaa8689084788bf640d0b3e90a8977779fcf6d9dd30988</t>
         </is>
       </c>
     </row>
@@ -21274,12 +21298,12 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
@@ -21294,7 +21318,7 @@
       </c>
       <c r="N359" s="2" t="inlineStr">
         <is>
-          <t>2aad17d7261e53631df4ef311d46bdb9d37b2fbc79969f32c0689f65bf163b96</t>
+          <t>098f334c4eca6cf2cbc0f0501fa7ff6505360fbc683f216f930909357885bcb7</t>
         </is>
       </c>
     </row>
@@ -21342,7 +21366,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr"/>
@@ -21410,7 +21434,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21470,7 +21494,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21534,7 +21558,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr"/>
@@ -21594,7 +21618,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21662,7 +21686,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr"/>
@@ -21678,7 +21702,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>32eec940ea46c6891a7a967f0f01f66d9e102f7974586199538b2f0169258064</t>
+          <t>9815f0ea269140b867ef7f0919d83132f56373c0aff6932d9955b1273ca791c0</t>
         </is>
       </c>
     </row>
@@ -21730,7 +21754,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr"/>
@@ -21746,7 +21770,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>67dd9cee38bbc411028eeeb8a9c51d415c5a1db92bb27eb50ac66bd36cd0409b</t>
+          <t>6522d4d2dfb347568bece3565076a1e2da3e088b99c15d300ba72755e0f7988b</t>
         </is>
       </c>
     </row>
@@ -21798,7 +21822,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21870,7 +21894,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -21934,7 +21958,7 @@
       </c>
       <c r="J369" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K369" s="2" t="inlineStr"/>
@@ -21998,7 +22022,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22475,7 +22499,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22517,7 +22541,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22551,7 +22575,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22593,7 +22617,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22631,7 +22655,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22669,7 +22693,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22707,7 +22731,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22745,7 +22769,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22787,7 +22811,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22825,7 +22849,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22867,7 +22891,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22909,7 +22933,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -22951,7 +22975,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -22993,7 +23017,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23035,7 +23059,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -23077,7 +23101,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23119,7 +23143,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23161,7 +23185,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23203,7 +23227,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23245,7 +23269,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23287,7 +23311,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23329,7 +23353,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23371,7 +23395,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23409,7 +23433,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23451,7 +23475,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23489,7 +23513,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23531,7 +23555,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23573,7 +23597,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23615,7 +23639,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23657,7 +23681,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -23699,7 +23723,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23737,7 +23761,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23775,7 +23799,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23813,7 +23837,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23855,7 +23879,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23897,7 +23921,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -23935,7 +23959,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -23973,7 +23997,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24015,7 +24039,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24057,7 +24081,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24091,7 +24115,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24133,7 +24157,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24171,7 +24195,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24209,7 +24233,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24251,7 +24275,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24289,7 +24313,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24327,7 +24351,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24365,7 +24389,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24407,7 +24431,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24445,7 +24469,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24487,7 +24511,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24529,7 +24553,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24567,7 +24591,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24609,7 +24633,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24651,7 +24675,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24689,7 +24713,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24727,7 +24751,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24765,7 +24789,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24807,7 +24831,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24845,7 +24869,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24887,7 +24911,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -24929,7 +24953,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -24967,7 +24991,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25009,7 +25033,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25051,7 +25075,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25089,7 +25113,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25131,7 +25155,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25169,7 +25193,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25211,7 +25235,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25253,7 +25277,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25295,7 +25319,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25333,7 +25357,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25371,7 +25395,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25409,7 +25433,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25447,7 +25471,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25485,7 +25509,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25527,7 +25551,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25565,7 +25589,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25603,7 +25627,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25645,7 +25669,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25683,7 +25707,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25725,7 +25749,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25763,7 +25787,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25805,7 +25829,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25843,7 +25867,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25881,7 +25905,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25923,7 +25947,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26345,7 +26369,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -26387,7 +26411,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26429,7 +26453,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26471,7 +26495,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26513,7 +26537,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26555,7 +26579,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26597,7 +26621,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26639,7 +26663,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26681,7 +26705,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26723,7 +26747,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26765,7 +26789,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26807,7 +26831,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26849,7 +26873,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26891,7 +26915,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -26933,7 +26957,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -26975,7 +26999,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27017,7 +27041,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27059,7 +27083,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27101,7 +27125,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27143,7 +27167,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27185,7 +27209,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27227,7 +27251,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27269,7 +27293,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27311,7 +27335,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27353,7 +27377,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27395,7 +27419,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27442,7 +27466,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
@@ -27479,7 +27503,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27521,7 +27545,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27563,7 +27587,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27605,7 +27629,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27647,7 +27671,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27689,7 +27713,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -27731,7 +27755,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27773,7 +27797,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27815,7 +27839,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27857,7 +27881,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27899,7 +27923,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -27937,7 +27961,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -27979,7 +28003,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28021,7 +28045,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28063,7 +28087,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28105,7 +28129,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28147,7 +28171,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28189,7 +28213,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28231,7 +28255,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28273,7 +28297,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28315,7 +28339,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28357,7 +28381,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28399,7 +28423,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28441,7 +28465,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28483,7 +28507,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28525,7 +28549,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28567,7 +28591,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28609,7 +28633,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28651,7 +28675,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28693,7 +28717,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28735,7 +28759,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28777,7 +28801,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28819,7 +28843,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28861,7 +28885,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28903,7 +28927,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -28945,7 +28969,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -28987,7 +29011,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29029,7 +29053,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29071,7 +29095,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29113,7 +29137,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29155,7 +29179,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29197,7 +29221,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29239,7 +29263,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29281,7 +29305,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29323,7 +29347,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29365,7 +29389,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29407,7 +29431,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29449,7 +29473,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29491,7 +29515,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29533,7 +29557,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29575,7 +29599,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29617,7 +29641,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29659,7 +29683,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29701,7 +29725,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29743,7 +29767,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29785,7 +29809,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29827,7 +29851,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29869,7 +29893,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29911,7 +29935,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -29953,12 +29977,12 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H185" s="2" t="inlineStr">
@@ -29995,7 +30019,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30037,7 +30061,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30079,7 +30103,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30121,7 +30145,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30163,7 +30187,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30205,7 +30229,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30247,7 +30271,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30289,7 +30313,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30331,7 +30355,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30373,7 +30397,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30415,7 +30439,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30457,7 +30481,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30499,7 +30523,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30541,7 +30565,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30583,7 +30607,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30625,7 +30649,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30667,7 +30691,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30709,7 +30733,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30751,7 +30775,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30794,7 +30818,7 @@
       <c r="F205" s="2" t="inlineStr"/>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
@@ -30831,7 +30855,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30873,7 +30897,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -30915,7 +30939,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -30957,7 +30981,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -30999,7 +31023,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31041,7 +31065,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31083,7 +31107,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31125,7 +31149,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31167,7 +31191,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31209,7 +31233,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31251,7 +31275,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31293,7 +31317,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31335,7 +31359,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31377,7 +31401,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31419,7 +31443,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31461,7 +31485,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31503,7 +31527,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31545,7 +31569,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31587,7 +31611,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31629,7 +31653,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31671,7 +31695,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31713,7 +31737,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31755,7 +31779,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31797,7 +31821,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31839,7 +31863,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31881,7 +31905,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31923,7 +31947,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -31965,7 +31989,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32007,7 +32031,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32049,7 +32073,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32091,7 +32115,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32133,7 +32157,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32175,7 +32199,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32217,7 +32241,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32259,7 +32283,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32301,7 +32325,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32343,7 +32367,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32385,7 +32409,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32423,7 +32447,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32465,7 +32489,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32503,7 +32527,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32537,7 +32561,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32579,7 +32603,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32617,7 +32641,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32659,7 +32683,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32701,7 +32725,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32739,7 +32763,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32777,7 +32801,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32815,7 +32839,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32853,7 +32877,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32895,7 +32919,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -32933,7 +32957,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -32967,7 +32991,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33005,7 +33029,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33043,7 +33067,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33081,7 +33105,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33123,7 +33147,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33165,7 +33189,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33203,7 +33227,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33245,7 +33269,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33279,7 +33303,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33317,7 +33341,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33355,7 +33379,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33393,7 +33417,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-17 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>72fa80328b9c4686227f4a986a19832ecf252d194f978f745948259f94b79a35</t>
+          <t>f7ebc9b82aca70cf9b2e3d51d38d076ae297b624cfe901ccf6f639663759724d</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6510,7 +6510,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7030,7 +7030,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8078,12 +8078,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8094,7 +8094,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>36cba3959afa1ebd074f0091369259c7a27b47ad1d3a48458e1dc9addc73cd58</t>
+          <t>7baab17d8d8f534c7aef22d84237d371f192ac67e33567a1971168a3a2bcebda</t>
         </is>
       </c>
     </row>
@@ -8146,12 +8146,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8162,7 +8162,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>312937aeef7a59572980b7056eb17f932d193ed21fc77219b6fde9baec9335d9</t>
+          <t>6334ce46d206b82654de3a0cde8b8d8f9dbe192b39756d7d107023ce093d0ff8</t>
         </is>
       </c>
     </row>
@@ -8214,7 +8214,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8614,7 +8614,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8754,7 +8754,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8882,7 +8882,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10718,7 +10718,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10898,7 +10898,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10966,7 +10966,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11038,12 +11038,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11058,7 +11058,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>ca07f195765ce5464ebbb41ee48bc696c3d6bfcd55ca6935963cac3f0eb33fba</t>
+          <t>30fe8c2f142131715b9c15e475c8de94fb6d02257b35ac2776d7c25914279b50</t>
         </is>
       </c>
     </row>
@@ -11110,7 +11110,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11130,7 +11130,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>70e86499b9258eabdfa7947c036fab6c14abca885b2175748569ffa5ab7f8669</t>
+          <t>36139f42d3c8a3242c04ae064455730837b3860009feaaf9de03f59dfd2e2ab2</t>
         </is>
       </c>
     </row>
@@ -11182,14 +11182,14 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
+          <t>2026-10-17T11:48:17+00:00</t>
+        </is>
+      </c>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
           <t>2026-10-16T12:34:03+00:00</t>
         </is>
       </c>
-      <c r="K195" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-16T12:34:03+00:00</t>
-        </is>
-      </c>
       <c r="L195" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>32df9e260ab4093d0d9b60083b627784f3c48080b194b85688f06449dfc22f37</t>
+          <t>6adb41d16dc965d153ab2db214d04de1c6a3483ba810d3142360e38e43e83852</t>
         </is>
       </c>
     </row>
@@ -11254,7 +11254,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11326,7 +11326,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11466,7 +11466,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11610,7 +11610,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11750,7 +11750,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11822,7 +11822,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11842,7 +11842,7 @@
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>e386a49fc405e8f0578ce0070f1916df213f95355fa7210de1fe27beac7d0f97</t>
+          <t>ffb5beb7f39ba9a938dc63c73cb119609bd6bfd8a80196d3adbbc32fa4fe2ffd</t>
         </is>
       </c>
     </row>
@@ -11894,7 +11894,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12026,7 +12026,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12046,7 +12046,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>b2a60b2bda13220281b4129225034a4c70848f134bae8af314dc185d5619e5f6</t>
+          <t>abdcb5c9c9ba2fec3bbc78a104a53261117b2fc19cc2510708187da1cc60737f</t>
         </is>
       </c>
     </row>
@@ -12098,7 +12098,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12166,12 +12166,12 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
@@ -12186,7 +12186,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
+          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
         </is>
       </c>
     </row>
@@ -12238,7 +12238,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12534,7 +12534,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12782,7 +12782,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12854,12 +12854,12 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L220" s="2" t="inlineStr">
@@ -12874,7 +12874,7 @@
       </c>
       <c r="N220" s="2" t="inlineStr">
         <is>
-          <t>cfffc1773d5fcbeefc5f1f05d3996da8400db2f4c889dbe4c70b1df9730cffb1</t>
+          <t>19fab800776b7c2cb44522f479ef68fc38d89692f4288a4f9a96b46ab7cdee96</t>
         </is>
       </c>
     </row>
@@ -12926,12 +12926,12 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L221" s="2" t="inlineStr">
@@ -12946,7 +12946,7 @@
       </c>
       <c r="N221" s="2" t="inlineStr">
         <is>
-          <t>90a85363c454b0894939ab271ef928998ece74001cf74e1c6ccfa44ff72cfc6c</t>
+          <t>566d3742be876dd99562e6745a2dcec068bac6341538e8fd46873761dfb825a8</t>
         </is>
       </c>
     </row>
@@ -13118,12 +13118,12 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L224" s="2" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="N224" s="2" t="inlineStr">
         <is>
-          <t>51216777fbb4726211a885940169761b21a52d18b6357fa744629970d16f9f68</t>
+          <t>0cc238ff6f7dbe714fe0b679325ba9e11308a043e67a3fac0fa4e6d1b86d0b56</t>
         </is>
       </c>
     </row>
@@ -13190,12 +13190,12 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L225" s="2" t="inlineStr">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="N225" s="2" t="inlineStr">
         <is>
-          <t>b085021fb3874f27b526face8ac99466487c72a05b9c9f31af36c937a015c7d2</t>
+          <t>ef60379d56cadbbba4ae27644f59d9e8b84900d72f9f80ed2cd075e71d07da73</t>
         </is>
       </c>
     </row>
@@ -13262,7 +13262,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13330,7 +13330,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13398,7 +13398,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13466,7 +13466,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13590,7 +13590,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13610,7 +13610,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>84f5926aa0671dc0e4638c60833270b8caa5aed5ad58bf2a48a22437637be9e2</t>
+          <t>e7809469f697b463e46cfba1a909cab1ca36dcf6d1368ba77eb8d3c3c8560363</t>
         </is>
       </c>
     </row>
@@ -13902,12 +13902,12 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
@@ -13922,7 +13922,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>20731603a546316575d8e7b09a41dce5926d79d4e84fbf3566de18f902cd83a7</t>
+          <t>2c13498c744f343d33086f2c9ae01b496eaa4d63f096edc6c22febe763ba1cc7</t>
         </is>
       </c>
     </row>
@@ -18174,7 +18174,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18194,7 +18194,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>0d0903557b20b250d77fe4717ab0e84fd0e6cf11f2c019013fb01d38eac5720f</t>
+          <t>61b3451cf0944575a0f283ac95411d2886f36165ee8db5aec2cf7cbcece34bb1</t>
         </is>
       </c>
     </row>
@@ -18246,7 +18246,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
@@ -18266,7 +18266,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>50316d07b996d21720b7a8379e686ec76f0db2ccb316579fa9a2f5a564972f69</t>
+          <t>4616db71c764b6e6eb5bd20fd5f2578585169ff4948c75025dc7c555aec93c2e</t>
         </is>
       </c>
     </row>
@@ -18318,7 +18318,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18390,7 +18390,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18526,7 +18526,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18650,7 +18650,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19078,7 +19078,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19146,7 +19146,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19214,7 +19214,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19282,12 +19282,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19302,7 +19302,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>2e591b0c09df4e353760136ded8ef7f8d8812f4758686f6c12ab2c679ce6bb86</t>
+          <t>05294c4bbc2466ecf8ac919b938091a2977a12cbf44ef16119de8f3d52ddd1f3</t>
         </is>
       </c>
     </row>
@@ -19354,12 +19354,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19374,7 +19374,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>4a488d1ace17372fa512e68d9b22e710519ce4d9070faa8938f2a68e93c10252</t>
+          <t>9a5b449546d7465c21a93d205ecab5fac49f19f4deedbc80b010000e1c6e968c</t>
         </is>
       </c>
     </row>
@@ -19426,12 +19426,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19446,7 +19446,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>7944c275492ab2f1fea7287aa95c4e42d6b85ce22036152bcf526a5f46161816</t>
+          <t>7287ad8327cdfdfb51f0d48e5cb2425332266834ee184b0bbc0683bc21c8fb94</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19498,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr"/>
@@ -19622,7 +19622,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19690,7 +19690,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19758,7 +19758,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19826,7 +19826,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr"/>
@@ -19894,7 +19894,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr"/>
@@ -19962,7 +19962,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20030,7 +20030,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20098,7 +20098,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20166,12 +20166,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20186,7 +20186,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>0e91c37168f822ae6a127d93eda2e34af04d9fac70a4b1b8bf3321e2709eb87f</t>
+          <t>e7f94bc8b73143f194434a6334a9fd137ffba7dc9a911c6abf21148d33c41d91</t>
         </is>
       </c>
     </row>
@@ -20354,10 +20354,14 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
-        </is>
-      </c>
-      <c r="K345" s="2" t="inlineStr"/>
+          <t>2026-10-17T11:48:17+00:00</t>
+        </is>
+      </c>
+      <c r="K345" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:48:17+00:00</t>
+        </is>
+      </c>
       <c r="L345" s="2" t="inlineStr">
         <is>
           <t>2026-10-08</t>
@@ -20370,7 +20374,7 @@
       </c>
       <c r="N345" s="2" t="inlineStr">
         <is>
-          <t>c31211e6e78496e706641583348f9e7896ed2e9deced3e7afead68283d64a796</t>
+          <t>e76659ac627775637691c41a20eabcddc98efeb1fab5de61136736c231820cf8</t>
         </is>
       </c>
     </row>
@@ -20422,7 +20426,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20490,7 +20494,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20558,7 +20562,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20626,7 +20630,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20694,7 +20698,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20762,7 +20766,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20830,7 +20834,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20898,7 +20902,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20966,7 +20970,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21030,7 +21034,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21090,12 +21094,12 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L356" s="2" t="inlineStr">
@@ -21110,7 +21114,7 @@
       </c>
       <c r="N356" s="2" t="inlineStr">
         <is>
-          <t>c721347f59d4f0e22b59a19a86cd2a180bed800457aa9cf248f70a8c3328317e</t>
+          <t>27ac47efac33f73afa4ce1afc99223a29baa9e443c63aef58d793d50d4d6df17</t>
         </is>
       </c>
     </row>
@@ -21162,7 +21166,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21226,7 +21230,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21298,12 +21302,12 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
@@ -21318,7 +21322,7 @@
       </c>
       <c r="N359" s="2" t="inlineStr">
         <is>
-          <t>098f334c4eca6cf2cbc0f0501fa7ff6505360fbc683f216f930909357885bcb7</t>
+          <t>41f612f0e3ffcea81f8321b1e683e2175c83f8ab6ef9dbdc3d969489347cd0e1</t>
         </is>
       </c>
     </row>
@@ -21366,7 +21370,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr"/>
@@ -21434,7 +21438,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21494,7 +21498,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21558,7 +21562,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr"/>
@@ -21618,7 +21622,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21686,7 +21690,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr"/>
@@ -21702,7 +21706,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>9815f0ea269140b867ef7f0919d83132f56373c0aff6932d9955b1273ca791c0</t>
+          <t>c4881f1d79a1e69896a01eddecd87c63783b11e98872b8b54f4c1828c02dcdc3</t>
         </is>
       </c>
     </row>
@@ -21754,7 +21758,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr"/>
@@ -21770,7 +21774,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>6522d4d2dfb347568bece3565076a1e2da3e088b99c15d300ba72755e0f7988b</t>
+          <t>5258a21da90498d46b71d112e64904dd3259224dea95acda2c0bb8888aa44bd5</t>
         </is>
       </c>
     </row>
@@ -21822,7 +21826,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21894,7 +21898,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -21958,7 +21962,7 @@
       </c>
       <c r="J369" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K369" s="2" t="inlineStr"/>
@@ -22022,7 +22026,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22499,7 +22503,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22541,7 +22545,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22575,7 +22579,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22617,7 +22621,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22655,7 +22659,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22693,7 +22697,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22731,7 +22735,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22769,7 +22773,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22811,7 +22815,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22849,7 +22853,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22891,7 +22895,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22933,7 +22937,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -22975,7 +22979,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23017,7 +23021,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23059,7 +23063,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -23101,7 +23105,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23143,7 +23147,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23185,7 +23189,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23227,7 +23231,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23269,7 +23273,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23311,7 +23315,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23353,7 +23357,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23395,7 +23399,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23433,7 +23437,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23475,7 +23479,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23513,7 +23517,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23555,7 +23559,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23597,7 +23601,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23639,7 +23643,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23681,7 +23685,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -23723,7 +23727,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23761,7 +23765,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23799,7 +23803,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23837,7 +23841,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23879,7 +23883,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23921,7 +23925,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -23959,7 +23963,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -23997,7 +24001,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24039,7 +24043,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24081,7 +24085,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24115,7 +24119,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24157,7 +24161,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24195,7 +24199,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24233,7 +24237,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24275,7 +24279,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24313,7 +24317,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24351,7 +24355,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24389,7 +24393,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24431,7 +24435,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24469,7 +24473,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24511,7 +24515,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24553,7 +24557,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24591,7 +24595,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24633,7 +24637,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24675,7 +24679,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24713,7 +24717,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24751,7 +24755,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24789,7 +24793,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24831,7 +24835,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24869,7 +24873,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24911,7 +24915,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -24953,7 +24957,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -24991,7 +24995,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25033,7 +25037,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25075,7 +25079,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25113,7 +25117,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25155,7 +25159,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25193,7 +25197,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25235,7 +25239,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25277,7 +25281,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25319,7 +25323,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25357,7 +25361,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25395,7 +25399,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25433,7 +25437,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25471,7 +25475,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25509,7 +25513,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25551,7 +25555,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25589,7 +25593,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25627,7 +25631,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25669,7 +25673,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25707,7 +25711,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25749,7 +25753,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25787,7 +25791,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25829,7 +25833,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25867,7 +25871,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25905,7 +25909,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25947,7 +25951,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26369,7 +26373,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -26416,7 +26420,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
@@ -26453,7 +26457,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26495,7 +26499,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26537,7 +26541,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26579,7 +26583,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26621,7 +26625,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26663,7 +26667,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26705,7 +26709,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26747,7 +26751,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26789,7 +26793,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26831,7 +26835,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26873,7 +26877,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26915,7 +26919,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -26957,7 +26961,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -26999,7 +27003,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27041,7 +27045,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27083,7 +27087,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27125,7 +27129,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27167,7 +27171,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27209,7 +27213,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27251,7 +27255,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27293,7 +27297,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27335,7 +27339,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27377,7 +27381,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27419,7 +27423,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27461,12 +27465,12 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
@@ -27503,7 +27507,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27545,7 +27549,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27587,7 +27591,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27629,7 +27633,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27671,7 +27675,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27713,7 +27717,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -27755,7 +27759,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27797,7 +27801,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27839,7 +27843,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27881,7 +27885,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27923,7 +27927,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -27961,7 +27965,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28003,7 +28007,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28045,7 +28049,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28087,7 +28091,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28129,7 +28133,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28171,7 +28175,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28213,7 +28217,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28255,7 +28259,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28297,7 +28301,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28339,7 +28343,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28381,7 +28385,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28423,7 +28427,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28465,7 +28469,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28507,7 +28511,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28549,7 +28553,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28591,7 +28595,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28633,7 +28637,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28675,7 +28679,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28717,7 +28721,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28759,7 +28763,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28801,7 +28805,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28843,7 +28847,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28885,7 +28889,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28927,7 +28931,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -28969,7 +28973,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29011,7 +29015,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29053,7 +29057,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29095,7 +29099,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29137,7 +29141,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29179,7 +29183,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29221,7 +29225,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29263,7 +29267,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29305,7 +29309,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29347,7 +29351,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29389,7 +29393,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29431,7 +29435,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29473,7 +29477,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29515,7 +29519,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29557,7 +29561,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29599,7 +29603,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29641,7 +29645,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29683,7 +29687,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29725,7 +29729,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29767,7 +29771,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29809,7 +29813,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29851,7 +29855,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29893,7 +29897,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29935,7 +29939,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -29977,7 +29981,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30019,7 +30023,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30061,7 +30065,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30103,7 +30107,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30145,7 +30149,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30187,7 +30191,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30229,7 +30233,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30271,7 +30275,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30313,7 +30317,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30355,7 +30359,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30397,7 +30401,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30439,7 +30443,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30481,7 +30485,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30523,7 +30527,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30565,7 +30569,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30607,7 +30611,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30649,7 +30653,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30691,7 +30695,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30733,7 +30737,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30775,7 +30779,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30855,7 +30859,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30897,7 +30901,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -30939,7 +30943,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -30981,7 +30985,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31023,7 +31027,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31065,7 +31069,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31107,7 +31111,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31149,7 +31153,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31191,7 +31195,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31233,7 +31237,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31275,7 +31279,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31317,7 +31321,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31359,7 +31363,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31401,7 +31405,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31443,7 +31447,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31485,7 +31489,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31527,7 +31531,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31569,7 +31573,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31611,7 +31615,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31653,7 +31657,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31695,7 +31699,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31737,7 +31741,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31779,7 +31783,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31821,7 +31825,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31863,7 +31867,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31905,7 +31909,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31947,7 +31951,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -31989,7 +31993,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32031,7 +32035,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32073,7 +32077,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32115,7 +32119,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32157,7 +32161,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32199,7 +32203,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32241,7 +32245,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32283,7 +32287,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32325,7 +32329,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32367,7 +32371,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32409,7 +32413,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32447,7 +32451,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32489,7 +32493,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32527,7 +32531,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32561,7 +32565,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32603,7 +32607,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32641,7 +32645,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32683,7 +32687,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32725,7 +32729,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32763,7 +32767,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32801,7 +32805,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32839,7 +32843,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32877,7 +32881,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32919,7 +32923,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -32957,7 +32961,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -32991,7 +32995,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33029,7 +33033,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33067,7 +33071,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33105,7 +33109,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33147,7 +33151,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33189,7 +33193,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33227,7 +33231,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33269,7 +33273,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33303,7 +33307,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33341,7 +33345,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33379,7 +33383,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33417,7 +33421,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-18 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6510,7 +6510,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6682,7 +6682,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7030,7 +7030,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8014,7 +8014,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8078,12 +8078,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8094,7 +8094,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>7baab17d8d8f534c7aef22d84237d371f192ac67e33567a1971168a3a2bcebda</t>
+          <t>6a687e09dcbd44b47021710e5a1692edb93db1e96198b96dc9520b296aa1d2e0</t>
         </is>
       </c>
     </row>
@@ -8146,12 +8146,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8162,7 +8162,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>6334ce46d206b82654de3a0cde8b8d8f9dbe192b39756d7d107023ce093d0ff8</t>
+          <t>688b59e1940f8558ac7e55ed694a441ec9032ec1cffc16fac427b2f650e74f87</t>
         </is>
       </c>
     </row>
@@ -8214,7 +8214,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8614,7 +8614,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8754,7 +8754,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8882,7 +8882,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10718,7 +10718,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10898,7 +10898,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10966,7 +10966,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11038,12 +11038,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11058,7 +11058,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>30fe8c2f142131715b9c15e475c8de94fb6d02257b35ac2776d7c25914279b50</t>
+          <t>a451f82ddec64c75e8e51db868fd24fee6be5c990476fcde56c2f161b84ec8f5</t>
         </is>
       </c>
     </row>
@@ -11110,7 +11110,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11182,7 +11182,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11254,7 +11254,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11326,7 +11326,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11398,7 +11398,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11466,7 +11466,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11610,12 +11610,12 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L201" s="2" t="inlineStr">
@@ -11630,7 +11630,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>8eab33f6305b65fe1f19eaa8ea7b68e36a0809fc821a1d1994609db876cec98b</t>
+          <t>56094f2b4d126f65a87c1ecfaea43016bd44c932ad5273febaa3a31c97272732</t>
         </is>
       </c>
     </row>
@@ -11682,7 +11682,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11750,7 +11750,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11822,7 +11822,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11894,7 +11894,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12026,7 +12026,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12046,7 +12046,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>abdcb5c9c9ba2fec3bbc78a104a53261117b2fc19cc2510708187da1cc60737f</t>
+          <t>e96aa77982e88d1fa8e4974e36d2b784c94a6b97cf7f3edaf5d2778bddd01fca</t>
         </is>
       </c>
     </row>
@@ -12098,7 +12098,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12166,7 +12166,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12238,7 +12238,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12534,7 +12534,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12782,7 +12782,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12854,7 +12854,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
@@ -12926,7 +12926,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13118,12 +13118,12 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L224" s="2" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="N224" s="2" t="inlineStr">
         <is>
-          <t>0cc238ff6f7dbe714fe0b679325ba9e11308a043e67a3fac0fa4e6d1b86d0b56</t>
+          <t>2e2894032e176a76d127e4db8a9f3833d33514260d5800f0ece93f0afc6cd36f</t>
         </is>
       </c>
     </row>
@@ -13190,12 +13190,12 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L225" s="2" t="inlineStr">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="N225" s="2" t="inlineStr">
         <is>
-          <t>ef60379d56cadbbba4ae27644f59d9e8b84900d72f9f80ed2cd075e71d07da73</t>
+          <t>110854495c4db790459d37d4697b16a590f53433911d7e99adc6c8208be619af</t>
         </is>
       </c>
     </row>
@@ -13262,7 +13262,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13330,7 +13330,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13398,7 +13398,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13466,7 +13466,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13590,7 +13590,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13610,7 +13610,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>e7809469f697b463e46cfba1a909cab1ca36dcf6d1368ba77eb8d3c3c8560363</t>
+          <t>a55a21f9c39028df1294608bfa4eea59bcb8dbf9cd3fc8ac33b197e038e27e34</t>
         </is>
       </c>
     </row>
@@ -13902,12 +13902,12 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
@@ -13922,7 +13922,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>2c13498c744f343d33086f2c9ae01b496eaa4d63f096edc6c22febe763ba1cc7</t>
+          <t>2e25a95222d317078bbf8dfa9601f6462e9f5a4ab14074055ba43c832480b32e</t>
         </is>
       </c>
     </row>
@@ -18174,7 +18174,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18194,7 +18194,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>61b3451cf0944575a0f283ac95411d2886f36165ee8db5aec2cf7cbcece34bb1</t>
+          <t>0d0903557b20b250d77fe4717ab0e84fd0e6cf11f2c019013fb01d38eac5720f</t>
         </is>
       </c>
     </row>
@@ -18246,7 +18246,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
@@ -18318,7 +18318,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18390,7 +18390,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18458,7 +18458,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18526,7 +18526,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18650,7 +18650,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19078,7 +19078,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19146,7 +19146,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19214,7 +19214,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19282,12 +19282,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19302,7 +19302,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>05294c4bbc2466ecf8ac919b938091a2977a12cbf44ef16119de8f3d52ddd1f3</t>
+          <t>72a174dcb1631cc60d7930249d35e4ae17f3e629526663a9d781a1f3ebf1a443</t>
         </is>
       </c>
     </row>
@@ -19354,14 +19354,14 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
+          <t>2026-10-18T12:17:25+00:00</t>
+        </is>
+      </c>
+      <c r="K330" s="2" t="inlineStr">
+        <is>
           <t>2026-10-17T11:48:17+00:00</t>
         </is>
       </c>
-      <c r="K330" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-17T11:48:17+00:00</t>
-        </is>
-      </c>
       <c r="L330" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -19374,7 +19374,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>9a5b449546d7465c21a93d205ecab5fac49f19f4deedbc80b010000e1c6e968c</t>
+          <t>fcfca8b6f889c15e0cbf6cb71c2a5065776afc881ac325f53b42ec151be3b4b8</t>
         </is>
       </c>
     </row>
@@ -19426,12 +19426,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19446,7 +19446,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>7287ad8327cdfdfb51f0d48e5cb2425332266834ee184b0bbc0683bc21c8fb94</t>
+          <t>123b67aadcd8164eb719761b68ac3e636b431c24f3b1c3ec8da859e1c21abad8</t>
         </is>
       </c>
     </row>
@@ -19498,7 +19498,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr"/>
@@ -19622,7 +19622,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19690,7 +19690,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19758,7 +19758,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19826,7 +19826,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr"/>
@@ -19894,7 +19894,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr"/>
@@ -19962,7 +19962,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20030,7 +20030,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20098,7 +20098,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20166,12 +20166,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20186,7 +20186,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>e7f94bc8b73143f194434a6334a9fd137ffba7dc9a911c6abf21148d33c41d91</t>
+          <t>d1bafb5c8d38ee8e3d01b1fd0699c476fb41dac9ce457811e781c68cc102d2f7</t>
         </is>
       </c>
     </row>
@@ -20354,7 +20354,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
@@ -20426,7 +20426,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20494,7 +20494,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20562,7 +20562,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20630,7 +20630,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20698,7 +20698,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20766,7 +20766,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20834,7 +20834,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20902,7 +20902,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20970,7 +20970,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21034,7 +21034,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21094,12 +21094,12 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L356" s="2" t="inlineStr">
@@ -21114,7 +21114,7 @@
       </c>
       <c r="N356" s="2" t="inlineStr">
         <is>
-          <t>27ac47efac33f73afa4ce1afc99223a29baa9e443c63aef58d793d50d4d6df17</t>
+          <t>c721347f59d4f0e22b59a19a86cd2a180bed800457aa9cf248f70a8c3328317e</t>
         </is>
       </c>
     </row>
@@ -21166,7 +21166,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21230,7 +21230,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21302,12 +21302,12 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
@@ -21322,7 +21322,7 @@
       </c>
       <c r="N359" s="2" t="inlineStr">
         <is>
-          <t>41f612f0e3ffcea81f8321b1e683e2175c83f8ab6ef9dbdc3d969489347cd0e1</t>
+          <t>38743bb78af9166ea525f7b20c558f810adcc480dc2ab6f996629b82dc428c09</t>
         </is>
       </c>
     </row>
@@ -21370,7 +21370,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr"/>
@@ -21438,7 +21438,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21498,7 +21498,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21562,7 +21562,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr"/>
@@ -21622,7 +21622,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21690,7 +21690,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr"/>
@@ -21758,7 +21758,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr"/>
@@ -21774,7 +21774,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>5258a21da90498d46b71d112e64904dd3259224dea95acda2c0bb8888aa44bd5</t>
+          <t>0de74c5f149310d319d1487b66fd757a5947800233f8a565a73f61104c2a9ec9</t>
         </is>
       </c>
     </row>
@@ -21826,7 +21826,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21898,7 +21898,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -21962,7 +21962,7 @@
       </c>
       <c r="J369" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K369" s="2" t="inlineStr"/>
@@ -22026,7 +22026,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22503,7 +22503,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22545,7 +22545,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22579,7 +22579,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22621,7 +22621,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22659,7 +22659,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22697,7 +22697,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22735,7 +22735,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22773,7 +22773,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22815,7 +22815,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22853,7 +22853,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22895,7 +22895,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22937,7 +22937,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -22979,7 +22979,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23021,7 +23021,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23063,7 +23063,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -23105,7 +23105,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23147,7 +23147,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23189,7 +23189,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23231,7 +23231,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23273,7 +23273,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23315,7 +23315,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23357,7 +23357,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23399,7 +23399,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23437,7 +23437,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23479,7 +23479,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23517,7 +23517,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23559,7 +23559,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23601,7 +23601,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23643,7 +23643,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23685,7 +23685,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -23727,7 +23727,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23765,7 +23765,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23803,7 +23803,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23841,7 +23841,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23883,7 +23883,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23925,7 +23925,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -23963,7 +23963,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24001,7 +24001,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24043,7 +24043,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24085,7 +24085,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24119,7 +24119,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24161,7 +24161,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24199,7 +24199,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24237,7 +24237,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24279,7 +24279,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24317,7 +24317,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24355,7 +24355,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24393,7 +24393,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24435,7 +24435,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24473,7 +24473,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24515,7 +24515,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24557,7 +24557,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24595,7 +24595,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24637,7 +24637,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24679,7 +24679,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24717,7 +24717,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24755,7 +24755,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24793,7 +24793,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24835,7 +24835,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24873,7 +24873,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24915,7 +24915,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -24957,7 +24957,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -24995,7 +24995,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25037,7 +25037,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25079,7 +25079,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25117,7 +25117,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25159,7 +25159,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25197,7 +25197,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25239,7 +25239,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25281,7 +25281,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25323,7 +25323,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25361,7 +25361,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25399,7 +25399,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25437,7 +25437,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25475,7 +25475,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25513,7 +25513,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25555,7 +25555,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25593,7 +25593,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25631,7 +25631,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25673,7 +25673,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25711,7 +25711,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25753,7 +25753,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25791,7 +25791,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25833,7 +25833,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25871,7 +25871,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25909,7 +25909,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25951,7 +25951,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26373,7 +26373,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -26415,12 +26415,12 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26499,7 +26499,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26541,7 +26541,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26583,7 +26583,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26625,7 +26625,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26667,7 +26667,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26709,7 +26709,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26751,7 +26751,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26793,7 +26793,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26835,7 +26835,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26877,7 +26877,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26919,7 +26919,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -26961,7 +26961,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27003,7 +27003,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27045,7 +27045,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27087,7 +27087,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27129,7 +27129,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27171,7 +27171,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27213,7 +27213,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27297,7 +27297,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27339,7 +27339,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27381,7 +27381,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27423,7 +27423,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27465,7 +27465,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27507,7 +27507,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27549,7 +27549,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27591,7 +27591,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27633,7 +27633,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27675,7 +27675,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27717,7 +27717,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -27759,7 +27759,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27801,7 +27801,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27843,7 +27843,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27885,7 +27885,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27927,7 +27927,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -27965,7 +27965,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28007,7 +28007,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28049,7 +28049,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28091,7 +28091,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28133,7 +28133,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28175,7 +28175,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28217,7 +28217,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28259,7 +28259,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28301,7 +28301,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28343,7 +28343,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28385,7 +28385,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28427,7 +28427,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28469,7 +28469,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28511,7 +28511,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28553,7 +28553,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28595,7 +28595,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28637,7 +28637,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28679,7 +28679,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28721,7 +28721,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28763,7 +28763,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28805,7 +28805,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28847,7 +28847,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28889,7 +28889,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28931,7 +28931,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -28973,7 +28973,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29015,7 +29015,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29057,7 +29057,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29099,7 +29099,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29141,7 +29141,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29183,7 +29183,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29225,7 +29225,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29267,7 +29267,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29309,7 +29309,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29351,7 +29351,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29393,7 +29393,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29435,7 +29435,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29477,7 +29477,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29519,7 +29519,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29561,7 +29561,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29603,7 +29603,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29645,7 +29645,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29687,7 +29687,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29729,7 +29729,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29771,7 +29771,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29813,7 +29813,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29855,7 +29855,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29897,7 +29897,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29939,7 +29939,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -29981,7 +29981,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30023,7 +30023,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30065,7 +30065,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30107,7 +30107,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30149,7 +30149,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30191,7 +30191,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30233,7 +30233,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30275,7 +30275,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30317,7 +30317,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30359,7 +30359,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30401,7 +30401,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30443,7 +30443,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30485,7 +30485,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30527,7 +30527,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30569,7 +30569,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30611,7 +30611,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30653,7 +30653,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30695,7 +30695,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30737,7 +30737,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30779,7 +30779,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30822,7 +30822,7 @@
       <c r="F205" s="2" t="inlineStr"/>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
@@ -30859,7 +30859,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30901,7 +30901,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -30943,7 +30943,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -30985,7 +30985,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31027,7 +31027,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31069,7 +31069,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31111,7 +31111,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31153,7 +31153,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31195,7 +31195,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31237,7 +31237,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31279,7 +31279,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31321,7 +31321,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31363,7 +31363,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31405,7 +31405,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31447,7 +31447,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31489,7 +31489,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31531,7 +31531,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31573,7 +31573,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31615,7 +31615,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31657,7 +31657,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31699,7 +31699,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31741,7 +31741,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31783,7 +31783,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31825,7 +31825,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31867,7 +31867,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31909,7 +31909,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -31993,7 +31993,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32035,7 +32035,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32077,7 +32077,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32119,7 +32119,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32161,7 +32161,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32203,7 +32203,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32245,7 +32245,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32287,7 +32287,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32329,7 +32329,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32371,7 +32371,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32413,7 +32413,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32451,7 +32451,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32493,7 +32493,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32531,7 +32531,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32565,7 +32565,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32607,7 +32607,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32645,7 +32645,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32687,7 +32687,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32729,7 +32729,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32767,7 +32767,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32805,7 +32805,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32843,7 +32843,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32881,7 +32881,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32923,7 +32923,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -32961,7 +32961,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -32995,7 +32995,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33033,7 +33033,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33071,7 +33071,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33109,7 +33109,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33151,7 +33151,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33193,7 +33193,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33231,7 +33231,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33273,7 +33273,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33307,7 +33307,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33345,7 +33345,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33383,7 +33383,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33421,7 +33421,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-18T12:17:25+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-20 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4606,7 +4606,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5130,7 +5130,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6686,7 +6686,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6814,7 +6814,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7034,7 +7034,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8018,7 +8018,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8082,12 +8082,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8098,7 +8098,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>1b7040d1f354b91588a40927b30a5932140fd4936046a12410883621dc7a524a</t>
+          <t>c021c4041ce4dc03831616e440890021b615291cdd179e1f1bcadf9f41de4335</t>
         </is>
       </c>
     </row>
@@ -8150,12 +8150,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8166,7 +8166,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>aa3ace8d84a08a27619d007038e8d23656b54b6fea38a1de634c8cab91e7531d</t>
+          <t>910a08a9481d0d46f86571f7d76ffe8441d4d15d8ea85a5c39e1d6223789262e</t>
         </is>
       </c>
     </row>
@@ -8218,7 +8218,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8282,7 +8282,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8618,7 +8618,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8686,7 +8686,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8886,7 +8886,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8954,7 +8954,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9026,7 +9026,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10722,7 +10722,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10970,7 +10970,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11042,12 +11042,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11062,7 +11062,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>8efef8cf5d6b6f0b6f835eb87f7c5160ebe5a2935e268cddc49afb26b0137c02</t>
+          <t>cd0cce8218c4575ec3af4f8bb933efafdf1588bda7e40c12c90776d1c5f3023b</t>
         </is>
       </c>
     </row>
@@ -11114,7 +11114,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11134,7 +11134,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>36139f42d3c8a3242c04ae064455730837b3860009feaaf9de03f59dfd2e2ab2</t>
+          <t>c6ed104cf8e1d42a1384100a7ddb77237218d475dec8ee7d0e7ac173091b2784</t>
         </is>
       </c>
     </row>
@@ -11186,7 +11186,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11258,7 +11258,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11278,7 +11278,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>b6b27a7efe1d73b642f07e8f2ffa02beea94d20c7ba545b0d8ec777beb02589c</t>
+          <t>bdf3568cdc3ba102a5f566e30d8212ed74540600f72c5f313b3ecbc2fd5e7dfd</t>
         </is>
       </c>
     </row>
@@ -11330,7 +11330,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11402,7 +11402,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11470,7 +11470,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11542,7 +11542,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11614,7 +11614,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11686,7 +11686,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11754,7 +11754,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11826,7 +11826,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11898,7 +11898,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12030,7 +12030,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12050,7 +12050,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>e86c3556d34454e09cb752a904458e89943d5351b97a0ac4a3e015313909eb86</t>
+          <t>06087b9e6a42cd27c16a90c9604b634af5ed9e643e26c0d5a61830976615ff5d</t>
         </is>
       </c>
     </row>
@@ -12102,7 +12102,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12170,7 +12170,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12242,7 +12242,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12538,7 +12538,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12786,7 +12786,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12858,7 +12858,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
@@ -12930,7 +12930,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13122,7 +13122,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
@@ -13194,7 +13194,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
@@ -13266,7 +13266,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13334,7 +13334,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13402,7 +13402,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13470,7 +13470,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13594,7 +13594,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13906,12 +13906,12 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T12:17:25+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
@@ -13926,7 +13926,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>568d2f61e69c05bd3b213c5a8066003df041553bbadada8d2af7d23f2242ff56</t>
+          <t>fbd52d099b3cd790415c9b4b7102254ae76bb6fcea716a16a3a9dd19071c2ba7</t>
         </is>
       </c>
     </row>
@@ -18178,7 +18178,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18245,17 +18245,17 @@
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>open</t>
         </is>
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L313" s="2" t="inlineStr">
@@ -18270,7 +18270,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>7e3beb4b17becfcb7b8c3472521dd12af42112052aeb2ae7588d2da76c22f686</t>
+          <t>14e70d7c9a42cbe6a76662006e078f068b5e1acba1aeb715646fdd064d401ade</t>
         </is>
       </c>
     </row>
@@ -18322,7 +18322,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18394,7 +18394,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18462,7 +18462,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18530,7 +18530,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18654,7 +18654,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19082,7 +19082,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19150,7 +19150,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19218,7 +19218,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19286,12 +19286,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19306,7 +19306,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>e228c366ab3993f5dd32a84f4999a55ae565583901dbd8198a5b47e5becf5ba2</t>
+          <t>8e46886461a72f2868f1bff40bde0a367fe70c6a382f518d572eff16ac23e140</t>
         </is>
       </c>
     </row>
@@ -19358,12 +19358,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19378,7 +19378,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>1ab0bb37c414099c91230203c0c4d1893a6fcfffa5731e1c1419dd5f0de90571</t>
+          <t>0ae11458ac0177bcb5f1c83271eddff0ac4983af740f98ec95a6e80193beea15</t>
         </is>
       </c>
     </row>
@@ -19430,12 +19430,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T12:17:25+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19450,7 +19450,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>4a2c7248e4ada9ce3d1ee8264f6f35bc7d4ba160b2aeda14d68a6d7e2531ec09</t>
+          <t>b109beef131f84dba656c91e4c6a53cc2d74cc0872796db986f5c6fdd70fe3d9</t>
         </is>
       </c>
     </row>
@@ -19502,7 +19502,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr"/>
@@ -19626,7 +19626,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19694,7 +19694,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19762,7 +19762,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19830,7 +19830,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr"/>
@@ -19898,7 +19898,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
@@ -19970,7 +19970,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20038,7 +20038,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20106,7 +20106,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20174,12 +20174,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20194,7 +20194,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>281eb2a97ff4c38c050532738de24e7f7c33a208c71d58f7e7064571a1e0fb1d</t>
+          <t>e7119ca281c6cde2573e4e86bbfbe8bafc112365df40306f9380d498643901b9</t>
         </is>
       </c>
     </row>
@@ -20362,12 +20362,12 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L345" s="2" t="inlineStr">
@@ -20382,7 +20382,7 @@
       </c>
       <c r="N345" s="2" t="inlineStr">
         <is>
-          <t>6c91b2968037233883f4d361f5184c14b2a27fe17b5feace6fd1a8eb7735447d</t>
+          <t>09e3d13d618416b17d293449518960b6a61d3ad9c936275336619d5a8cad8155</t>
         </is>
       </c>
     </row>
@@ -20434,7 +20434,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20502,7 +20502,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20570,7 +20570,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20638,7 +20638,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20706,7 +20706,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20774,7 +20774,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20842,7 +20842,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20910,7 +20910,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20978,7 +20978,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21042,7 +21042,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21102,12 +21102,12 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T12:17:25+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="L356" s="2" t="inlineStr">
@@ -21122,7 +21122,7 @@
       </c>
       <c r="N356" s="2" t="inlineStr">
         <is>
-          <t>c721347f59d4f0e22b59a19a86cd2a180bed800457aa9cf248f70a8c3328317e</t>
+          <t>a2af2ebdebf208620cf66854edcb74df672ccd44856b6b7f7fa358a681717078</t>
         </is>
       </c>
     </row>
@@ -21174,7 +21174,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21238,7 +21238,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21310,7 +21310,7 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
@@ -21378,7 +21378,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr"/>
@@ -21446,7 +21446,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21506,7 +21506,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21570,7 +21570,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
@@ -21634,7 +21634,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21702,7 +21702,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr"/>
@@ -21718,7 +21718,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>8e37468d116c824dadfd8db3939d434a3a65c746d65cc61b59a5c8e7346691c3</t>
+          <t>73f37e34ea183958d5a798bf611b845b2785a66be374a18f4fe96664912946cc</t>
         </is>
       </c>
     </row>
@@ -21770,14 +21770,14 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
+          <t>2026-10-20T12:58:58+00:00</t>
+        </is>
+      </c>
+      <c r="K366" s="2" t="inlineStr">
+        <is>
           <t>2026-10-19T14:54:11+00:00</t>
         </is>
       </c>
-      <c r="K366" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-19T14:54:11+00:00</t>
-        </is>
-      </c>
       <c r="L366" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21790,7 +21790,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>7867cb40d4e5f01bf3c9220210b561faef3093f68f67092f72126bba52001447</t>
+          <t>6f6dcd9ae87113ceff3fc43e747ba0e1be51a552b37e4540268e650849b93621</t>
         </is>
       </c>
     </row>
@@ -21842,7 +21842,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21914,7 +21914,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -21978,7 +21978,7 @@
       </c>
       <c r="J369" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K369" s="2" t="inlineStr"/>
@@ -22042,7 +22042,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22519,7 +22519,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22561,7 +22561,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22595,7 +22595,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22637,7 +22637,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22675,7 +22675,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22713,7 +22713,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22751,7 +22751,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22789,7 +22789,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22831,7 +22831,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22869,7 +22869,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22911,7 +22911,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22953,7 +22953,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -22995,7 +22995,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23079,7 +23079,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -23121,7 +23121,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23163,7 +23163,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23205,7 +23205,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23247,7 +23247,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23289,7 +23289,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23331,7 +23331,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23373,7 +23373,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23415,7 +23415,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23453,7 +23453,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23495,7 +23495,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23533,7 +23533,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23575,7 +23575,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23617,7 +23617,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23659,7 +23659,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23701,7 +23701,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -23743,7 +23743,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23781,7 +23781,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23819,7 +23819,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23857,7 +23857,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23899,7 +23899,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23941,7 +23941,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -23979,7 +23979,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24017,7 +24017,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24059,7 +24059,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24101,7 +24101,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24135,7 +24135,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24215,7 +24215,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24253,7 +24253,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24295,7 +24295,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24333,7 +24333,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24371,7 +24371,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24409,7 +24409,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24451,7 +24451,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24489,7 +24489,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24531,7 +24531,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24573,7 +24573,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24611,7 +24611,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24653,7 +24653,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24695,7 +24695,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24733,7 +24733,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24776,7 +24776,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -24809,7 +24809,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24851,7 +24851,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24889,7 +24889,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24931,7 +24931,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -24973,7 +24973,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -25011,7 +25011,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25053,7 +25053,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25095,7 +25095,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25133,7 +25133,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25175,7 +25175,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25213,7 +25213,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25255,7 +25255,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25297,7 +25297,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25339,7 +25339,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25377,7 +25377,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25415,7 +25415,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25453,7 +25453,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25491,7 +25491,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25529,7 +25529,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25571,7 +25571,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25609,7 +25609,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25647,7 +25647,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25689,7 +25689,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25727,7 +25727,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25769,7 +25769,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25807,7 +25807,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25849,7 +25849,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25925,7 +25925,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25967,7 +25967,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26389,7 +26389,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -26431,7 +26431,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26473,7 +26473,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26515,7 +26515,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26557,7 +26557,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26599,7 +26599,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26641,7 +26641,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26683,7 +26683,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26725,7 +26725,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26767,7 +26767,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26809,7 +26809,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26851,7 +26851,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26893,7 +26893,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26935,7 +26935,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -26977,7 +26977,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27019,7 +27019,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27061,7 +27061,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27103,7 +27103,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27145,7 +27145,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27187,7 +27187,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27229,7 +27229,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27271,7 +27271,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27313,7 +27313,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27355,7 +27355,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27397,7 +27397,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27439,7 +27439,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27481,12 +27481,12 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T12:17:25+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27565,7 +27565,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27607,7 +27607,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27649,7 +27649,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27691,7 +27691,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27733,7 +27733,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -27775,7 +27775,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27817,7 +27817,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27859,7 +27859,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27901,7 +27901,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27943,7 +27943,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -27981,7 +27981,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28023,7 +28023,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28065,7 +28065,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28107,7 +28107,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28149,7 +28149,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28191,7 +28191,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28233,7 +28233,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28275,7 +28275,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28317,7 +28317,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28359,7 +28359,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28401,7 +28401,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28443,7 +28443,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28485,7 +28485,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28527,7 +28527,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28569,7 +28569,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28611,7 +28611,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28653,7 +28653,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28695,7 +28695,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28779,7 +28779,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28821,7 +28821,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28863,12 +28863,12 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T12:17:25+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr">
@@ -28905,7 +28905,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28947,7 +28947,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -28989,7 +28989,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29031,7 +29031,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29073,7 +29073,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29115,7 +29115,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29157,7 +29157,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29199,7 +29199,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29241,7 +29241,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29283,7 +29283,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29325,7 +29325,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29367,7 +29367,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29409,7 +29409,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29451,7 +29451,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29493,7 +29493,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29577,7 +29577,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29619,7 +29619,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29661,7 +29661,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29703,7 +29703,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29745,7 +29745,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29787,7 +29787,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29829,7 +29829,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29871,7 +29871,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29913,7 +29913,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29955,7 +29955,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -29997,7 +29997,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30039,7 +30039,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30081,7 +30081,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30123,7 +30123,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30165,7 +30165,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30207,7 +30207,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30249,7 +30249,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30291,7 +30291,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30375,7 +30375,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30417,7 +30417,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30459,7 +30459,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30501,7 +30501,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30543,7 +30543,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30585,7 +30585,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30627,7 +30627,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30669,7 +30669,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30711,7 +30711,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30753,7 +30753,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30795,7 +30795,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30838,7 +30838,7 @@
       <c r="F205" s="2" t="inlineStr"/>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
@@ -30875,7 +30875,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30917,7 +30917,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -30959,7 +30959,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -31001,7 +31001,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31043,7 +31043,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31085,7 +31085,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31127,7 +31127,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31169,7 +31169,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31211,7 +31211,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31253,7 +31253,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31295,7 +31295,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31337,7 +31337,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31379,7 +31379,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31421,7 +31421,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31463,7 +31463,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31505,7 +31505,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31547,7 +31547,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31589,7 +31589,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31631,7 +31631,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31673,7 +31673,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31715,7 +31715,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31757,7 +31757,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31799,7 +31799,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31841,7 +31841,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31883,7 +31883,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31925,7 +31925,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31967,7 +31967,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -32009,7 +32009,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32051,7 +32051,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32093,7 +32093,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32135,7 +32135,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32177,7 +32177,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32219,7 +32219,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32261,7 +32261,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32303,7 +32303,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32345,7 +32345,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32387,7 +32387,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32429,7 +32429,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32467,7 +32467,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32509,7 +32509,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32547,7 +32547,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32581,7 +32581,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32623,7 +32623,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32661,7 +32661,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32703,7 +32703,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32745,7 +32745,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32783,7 +32783,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32821,7 +32821,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32859,7 +32859,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32897,7 +32897,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32939,7 +32939,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -32977,7 +32977,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -33011,7 +33011,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33049,7 +33049,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33087,7 +33087,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33125,7 +33125,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33167,7 +33167,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33209,7 +33209,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33247,7 +33247,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33289,7 +33289,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33323,7 +33323,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33361,7 +33361,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33404,7 +33404,7 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr">
@@ -33437,7 +33437,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-20T12:58:58+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-22 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6754,7 +6754,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8022,7 +8022,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8086,12 +8086,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>1e7e517d70270b5bddd175b23e97db617491ec202444860c846805f3c280aa8b</t>
+          <t>32c91fffe842015f02b777b5e77bf74e0165b4b315e3e5a9bfa3ffd3ffb9a7ec</t>
         </is>
       </c>
     </row>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8222,7 +8222,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8622,7 +8622,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8690,7 +8690,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="N153" s="2" t="inlineStr">
         <is>
-          <t>6719b2608fc54b0cd475a3bec8eddd667a0640a47d368c62655d2344e22e2a66</t>
+          <t>5cab8e3dfb94db05f3ad9ed1df3e4ddc7ae7073cbf100c264896a197ae26d3fc</t>
         </is>
       </c>
     </row>
@@ -8762,7 +8762,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8958,7 +8958,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10906,7 +10906,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10974,7 +10974,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -10994,7 +10994,7 @@
       </c>
       <c r="N192" s="2" t="inlineStr">
         <is>
-          <t>650a293414a2ed55794add852584991215842908be7f45aa94b52cc7616e798a</t>
+          <t>aaf27aac7cfbdfd186ccb80f279814b64890cc27087b3bd14d80bfa6640f06a7</t>
         </is>
       </c>
     </row>
@@ -11046,12 +11046,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>678fa3a417962c1490d96558cb2c34cfa41915fd5d9bfc931b6085acabe23015</t>
+          <t>606fdb60cac16a6c1cded6e25540b819a363a6dfc55f9313dbb0a6113666afb1</t>
         </is>
       </c>
     </row>
@@ -11118,12 +11118,12 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T13:09:42+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
@@ -11138,7 +11138,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>7ce8d871997e8f19eb309c3965901ec180067708f17a53d4231f183351d777fc</t>
+          <t>97cc418ac6e66ed80d489b22f843a6200de503f72b2c882d2480e4aba398d8c5</t>
         </is>
       </c>
     </row>
@@ -11190,12 +11190,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11210,7 +11210,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>b6969218dbd08eec51bd774815027f3f434418d5c5920a172b332cde8a9bd5b5</t>
+          <t>8b17a94cac8733531c1b485377425ed413cf9e66c7391bf7dbb4474d4ae5b49f</t>
         </is>
       </c>
     </row>
@@ -11262,12 +11262,12 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T12:34:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
@@ -11282,7 +11282,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>bdf3568cdc3ba102a5f566e30d8212ed74540600f72c5f313b3ecbc2fd5e7dfd</t>
+          <t>0745e4daffbfbea70f242d03537b22efa114a73278b46e548f09d223fbef3eac</t>
         </is>
       </c>
     </row>
@@ -11334,7 +11334,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11474,7 +11474,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11546,7 +11546,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11638,7 +11638,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>56094f2b4d126f65a87c1ecfaea43016bd44c932ad5273febaa3a31c97272732</t>
+          <t>39a5b5aec077f70883b6209af0e2f1382a8234a06b7bd7fe7ca93e263a5fa4dd</t>
         </is>
       </c>
     </row>
@@ -11690,7 +11690,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11758,7 +11758,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11830,12 +11830,12 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L204" s="2" t="inlineStr">
@@ -11850,7 +11850,7 @@
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>ffb5beb7f39ba9a938dc63c73cb119609bd6bfd8a80196d3adbbc32fa4fe2ffd</t>
+          <t>fa804089f86eb43c9cad3641daeaf381d2ac214945b35bfd926a5205f09a3a0c</t>
         </is>
       </c>
     </row>
@@ -11902,7 +11902,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12034,7 +12034,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12054,7 +12054,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>e96aa77982e88d1fa8e4974e36d2b784c94a6b97cf7f3edaf5d2778bddd01fca</t>
+          <t>abdcb5c9c9ba2fec3bbc78a104a53261117b2fc19cc2510708187da1cc60737f</t>
         </is>
       </c>
     </row>
@@ -12106,10 +12106,14 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
-        </is>
-      </c>
-      <c r="K208" s="2" t="inlineStr"/>
+          <t>2026-10-22T13:25:45+00:00</t>
+        </is>
+      </c>
+      <c r="K208" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22T13:25:45+00:00</t>
+        </is>
+      </c>
       <c r="L208" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -12122,7 +12126,7 @@
       </c>
       <c r="N208" s="2" t="inlineStr">
         <is>
-          <t>9c59401737e475f5593a4805dbaf3844fcd070e965b229f7c128ebf03ad82dd3</t>
+          <t>1d70967557a837a66f212cd331f62bdd93ea3b428e454f140771ce298ef05c4e</t>
         </is>
       </c>
     </row>
@@ -12174,7 +12178,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12246,7 +12250,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12542,7 +12546,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12790,7 +12794,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12862,7 +12866,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
@@ -12934,7 +12938,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13126,7 +13130,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
@@ -13198,7 +13202,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
@@ -13270,7 +13274,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13338,7 +13342,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13406,7 +13410,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13474,7 +13478,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13598,7 +13602,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13618,7 +13622,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>a55a21f9c39028df1294608bfa4eea59bcb8dbf9cd3fc8ac33b197e038e27e34</t>
+          <t>48e81c8b31547c08652044290e37ba96ce52798aff926af59882658059ac2b6b</t>
         </is>
       </c>
     </row>
@@ -13910,14 +13914,14 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
+          <t>2026-10-22T13:25:45+00:00</t>
+        </is>
+      </c>
+      <c r="K236" s="2" t="inlineStr">
+        <is>
           <t>2026-10-21T13:15:03+00:00</t>
         </is>
       </c>
-      <c r="K236" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21T13:15:03+00:00</t>
-        </is>
-      </c>
       <c r="L236" s="2" t="inlineStr">
         <is>
           <t>2026-09-30</t>
@@ -13930,7 +13934,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>51866836cebde3b9710b3b0e1542f571623bf049d29182ed9cd7a83425e3832d</t>
+          <t>fbd52d099b3cd790415c9b4b7102254ae76bb6fcea716a16a3a9dd19071c2ba7</t>
         </is>
       </c>
     </row>
@@ -18182,7 +18186,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18202,7 +18206,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>0d0903557b20b250d77fe4717ab0e84fd0e6cf11f2c019013fb01d38eac5720f</t>
+          <t>61b3451cf0944575a0f283ac95411d2886f36165ee8db5aec2cf7cbcece34bb1</t>
         </is>
       </c>
     </row>
@@ -18254,7 +18258,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
@@ -18274,7 +18278,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>6d6629ee0e598e5cf89761e971051949a67c9e56f1edfec8ef5838dcae414484</t>
+          <t>eb0bbfe1326d748771c56f0397f6f79908a2fc93ad234373ec44e093e8137d59</t>
         </is>
       </c>
     </row>
@@ -18326,7 +18330,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18398,7 +18402,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18466,7 +18470,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18534,7 +18538,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18658,7 +18662,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19086,7 +19090,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19154,7 +19158,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19222,7 +19226,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19290,12 +19294,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20T12:58:58+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19310,7 +19314,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>fae55bbd39ec8cbf47e12077e497b8a01701201163792fbd886e08e69f7a1a7a</t>
+          <t>31a99f62f577fd37d8675ff24deff89405f348981be108f08fa420cf61ebd3a3</t>
         </is>
       </c>
     </row>
@@ -19362,12 +19366,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19382,7 +19386,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>569dd1edb7ab1faa9708834515375bc5b8da5074426d349e10fb28cd3e6641c9</t>
+          <t>74e761b05d4d32ef2ab79856933b74d99604d49b18c3e555c050ac5dcebc91bf</t>
         </is>
       </c>
     </row>
@@ -19434,12 +19438,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19454,7 +19458,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>e7edc7c9339c53d352023c900164853c0cb31aa67547a430c685e2597b0ee2cb</t>
+          <t>9b14b6d7c91e6951de1b04953515ea703bfa46036a739b3f0d7f91dc3d78a667</t>
         </is>
       </c>
     </row>
@@ -19506,7 +19510,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr">
@@ -19634,7 +19638,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19702,7 +19706,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19770,7 +19774,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19838,10 +19842,14 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
-        </is>
-      </c>
-      <c r="K337" s="2" t="inlineStr"/>
+          <t>2026-10-22T13:25:45+00:00</t>
+        </is>
+      </c>
+      <c r="K337" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22T13:25:45+00:00</t>
+        </is>
+      </c>
       <c r="L337" s="2" t="inlineStr">
         <is>
           <t>2026-10-08</t>
@@ -19854,7 +19862,7 @@
       </c>
       <c r="N337" s="2" t="inlineStr">
         <is>
-          <t>b974bde6fb9765f483d9acb34135a5d37f925aecea5037ec34a676b0394c30e9</t>
+          <t>43a402336a674da1b0b03d2040f92387ba0b1845d1c5c991801d8c0d99f9b67f</t>
         </is>
       </c>
     </row>
@@ -19906,7 +19914,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
@@ -19978,7 +19986,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20046,7 +20054,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20114,7 +20122,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20182,12 +20190,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20202,7 +20210,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>3c68283a3da26c6cc101f0becacea281fe15bb350fbdf775299eca99fee9934a</t>
+          <t>d2403213656194381b8d22f87479f257fedf7ccc3be4ad95b779083ddb029f56</t>
         </is>
       </c>
     </row>
@@ -20370,7 +20378,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
@@ -20442,7 +20450,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20510,7 +20518,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20578,7 +20586,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20646,7 +20654,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20714,7 +20722,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20782,7 +20790,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20850,7 +20858,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20918,7 +20926,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20986,7 +20994,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21050,7 +21058,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21110,7 +21118,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21182,7 +21190,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21246,7 +21254,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21318,12 +21326,12 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
@@ -21338,7 +21346,7 @@
       </c>
       <c r="N359" s="2" t="inlineStr">
         <is>
-          <t>d080f4d6171318a1aca6606148bd9bda1b93193acf09291580d3911f802f28e0</t>
+          <t>2884670e5278e822c4691b7c615ee6c2a6f63cc37ba806197ddff393bdf4c62a</t>
         </is>
       </c>
     </row>
@@ -21386,7 +21394,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr">
@@ -21458,7 +21466,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21518,7 +21526,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21582,7 +21590,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
@@ -21646,7 +21654,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21714,7 +21722,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr"/>
@@ -21782,12 +21790,12 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="L366" s="2" t="inlineStr">
@@ -21802,7 +21810,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>784fd73dcc7f768128f6874551020a4f1c2428e1e4b0188edae280e6e120daff</t>
+          <t>a08dc649dbd54a5c3ee0eecbbd3f9b3e42d81390920f507a74587eb4f25fad8c</t>
         </is>
       </c>
     </row>
@@ -21854,7 +21862,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21926,7 +21934,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -22054,7 +22062,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22531,7 +22539,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22573,7 +22581,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22607,7 +22615,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22649,7 +22657,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22687,7 +22695,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22725,7 +22733,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22763,7 +22771,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22801,7 +22809,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22839,7 +22847,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22881,7 +22889,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22919,7 +22927,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22961,7 +22969,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -23003,7 +23011,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23045,7 +23053,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23092,7 +23100,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -23129,7 +23137,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23171,7 +23179,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23213,7 +23221,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23255,7 +23263,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23297,7 +23305,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23339,7 +23347,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23381,7 +23389,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23423,7 +23431,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23465,7 +23473,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23503,7 +23511,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23545,7 +23553,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23583,7 +23591,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23625,7 +23633,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23667,7 +23675,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23709,7 +23717,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -23751,7 +23759,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23793,7 +23801,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23831,7 +23839,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23869,7 +23877,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23907,7 +23915,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23949,7 +23957,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -23991,7 +23999,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24029,7 +24037,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24067,7 +24075,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24109,7 +24117,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24151,7 +24159,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24185,7 +24193,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24227,7 +24235,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24265,7 +24273,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24303,7 +24311,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24345,7 +24353,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24383,7 +24391,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24421,7 +24429,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24459,7 +24467,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24501,7 +24509,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24539,7 +24547,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24581,7 +24589,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24623,7 +24631,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24661,7 +24669,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24703,7 +24711,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24745,7 +24753,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24783,7 +24791,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24821,7 +24829,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24863,7 +24871,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24901,7 +24909,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24943,7 +24951,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -24985,7 +24993,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -25023,7 +25031,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25065,7 +25073,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25107,7 +25115,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25145,7 +25153,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25187,7 +25195,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25225,7 +25233,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25267,7 +25275,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25309,7 +25317,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25351,7 +25359,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25389,7 +25397,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25427,7 +25435,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25465,7 +25473,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25503,7 +25511,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25541,7 +25549,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25583,7 +25591,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25621,7 +25629,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25659,7 +25667,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25701,7 +25709,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25739,7 +25747,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25781,7 +25789,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25819,7 +25827,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25861,7 +25869,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25899,7 +25907,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25937,7 +25945,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25979,7 +25987,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26439,7 +26447,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26481,7 +26489,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26523,7 +26531,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26565,7 +26573,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26607,7 +26615,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26649,7 +26657,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26691,7 +26699,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26733,7 +26741,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26775,7 +26783,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26817,7 +26825,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26859,7 +26867,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26901,7 +26909,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26943,7 +26951,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -26985,7 +26993,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27027,7 +27035,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27069,7 +27077,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27111,7 +27119,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27153,7 +27161,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27195,7 +27203,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27237,7 +27245,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27279,7 +27287,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27321,7 +27329,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27363,7 +27371,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27405,7 +27413,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27447,7 +27455,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27489,7 +27497,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27531,7 +27539,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27573,7 +27581,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27615,7 +27623,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27657,7 +27665,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27699,7 +27707,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27746,7 +27754,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -27783,7 +27791,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27825,7 +27833,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27867,7 +27875,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27909,7 +27917,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27951,7 +27959,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -27993,7 +28001,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28031,7 +28039,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28073,7 +28081,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28115,7 +28123,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28157,7 +28165,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28199,7 +28207,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28241,7 +28249,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28283,7 +28291,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28325,7 +28333,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28367,7 +28375,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28409,7 +28417,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28451,7 +28459,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28493,7 +28501,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28535,7 +28543,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28577,7 +28585,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28619,7 +28627,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28661,7 +28669,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28703,7 +28711,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28745,7 +28753,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28787,7 +28795,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28829,7 +28837,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28871,7 +28879,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28913,7 +28921,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28955,7 +28963,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -28997,7 +29005,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29039,7 +29047,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29081,7 +29089,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29123,7 +29131,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29165,7 +29173,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29207,7 +29215,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29249,7 +29257,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29291,7 +29299,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29333,7 +29341,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29375,7 +29383,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29417,7 +29425,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29459,7 +29467,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29501,7 +29509,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29543,7 +29551,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29585,7 +29593,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29627,7 +29635,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29669,7 +29677,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29711,7 +29719,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29753,7 +29761,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29795,7 +29803,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29837,7 +29845,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29879,7 +29887,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29921,7 +29929,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29963,7 +29971,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -30005,7 +30013,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30047,7 +30055,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30089,7 +30097,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30131,7 +30139,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30173,7 +30181,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30215,7 +30223,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30257,7 +30265,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30299,7 +30307,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30341,7 +30349,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30383,7 +30391,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30425,7 +30433,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30467,7 +30475,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30509,7 +30517,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30551,7 +30559,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30593,7 +30601,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30635,7 +30643,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30677,7 +30685,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30719,7 +30727,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30761,7 +30769,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30803,7 +30811,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30845,7 +30853,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -30887,7 +30895,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30929,7 +30937,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -30971,7 +30979,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -31013,7 +31021,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31055,7 +31063,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31097,7 +31105,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31139,7 +31147,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31181,7 +31189,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31223,7 +31231,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31265,7 +31273,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31307,7 +31315,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31349,7 +31357,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31391,7 +31399,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31433,7 +31441,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31475,7 +31483,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31517,7 +31525,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31559,7 +31567,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31601,7 +31609,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31643,7 +31651,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31685,7 +31693,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31727,7 +31735,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31769,7 +31777,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31811,7 +31819,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31853,7 +31861,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31895,7 +31903,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31937,7 +31945,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31979,7 +31987,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -32021,12 +32029,12 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20T12:58:58+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H233" s="2" t="inlineStr">
@@ -32063,7 +32071,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32105,7 +32113,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32147,7 +32155,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32189,7 +32197,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32231,7 +32239,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32273,7 +32281,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32315,7 +32323,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32357,7 +32365,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32399,7 +32407,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32441,7 +32449,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32483,7 +32491,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32525,7 +32533,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32563,7 +32571,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32605,7 +32613,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32643,7 +32651,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32677,7 +32685,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32719,7 +32727,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32757,7 +32765,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32799,7 +32807,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32841,7 +32849,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32879,7 +32887,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32917,7 +32925,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32955,7 +32963,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -32993,7 +33001,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -33035,7 +33043,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33073,7 +33081,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33107,7 +33115,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33145,7 +33153,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33183,7 +33191,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33221,7 +33229,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33263,7 +33271,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33305,7 +33313,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33343,7 +33351,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33385,7 +33393,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33419,7 +33427,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33457,7 +33465,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">
@@ -33495,7 +33503,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -33533,7 +33541,7 @@
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-23 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6754,7 +6754,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8022,7 +8022,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8086,12 +8086,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>32c91fffe842015f02b777b5e77bf74e0165b4b315e3e5a9bfa3ffd3ffb9a7ec</t>
+          <t>57b89c49671a2ce829c4dbc8b11f30a5e93dce0a13f77011c8feeea62ad34844</t>
         </is>
       </c>
     </row>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8222,7 +8222,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8622,7 +8622,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8690,7 +8690,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8762,7 +8762,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8958,7 +8958,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10906,7 +10906,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10974,7 +10974,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11046,12 +11046,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>606fdb60cac16a6c1cded6e25540b819a363a6dfc55f9313dbb0a6113666afb1</t>
+          <t>be15e1f5cfc9f24e1246c302cbd1ca38e3ab4f1ae98780f4f8d51a625b272e4a</t>
         </is>
       </c>
     </row>
@@ -11118,14 +11118,14 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
+          <t>2026-10-23T12:52:38+00:00</t>
+        </is>
+      </c>
+      <c r="K194" s="2" t="inlineStr">
+        <is>
           <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
-      <c r="K194" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-22T13:25:45+00:00</t>
-        </is>
-      </c>
       <c r="L194" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11138,7 +11138,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>97cc418ac6e66ed80d489b22f843a6200de503f72b2c882d2480e4aba398d8c5</t>
+          <t>d61d4d289a2bf8129a529403eb6435c09ac7ad1141cce1b809d6ecee90342f05</t>
         </is>
       </c>
     </row>
@@ -11190,12 +11190,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11210,7 +11210,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>8b17a94cac8733531c1b485377425ed413cf9e66c7391bf7dbb4474d4ae5b49f</t>
+          <t>ed5b9f6224e5d4204e5a5738faad9ac2214f210f1a6cac5d868b1a3177fc2a5c</t>
         </is>
       </c>
     </row>
@@ -11262,14 +11262,14 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
+          <t>2026-10-23T12:52:38+00:00</t>
+        </is>
+      </c>
+      <c r="K196" s="2" t="inlineStr">
+        <is>
           <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
-      <c r="K196" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-22T13:25:45+00:00</t>
-        </is>
-      </c>
       <c r="L196" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11282,7 +11282,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>0745e4daffbfbea70f242d03537b22efa114a73278b46e548f09d223fbef3eac</t>
+          <t>b553791e02752225773f1c294acddab7050f94ba36bf73a3f15c1d714e5a7f9b</t>
         </is>
       </c>
     </row>
@@ -11334,7 +11334,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11474,7 +11474,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11546,7 +11546,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11690,7 +11690,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11758,7 +11758,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11902,7 +11902,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12034,7 +12034,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12054,7 +12054,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>abdcb5c9c9ba2fec3bbc78a104a53261117b2fc19cc2510708187da1cc60737f</t>
+          <t>06087b9e6a42cd27c16a90c9604b634af5ed9e643e26c0d5a61830976615ff5d</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr">
@@ -12178,7 +12178,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12198,7 +12198,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
+          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
         </is>
       </c>
     </row>
@@ -12250,7 +12250,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12546,7 +12546,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12794,7 +12794,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12866,7 +12866,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
@@ -12938,7 +12938,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13130,7 +13130,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
@@ -13202,7 +13202,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
@@ -13274,7 +13274,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13342,7 +13342,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13410,7 +13410,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13478,7 +13478,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13602,7 +13602,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13622,7 +13622,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>48e81c8b31547c08652044290e37ba96ce52798aff926af59882658059ac2b6b</t>
+          <t>a55a21f9c39028df1294608bfa4eea59bcb8dbf9cd3fc8ac33b197e038e27e34</t>
         </is>
       </c>
     </row>
@@ -13914,12 +13914,12 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
@@ -13934,7 +13934,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>fbd52d099b3cd790415c9b4b7102254ae76bb6fcea716a16a3a9dd19071c2ba7</t>
+          <t>a1aa4e325d8bc7f9546ee74bebf0487d2135b8cebe621e74adcd7ed4ef5feb1c</t>
         </is>
       </c>
     </row>
@@ -18186,7 +18186,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18206,7 +18206,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>61b3451cf0944575a0f283ac95411d2886f36165ee8db5aec2cf7cbcece34bb1</t>
+          <t>0d0903557b20b250d77fe4717ab0e84fd0e6cf11f2c019013fb01d38eac5720f</t>
         </is>
       </c>
     </row>
@@ -18258,7 +18258,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
@@ -18278,7 +18278,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>eb0bbfe1326d748771c56f0397f6f79908a2fc93ad234373ec44e093e8137d59</t>
+          <t>fbdf7a1a38ed2d4c7e55ec16da3f1bba2443a7969aa9329596156bd52dbcafa9</t>
         </is>
       </c>
     </row>
@@ -18330,7 +18330,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18402,7 +18402,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18470,7 +18470,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18538,7 +18538,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18662,7 +18662,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19090,7 +19090,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19158,7 +19158,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19226,7 +19226,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19294,12 +19294,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19314,7 +19314,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>31a99f62f577fd37d8675ff24deff89405f348981be108f08fa420cf61ebd3a3</t>
+          <t>5b3134f43838a6ee8134a5a6291eb9617eda5d31364621aab4134995e02457ca</t>
         </is>
       </c>
     </row>
@@ -19366,12 +19366,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19386,7 +19386,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>74e761b05d4d32ef2ab79856933b74d99604d49b18c3e555c050ac5dcebc91bf</t>
+          <t>86c6ac629625df931b9beefd066e0c068212b6d0c714993cfc54e72b4077bb02</t>
         </is>
       </c>
     </row>
@@ -19438,12 +19438,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19458,7 +19458,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>9b14b6d7c91e6951de1b04953515ea703bfa46036a739b3f0d7f91dc3d78a667</t>
+          <t>3282a077a568b7f6859042eb5afbc18597e3d765164d6f5631f12b9f34e1b3d3</t>
         </is>
       </c>
     </row>
@@ -19510,7 +19510,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr">
@@ -19638,7 +19638,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19706,7 +19706,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19774,7 +19774,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19842,7 +19842,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr">
@@ -19914,7 +19914,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
@@ -19986,7 +19986,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20054,7 +20054,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20122,7 +20122,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20190,12 +20190,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20210,7 +20210,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>d2403213656194381b8d22f87479f257fedf7ccc3be4ad95b779083ddb029f56</t>
+          <t>19796330dfaa06ef399b962b7b0f6518be460d6f6b4583cfde852e24797c2dec</t>
         </is>
       </c>
     </row>
@@ -20378,12 +20378,12 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20T12:58:58+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="L345" s="2" t="inlineStr">
@@ -20398,7 +20398,7 @@
       </c>
       <c r="N345" s="2" t="inlineStr">
         <is>
-          <t>09e3d13d618416b17d293449518960b6a61d3ad9c936275336619d5a8cad8155</t>
+          <t>0ade81f7cf9df5160b9edeaf93a43b052617c8d79e7779605e831d7d41641d1b</t>
         </is>
       </c>
     </row>
@@ -20450,7 +20450,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20518,7 +20518,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20586,7 +20586,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20654,7 +20654,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20722,7 +20722,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20790,7 +20790,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20858,7 +20858,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20926,7 +20926,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20994,7 +20994,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21058,7 +21058,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21118,7 +21118,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21190,7 +21190,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21254,7 +21254,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21326,7 +21326,7 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
@@ -21394,7 +21394,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr">
@@ -21466,7 +21466,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21526,7 +21526,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21590,7 +21590,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21722,10 +21722,14 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
-        </is>
-      </c>
-      <c r="K365" s="2" t="inlineStr"/>
+          <t>2026-10-23T12:52:38+00:00</t>
+        </is>
+      </c>
+      <c r="K365" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23T12:52:38+00:00</t>
+        </is>
+      </c>
       <c r="L365" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21738,7 +21742,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>655094256611121fa61e4899483a1255a5cb9903a99f0f3daa3f82c8b09a55a8</t>
+          <t>b27af5a22c6503e997c6f24c9adc93b672125a489e8b9dfebd2205174c291510</t>
         </is>
       </c>
     </row>
@@ -21790,14 +21794,14 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
+          <t>2026-10-23T12:52:38+00:00</t>
+        </is>
+      </c>
+      <c r="K366" s="2" t="inlineStr">
+        <is>
           <t>2026-10-22T13:25:45+00:00</t>
         </is>
       </c>
-      <c r="K366" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-22T13:25:45+00:00</t>
-        </is>
-      </c>
       <c r="L366" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21810,7 +21814,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>a08dc649dbd54a5c3ee0eecbbd3f9b3e42d81390920f507a74587eb4f25fad8c</t>
+          <t>1348e9dec6987cdd4515da0e710a7caf1c9f95fc9261ebdb83f58050130b6642</t>
         </is>
       </c>
     </row>
@@ -21862,7 +21866,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21934,7 +21938,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -22062,7 +22066,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22539,7 +22543,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22581,7 +22585,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22615,7 +22619,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22657,7 +22661,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22695,7 +22699,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22733,7 +22737,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22771,7 +22775,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22809,7 +22813,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22847,7 +22851,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22889,7 +22893,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22927,7 +22931,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22969,7 +22973,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -23011,7 +23015,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23053,7 +23057,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23100,7 +23104,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -23137,7 +23141,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23179,7 +23183,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23221,7 +23225,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23263,7 +23267,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23305,7 +23309,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23347,7 +23351,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23389,7 +23393,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23431,7 +23435,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23473,7 +23477,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23511,7 +23515,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23553,7 +23557,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23591,7 +23595,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23633,7 +23637,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23675,7 +23679,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23717,7 +23721,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -23759,7 +23763,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23801,7 +23805,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23839,7 +23843,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23877,7 +23881,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23915,7 +23919,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23957,7 +23961,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -23999,7 +24003,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24037,7 +24041,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24075,7 +24079,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24117,7 +24121,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24159,7 +24163,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24193,7 +24197,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24235,7 +24239,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24273,7 +24277,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24311,7 +24315,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24353,7 +24357,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24391,7 +24395,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24429,7 +24433,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24467,7 +24471,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24509,7 +24513,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24547,7 +24551,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24589,7 +24593,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24631,7 +24635,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24669,7 +24673,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24711,7 +24715,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24753,7 +24757,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24791,7 +24795,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24829,7 +24833,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24871,7 +24875,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24909,7 +24913,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24951,7 +24955,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -24993,7 +24997,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -25031,7 +25035,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25073,7 +25077,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25115,7 +25119,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25153,7 +25157,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25195,7 +25199,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25233,7 +25237,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25275,7 +25279,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25317,7 +25321,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25359,7 +25363,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25397,7 +25401,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25435,7 +25439,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25473,7 +25477,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25511,7 +25515,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25549,7 +25553,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25591,7 +25595,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25629,7 +25633,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25667,7 +25671,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25709,7 +25713,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25747,7 +25751,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25789,7 +25793,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25827,7 +25831,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25869,7 +25873,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25907,7 +25911,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25945,7 +25949,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25987,7 +25991,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26447,7 +26451,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26489,7 +26493,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26531,7 +26535,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26573,7 +26577,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26615,7 +26619,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26657,7 +26661,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26699,7 +26703,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26741,7 +26745,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26783,7 +26787,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26825,7 +26829,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26867,7 +26871,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26909,7 +26913,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26951,7 +26955,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -26993,7 +26997,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27035,7 +27039,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27077,7 +27081,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27119,7 +27123,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27161,7 +27165,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27203,7 +27207,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27245,7 +27249,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27287,7 +27291,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27329,7 +27333,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27371,7 +27375,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27413,7 +27417,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27455,7 +27459,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27497,7 +27501,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27544,7 +27548,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -27581,7 +27585,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27623,7 +27627,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27665,7 +27669,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27707,7 +27711,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27754,7 +27758,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -27791,7 +27795,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27833,7 +27837,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27875,7 +27879,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27917,7 +27921,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27959,7 +27963,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -28001,7 +28005,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28039,7 +28043,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28081,7 +28085,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28123,7 +28127,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28165,7 +28169,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28207,7 +28211,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28249,7 +28253,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28291,7 +28295,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28333,7 +28337,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28375,7 +28379,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28417,7 +28421,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28459,7 +28463,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28501,7 +28505,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28543,7 +28547,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28585,7 +28589,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28627,7 +28631,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28669,7 +28673,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28711,7 +28715,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28753,7 +28757,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28795,7 +28799,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28837,7 +28841,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28879,7 +28883,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28921,7 +28925,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28963,7 +28967,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -29005,7 +29009,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29047,7 +29051,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29089,7 +29093,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29131,7 +29135,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29173,7 +29177,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29215,7 +29219,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29257,7 +29261,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29299,7 +29303,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29341,7 +29345,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29383,7 +29387,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29425,7 +29429,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29467,7 +29471,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29509,7 +29513,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29551,7 +29555,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29593,7 +29597,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29635,7 +29639,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29677,7 +29681,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29719,7 +29723,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29761,7 +29765,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29803,7 +29807,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29845,7 +29849,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29887,7 +29891,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29929,7 +29933,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29971,7 +29975,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -30013,7 +30017,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30055,7 +30059,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30097,7 +30101,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30139,7 +30143,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30181,7 +30185,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30223,7 +30227,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30265,7 +30269,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30307,7 +30311,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30349,7 +30353,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30391,7 +30395,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30433,7 +30437,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30475,7 +30479,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30517,7 +30521,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30559,7 +30563,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30601,7 +30605,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30643,7 +30647,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30685,7 +30689,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30727,7 +30731,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30769,7 +30773,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30811,7 +30815,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30853,7 +30857,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -30895,7 +30899,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30942,7 +30946,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
@@ -30979,7 +30983,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -31021,7 +31025,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31063,7 +31067,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31110,7 +31114,7 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr">
@@ -31147,7 +31151,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31189,7 +31193,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31231,7 +31235,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31273,7 +31277,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31315,7 +31319,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31357,7 +31361,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31399,7 +31403,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31441,7 +31445,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31483,7 +31487,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31525,7 +31529,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31567,7 +31571,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31609,7 +31613,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31651,7 +31655,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31693,7 +31697,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31735,7 +31739,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31777,7 +31781,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31819,7 +31823,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31861,7 +31865,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31903,7 +31907,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31945,7 +31949,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31987,7 +31991,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -32029,7 +32033,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32071,7 +32075,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32113,7 +32117,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32155,7 +32159,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32197,7 +32201,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32239,7 +32243,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32281,7 +32285,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32323,7 +32327,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32365,7 +32369,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32407,7 +32411,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32449,7 +32453,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32491,7 +32495,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32533,7 +32537,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32571,7 +32575,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32613,7 +32617,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32651,7 +32655,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32685,7 +32689,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32727,7 +32731,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32765,7 +32769,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32807,7 +32811,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32849,7 +32853,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32887,7 +32891,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32925,7 +32929,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32963,7 +32967,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -33001,7 +33005,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -33043,7 +33047,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33081,7 +33085,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33115,7 +33119,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33153,7 +33157,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33191,7 +33195,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33229,7 +33233,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33271,7 +33275,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33313,7 +33317,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33351,7 +33355,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33393,7 +33397,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33427,7 +33431,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33465,7 +33469,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">
@@ -33503,7 +33507,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -33541,7 +33545,7 @@
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-24 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6754,7 +6754,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8022,7 +8022,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8086,12 +8086,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>57b89c49671a2ce829c4dbc8b11f30a5e93dce0a13f77011c8feeea62ad34844</t>
+          <t>ec16154b2e6cb0039685099ba4e443616a578f95791b0d5c48d16015fbc6c010</t>
         </is>
       </c>
     </row>
@@ -8154,12 +8154,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8170,7 +8170,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>e0ae215df5264afe3e67f2d2d004ff694231af627c2f5df8d4b4ba445505c477</t>
+          <t>fd60184c7dfc9872b33b3e0997ba1ca80028c23b93cbfd2be5dc10a450ab1564</t>
         </is>
       </c>
     </row>
@@ -8222,7 +8222,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8622,7 +8622,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8690,7 +8690,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8762,7 +8762,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8958,7 +8958,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10906,7 +10906,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10974,7 +10974,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11046,12 +11046,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>be15e1f5cfc9f24e1246c302cbd1ca38e3ab4f1ae98780f4f8d51a625b272e4a</t>
+          <t>07d867fd269caf9e144b0cba858438e669c2cc75144b79eea23d23004533efc7</t>
         </is>
       </c>
     </row>
@@ -11118,7 +11118,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11190,14 +11190,14 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
+          <t>2026-10-24T12:15:32+00:00</t>
+        </is>
+      </c>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
           <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
-      <c r="K195" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-23T12:52:38+00:00</t>
-        </is>
-      </c>
       <c r="L195" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11210,7 +11210,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>ed5b9f6224e5d4204e5a5738faad9ac2214f210f1a6cac5d868b1a3177fc2a5c</t>
+          <t>3184c99249877695e5c89421a1d59ab1f51f04c6ee87a489401c8d4f62ed7ef3</t>
         </is>
       </c>
     </row>
@@ -11262,12 +11262,12 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
@@ -11282,7 +11282,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>b553791e02752225773f1c294acddab7050f94ba36bf73a3f15c1d714e5a7f9b</t>
+          <t>eb789638a5ee15f92f6fe638b324161691782dbe1373f2359585f1bc229cd874</t>
         </is>
       </c>
     </row>
@@ -11334,7 +11334,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11474,7 +11474,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11546,7 +11546,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11690,7 +11690,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11758,7 +11758,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11902,7 +11902,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12029,17 +12029,17 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>open</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-11T14:09:30+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -12054,7 +12054,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>06087b9e6a42cd27c16a90c9604b634af5ed9e643e26c0d5a61830976615ff5d</t>
+          <t>bf359ee82e724c180760278da6a06d5eab8aff10089ae2bee940fd935c706882</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr">
@@ -12178,12 +12178,12 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17T11:48:17+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
@@ -12198,7 +12198,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
+          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
         </is>
       </c>
     </row>
@@ -12250,7 +12250,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12546,10 +12546,14 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
-        </is>
-      </c>
-      <c r="K215" s="2" t="inlineStr"/>
+          <t>2026-10-24T12:15:32+00:00</t>
+        </is>
+      </c>
+      <c r="K215" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24T12:15:32+00:00</t>
+        </is>
+      </c>
       <c r="L215" s="2" t="inlineStr">
         <is>
           <t>2026-09-30</t>
@@ -12562,7 +12566,7 @@
       </c>
       <c r="N215" s="2" t="inlineStr">
         <is>
-          <t>ed6a8a02b232ac5df3e78f4adc828102781b429393e70e9539a73a394f26641f</t>
+          <t>7cba76456716917480833e5ffec9e9202882506d699a87d84abb4c2094d215ea</t>
         </is>
       </c>
     </row>
@@ -12794,12 +12798,12 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L219" s="2" t="inlineStr">
@@ -12814,7 +12818,7 @@
       </c>
       <c r="N219" s="2" t="inlineStr">
         <is>
-          <t>7d213556641924980cf256ce1311f268027b171bf8a2169f1823bfa973743e3b</t>
+          <t>69f9c26880d5f8d0d9d65bf21f2fac5d8bf45ad1bba065052bd69f75d55fe107</t>
         </is>
       </c>
     </row>
@@ -12866,7 +12870,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
@@ -12938,7 +12942,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13130,7 +13134,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
@@ -13202,7 +13206,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
@@ -13274,7 +13278,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13342,7 +13346,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13410,7 +13414,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13478,7 +13482,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13602,7 +13606,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13914,12 +13918,12 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
@@ -13934,7 +13938,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>a1aa4e325d8bc7f9546ee74bebf0487d2135b8cebe621e74adcd7ed4ef5feb1c</t>
+          <t>2224b6300fb7a2f065abeb558f42bcf0f9e1396d514ce4ce25e7647ebf6b593b</t>
         </is>
       </c>
     </row>
@@ -18186,7 +18190,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18206,7 +18210,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>0d0903557b20b250d77fe4717ab0e84fd0e6cf11f2c019013fb01d38eac5720f</t>
+          <t>61b3451cf0944575a0f283ac95411d2886f36165ee8db5aec2cf7cbcece34bb1</t>
         </is>
       </c>
     </row>
@@ -18258,7 +18262,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
@@ -18278,7 +18282,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>fbdf7a1a38ed2d4c7e55ec16da3f1bba2443a7969aa9329596156bd52dbcafa9</t>
+          <t>47778e395446938a5eff70c74fcd71217761cffaf69109c6a3fda3b66b7508c6</t>
         </is>
       </c>
     </row>
@@ -18330,7 +18334,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18402,7 +18406,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18470,7 +18474,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18538,7 +18542,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18662,7 +18666,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19090,7 +19094,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19158,7 +19162,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19226,7 +19230,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19294,12 +19298,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19314,7 +19318,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>5b3134f43838a6ee8134a5a6291eb9617eda5d31364621aab4134995e02457ca</t>
+          <t>b0ef731f7675309ac4a16be433d63a7138d98382431aa0d8acfc9c8f9f236849</t>
         </is>
       </c>
     </row>
@@ -19366,12 +19370,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19386,7 +19390,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>86c6ac629625df931b9beefd066e0c068212b6d0c714993cfc54e72b4077bb02</t>
+          <t>1d3e04e652eea2e4962588e50ee2a7e70ebef21b069f561cf63b9587abd82c99</t>
         </is>
       </c>
     </row>
@@ -19438,12 +19442,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19458,7 +19462,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>3282a077a568b7f6859042eb5afbc18597e3d765164d6f5631f12b9f34e1b3d3</t>
+          <t>ecc2726efe9c8a66438b8d01ae204f4b39cc5e65e2a2855bd2ba929c7f6eadb9</t>
         </is>
       </c>
     </row>
@@ -19510,7 +19514,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr">
@@ -19638,7 +19642,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19706,7 +19710,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19774,7 +19778,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19842,7 +19846,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr">
@@ -19914,7 +19918,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
@@ -19986,7 +19990,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20054,7 +20058,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20122,7 +20126,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20190,12 +20194,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20210,7 +20214,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>19796330dfaa06ef399b962b7b0f6518be460d6f6b4583cfde852e24797c2dec</t>
+          <t>0f386bd079120e1ec47a52702a962fb0230f0908b2e799e06332779392bd3a01</t>
         </is>
       </c>
     </row>
@@ -20378,7 +20382,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
@@ -20450,7 +20454,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20518,7 +20522,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20586,7 +20590,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20654,7 +20658,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20722,7 +20726,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20790,7 +20794,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20858,7 +20862,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20926,7 +20930,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20994,7 +20998,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21058,7 +21062,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21118,7 +21122,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21190,7 +21194,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21254,7 +21258,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21326,12 +21330,12 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
@@ -21346,7 +21350,7 @@
       </c>
       <c r="N359" s="2" t="inlineStr">
         <is>
-          <t>2884670e5278e822c4691b7c615ee6c2a6f63cc37ba806197ddff393bdf4c62a</t>
+          <t>428a7891f756a20e4159359161eecf2ac68bad8ae48bc49e274c4afe0816c36a</t>
         </is>
       </c>
     </row>
@@ -21394,7 +21398,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr">
@@ -21466,7 +21470,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21526,7 +21530,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21590,7 +21594,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
@@ -21654,7 +21658,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21722,14 +21726,14 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
+          <t>2026-10-24T12:15:32+00:00</t>
+        </is>
+      </c>
+      <c r="K365" s="2" t="inlineStr">
+        <is>
           <t>2026-10-23T12:52:38+00:00</t>
         </is>
       </c>
-      <c r="K365" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-23T12:52:38+00:00</t>
-        </is>
-      </c>
       <c r="L365" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21742,7 +21746,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>b27af5a22c6503e997c6f24c9adc93b672125a489e8b9dfebd2205174c291510</t>
+          <t>45a79498aa39c0931a47d6ea55f86a7e5693cb49d5a537299ab5bf6be2143c8a</t>
         </is>
       </c>
     </row>
@@ -21794,7 +21798,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr">
@@ -21814,7 +21818,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>1348e9dec6987cdd4515da0e710a7caf1c9f95fc9261ebdb83f58050130b6642</t>
+          <t>1e2c3d4268188d017728f0c4000325fe1522d472f3b6d3b8b3eb37efc6c6f267</t>
         </is>
       </c>
     </row>
@@ -21866,7 +21870,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21938,7 +21942,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -22066,7 +22070,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22543,7 +22547,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22585,7 +22589,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22619,7 +22623,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22661,7 +22665,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22699,7 +22703,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22737,7 +22741,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22775,7 +22779,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22813,7 +22817,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22851,7 +22855,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22893,7 +22897,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22931,7 +22935,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22973,7 +22977,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -23015,7 +23019,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23057,7 +23061,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23104,7 +23108,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -23141,7 +23145,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23183,7 +23187,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23225,7 +23229,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23267,7 +23271,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23309,7 +23313,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23351,7 +23355,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23393,7 +23397,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23435,7 +23439,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23477,7 +23481,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23515,7 +23519,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23557,7 +23561,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23595,7 +23599,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23637,7 +23641,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23679,7 +23683,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23726,7 +23730,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -23763,7 +23767,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23805,7 +23809,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23843,7 +23847,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23881,7 +23885,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23919,7 +23923,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23961,7 +23965,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -24003,7 +24007,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24041,7 +24045,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24079,7 +24083,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24121,7 +24125,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24163,7 +24167,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24197,7 +24201,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24239,7 +24243,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24277,7 +24281,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24315,7 +24319,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24357,7 +24361,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24395,7 +24399,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24433,7 +24437,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24471,7 +24475,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24513,7 +24517,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24551,7 +24555,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24593,7 +24597,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24635,7 +24639,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24673,7 +24677,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24715,7 +24719,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24757,7 +24761,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24795,7 +24799,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24833,7 +24837,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24875,7 +24879,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24913,7 +24917,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24955,7 +24959,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -24997,7 +25001,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -25035,7 +25039,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25077,7 +25081,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25119,7 +25123,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25157,7 +25161,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25199,7 +25203,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25237,7 +25241,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25279,7 +25283,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25321,7 +25325,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25363,7 +25367,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25401,7 +25405,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25439,7 +25443,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25477,7 +25481,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25515,7 +25519,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25553,7 +25557,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25595,7 +25599,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25633,7 +25637,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25671,7 +25675,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25713,7 +25717,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25751,7 +25755,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25793,7 +25797,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25831,7 +25835,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25873,7 +25877,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25911,7 +25915,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25949,7 +25953,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25991,7 +25995,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26451,7 +26455,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26493,7 +26497,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26535,7 +26539,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26577,7 +26581,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26619,7 +26623,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26661,7 +26665,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26703,7 +26707,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26745,7 +26749,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26787,7 +26791,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26829,7 +26833,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26871,7 +26875,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26913,7 +26917,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26955,7 +26959,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -26997,7 +27001,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27039,7 +27043,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27081,7 +27085,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27123,7 +27127,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27165,7 +27169,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27207,7 +27211,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27249,7 +27253,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27291,7 +27295,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27333,7 +27337,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27375,7 +27379,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27417,7 +27421,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27459,7 +27463,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27501,7 +27505,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27543,12 +27547,12 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -27585,7 +27589,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27627,7 +27631,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27669,7 +27673,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27711,7 +27715,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27758,7 +27762,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -27795,7 +27799,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27837,7 +27841,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27879,7 +27883,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27921,7 +27925,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27963,7 +27967,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -28005,7 +28009,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28043,7 +28047,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28085,7 +28089,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28127,7 +28131,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28169,7 +28173,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28211,7 +28215,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28253,7 +28257,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28295,7 +28299,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28337,7 +28341,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28379,7 +28383,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28421,7 +28425,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28463,7 +28467,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28505,7 +28509,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28547,7 +28551,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28589,7 +28593,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28631,7 +28635,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28673,7 +28677,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28715,7 +28719,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28757,7 +28761,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28799,7 +28803,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28841,7 +28845,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28883,7 +28887,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28925,7 +28929,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28967,7 +28971,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -29009,7 +29013,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29051,7 +29055,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29093,7 +29097,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29135,7 +29139,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29177,7 +29181,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29219,7 +29223,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29261,7 +29265,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29303,7 +29307,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29345,7 +29349,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29387,7 +29391,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29429,7 +29433,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29471,7 +29475,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29513,7 +29517,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29555,7 +29559,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29597,7 +29601,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29639,7 +29643,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29681,7 +29685,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29723,7 +29727,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29765,7 +29769,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29807,7 +29811,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29849,7 +29853,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29891,7 +29895,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29933,7 +29937,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29975,7 +29979,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -30017,7 +30021,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30059,7 +30063,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30101,7 +30105,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30143,7 +30147,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30185,7 +30189,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30227,7 +30231,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30269,7 +30273,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30311,7 +30315,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30353,7 +30357,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30395,7 +30399,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30437,7 +30441,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30479,7 +30483,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30521,7 +30525,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30563,7 +30567,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30605,7 +30609,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30647,7 +30651,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30689,7 +30693,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30731,7 +30735,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30773,7 +30777,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30815,7 +30819,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30857,7 +30861,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -30899,7 +30903,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30946,7 +30950,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
@@ -30983,7 +30987,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -31025,7 +31029,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31067,7 +31071,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31109,12 +31113,12 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr">
@@ -31151,7 +31155,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31193,7 +31197,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31235,7 +31239,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31277,7 +31281,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31319,7 +31323,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31361,7 +31365,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31403,7 +31407,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31445,7 +31449,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31487,7 +31491,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31529,7 +31533,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31571,7 +31575,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31613,7 +31617,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31655,7 +31659,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31697,7 +31701,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31739,7 +31743,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31781,7 +31785,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31823,7 +31827,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31865,7 +31869,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31907,7 +31911,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31949,7 +31953,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31991,7 +31995,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -32033,7 +32037,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32075,7 +32079,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32117,7 +32121,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32159,7 +32163,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32201,7 +32205,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32243,7 +32247,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32285,7 +32289,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32327,7 +32331,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32369,7 +32373,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32411,7 +32415,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32453,7 +32457,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32495,7 +32499,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32537,7 +32541,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32575,7 +32579,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32617,7 +32621,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32655,7 +32659,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32689,7 +32693,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32731,7 +32735,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32769,7 +32773,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32811,7 +32815,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32853,7 +32857,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32891,7 +32895,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32929,7 +32933,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32967,7 +32971,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -33005,7 +33009,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -33047,7 +33051,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33085,7 +33089,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33119,7 +33123,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33157,7 +33161,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33195,7 +33199,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33233,7 +33237,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33275,7 +33279,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33317,7 +33321,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33355,7 +33359,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33397,7 +33401,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33431,7 +33435,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33469,7 +33473,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">
@@ -33507,7 +33511,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -33545,7 +33549,7 @@
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-25 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,12 +2890,12 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>2959d548616852711e1dc9a8dabc9bed791fca8d77122e8792af1c662e96519b</t>
+          <t>36cfe7e7863f9d1460b8dc4a91e8c1baec01e9664a492fb99d918b34bf2b6ea3</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6754,7 +6754,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7038,7 +7038,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8022,7 +8022,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8086,12 +8086,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8102,7 +8102,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>ec16154b2e6cb0039685099ba4e443616a578f95791b0d5c48d16015fbc6c010</t>
+          <t>f94cbc4b6bc97adfa8f365b3fb2acc80b7a68efecb5b634513c7a34545e51199</t>
         </is>
       </c>
     </row>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8222,7 +8222,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8286,7 +8286,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8622,7 +8622,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8690,7 +8690,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8762,7 +8762,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8958,7 +8958,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9030,7 +9030,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10906,7 +10906,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10974,7 +10974,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11046,12 +11046,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>07d867fd269caf9e144b0cba858438e669c2cc75144b79eea23d23004533efc7</t>
+          <t>2b34bf0659b9d3f823f4fc93184c9a8754485801a7cbd1ff9c615fe28f07beee</t>
         </is>
       </c>
     </row>
@@ -11118,7 +11118,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11190,7 +11190,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11262,7 +11262,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11406,7 +11406,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11474,7 +11474,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11546,7 +11546,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11618,7 +11618,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11690,7 +11690,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11758,7 +11758,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11902,7 +11902,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12034,14 +12034,14 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
+          <t>2026-10-25T12:45:50+00:00</t>
+        </is>
+      </c>
+      <c r="K207" s="2" t="inlineStr">
+        <is>
           <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
-      <c r="K207" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24T12:15:32+00:00</t>
-        </is>
-      </c>
       <c r="L207" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -12054,7 +12054,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>bf359ee82e724c180760278da6a06d5eab8aff10089ae2bee940fd935c706882</t>
+          <t>d9429ee44a65c1c084d33f4a7eb0abca1088557980e0d275d23636bbedce2a78</t>
         </is>
       </c>
     </row>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr">
@@ -12178,7 +12178,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12250,7 +12250,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12546,7 +12546,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr">
@@ -12798,7 +12798,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
@@ -12942,7 +12942,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13134,7 +13134,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
@@ -13206,7 +13206,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
@@ -13278,7 +13278,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13346,7 +13346,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13414,7 +13414,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13482,7 +13482,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13606,7 +13606,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13918,7 +13918,7 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
@@ -18190,7 +18190,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>61b3451cf0944575a0f283ac95411d2886f36165ee8db5aec2cf7cbcece34bb1</t>
+          <t>0d0903557b20b250d77fe4717ab0e84fd0e6cf11f2c019013fb01d38eac5720f</t>
         </is>
       </c>
     </row>
@@ -18262,7 +18262,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
@@ -18334,7 +18334,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18406,7 +18406,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18474,7 +18474,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18542,7 +18542,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18666,7 +18666,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19094,7 +19094,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19162,7 +19162,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19230,7 +19230,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19298,14 +19298,14 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
+          <t>2026-10-25T12:45:50+00:00</t>
+        </is>
+      </c>
+      <c r="K329" s="2" t="inlineStr">
+        <is>
           <t>2026-10-24T12:15:32+00:00</t>
         </is>
       </c>
-      <c r="K329" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-24T12:15:32+00:00</t>
-        </is>
-      </c>
       <c r="L329" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -19318,7 +19318,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>b0ef731f7675309ac4a16be433d63a7138d98382431aa0d8acfc9c8f9f236849</t>
+          <t>439e944c83e680160a90f29a1101c423cf46ea8e6467d1e245454887f990b462</t>
         </is>
       </c>
     </row>
@@ -19370,12 +19370,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19390,7 +19390,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>1d3e04e652eea2e4962588e50ee2a7e70ebef21b069f561cf63b9587abd82c99</t>
+          <t>cf06341ba0ba8d2ca0e5ee9341e4e87acdc49ef2c3b8c45418727964e3344e1c</t>
         </is>
       </c>
     </row>
@@ -19442,12 +19442,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19462,7 +19462,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>ecc2726efe9c8a66438b8d01ae204f4b39cc5e65e2a2855bd2ba929c7f6eadb9</t>
+          <t>1f20b813ef9937e0a3af45f16c907c599c9ae7463d73cb60ca258af29e5c8cce</t>
         </is>
       </c>
     </row>
@@ -19514,7 +19514,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr">
@@ -19642,7 +19642,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19710,7 +19710,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19778,7 +19778,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19846,7 +19846,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr">
@@ -19918,7 +19918,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
@@ -19990,7 +19990,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20058,7 +20058,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20126,7 +20126,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20194,12 +20194,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20214,7 +20214,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>0f386bd079120e1ec47a52702a962fb0230f0908b2e799e06332779392bd3a01</t>
+          <t>909a600664825efb05172e5e39765a0dfffa220d0a215c5b5b862ddc6f62fd5e</t>
         </is>
       </c>
     </row>
@@ -20382,7 +20382,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
@@ -20454,7 +20454,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20522,7 +20522,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20590,7 +20590,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20658,7 +20658,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20726,7 +20726,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20794,7 +20794,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20862,7 +20862,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20930,7 +20930,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -20998,7 +20998,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21062,7 +21062,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21122,7 +21122,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21194,7 +21194,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21258,7 +21258,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21330,7 +21330,7 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
@@ -21398,7 +21398,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr">
@@ -21470,7 +21470,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21530,7 +21530,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21594,7 +21594,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
@@ -21658,7 +21658,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21726,7 +21726,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr">
@@ -21798,7 +21798,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr">
@@ -21870,7 +21870,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21942,7 +21942,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -22070,7 +22070,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22547,7 +22547,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22589,7 +22589,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22623,7 +22623,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22665,7 +22665,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22703,7 +22703,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22741,7 +22741,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22779,7 +22779,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22817,7 +22817,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22855,7 +22855,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22897,7 +22897,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22935,7 +22935,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22977,7 +22977,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -23019,7 +23019,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23061,7 +23061,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23108,7 +23108,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -23145,7 +23145,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23187,7 +23187,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23229,7 +23229,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23271,7 +23271,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23313,7 +23313,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23355,7 +23355,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23397,7 +23397,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23439,7 +23439,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23481,7 +23481,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23519,7 +23519,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23561,7 +23561,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23599,7 +23599,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23641,7 +23641,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23683,7 +23683,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23730,7 +23730,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -23767,7 +23767,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23809,7 +23809,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23847,7 +23847,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23885,7 +23885,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23923,7 +23923,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23965,7 +23965,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -24007,7 +24007,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24045,7 +24045,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24083,7 +24083,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24125,7 +24125,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24167,7 +24167,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24201,7 +24201,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24243,7 +24243,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24281,7 +24281,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24319,7 +24319,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24361,7 +24361,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24399,7 +24399,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24437,7 +24437,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24475,7 +24475,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24517,7 +24517,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24555,7 +24555,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24597,7 +24597,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24639,7 +24639,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24677,7 +24677,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24719,7 +24719,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24761,7 +24761,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24799,7 +24799,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24837,7 +24837,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24879,7 +24879,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24917,7 +24917,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24959,7 +24959,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -25001,7 +25001,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -25039,7 +25039,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25081,7 +25081,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25123,7 +25123,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25161,7 +25161,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25241,7 +25241,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25283,7 +25283,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25325,7 +25325,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25367,7 +25367,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25405,7 +25405,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25443,7 +25443,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25481,7 +25481,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25519,7 +25519,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25557,7 +25557,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25599,7 +25599,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25637,7 +25637,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25675,7 +25675,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25717,7 +25717,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25755,7 +25755,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25797,7 +25797,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25835,7 +25835,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25877,7 +25877,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25915,7 +25915,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25953,7 +25953,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25995,7 +25995,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26455,7 +26455,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26497,7 +26497,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26539,7 +26539,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26581,7 +26581,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26623,7 +26623,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26665,7 +26665,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26707,7 +26707,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26749,7 +26749,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26791,7 +26791,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26833,7 +26833,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26875,7 +26875,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26917,7 +26917,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26959,7 +26959,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -27001,7 +27001,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27043,7 +27043,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27085,7 +27085,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27127,7 +27127,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27169,7 +27169,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27211,7 +27211,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27253,7 +27253,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27295,7 +27295,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27337,7 +27337,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27379,7 +27379,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27421,7 +27421,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27463,7 +27463,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27505,7 +27505,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27552,7 +27552,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -27589,7 +27589,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27631,7 +27631,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27673,7 +27673,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27715,7 +27715,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27762,7 +27762,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -27799,7 +27799,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27841,7 +27841,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27883,7 +27883,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27925,7 +27925,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27967,7 +27967,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -28009,7 +28009,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28047,7 +28047,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28089,7 +28089,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28131,7 +28131,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28173,7 +28173,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28215,7 +28215,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28257,7 +28257,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28299,7 +28299,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28341,7 +28341,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28383,7 +28383,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28425,7 +28425,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28467,7 +28467,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28551,7 +28551,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28593,7 +28593,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28635,7 +28635,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28677,7 +28677,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28719,7 +28719,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28766,7 +28766,7 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
@@ -28803,7 +28803,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28845,7 +28845,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28887,7 +28887,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28929,7 +28929,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28971,7 +28971,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -29013,7 +29013,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29055,7 +29055,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29097,7 +29097,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29139,7 +29139,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29181,7 +29181,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29223,7 +29223,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29265,7 +29265,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29349,7 +29349,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29391,7 +29391,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29433,7 +29433,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29475,7 +29475,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29517,7 +29517,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29559,7 +29559,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29601,7 +29601,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29643,7 +29643,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29685,7 +29685,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29727,7 +29727,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29769,7 +29769,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29811,7 +29811,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29853,7 +29853,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29895,7 +29895,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29937,7 +29937,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29979,7 +29979,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -30021,7 +30021,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30063,7 +30063,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30147,7 +30147,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30189,7 +30189,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30231,7 +30231,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30273,7 +30273,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30315,7 +30315,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30357,7 +30357,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30399,7 +30399,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30441,7 +30441,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30483,7 +30483,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30525,7 +30525,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30567,7 +30567,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30609,7 +30609,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30651,7 +30651,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30693,7 +30693,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30735,7 +30735,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30777,7 +30777,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30819,7 +30819,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30861,7 +30861,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30950,7 +30950,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
@@ -30987,7 +30987,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -31029,7 +31029,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31071,7 +31071,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31113,7 +31113,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31155,7 +31155,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31197,7 +31197,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31239,7 +31239,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31281,7 +31281,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31323,7 +31323,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31365,7 +31365,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31407,7 +31407,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31449,7 +31449,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31491,7 +31491,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31533,7 +31533,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31575,7 +31575,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31617,7 +31617,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31659,7 +31659,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31743,7 +31743,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31785,7 +31785,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31827,7 +31827,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31869,7 +31869,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31911,7 +31911,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31953,7 +31953,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31995,7 +31995,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -32037,7 +32037,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32079,7 +32079,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32121,7 +32121,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32163,7 +32163,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32205,7 +32205,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32247,7 +32247,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32289,7 +32289,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32331,7 +32331,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32373,7 +32373,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32415,7 +32415,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32457,7 +32457,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32541,7 +32541,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32579,7 +32579,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32621,7 +32621,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32659,7 +32659,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32693,7 +32693,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32735,7 +32735,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32773,7 +32773,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32815,7 +32815,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32857,7 +32857,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32895,7 +32895,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32933,7 +32933,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32971,7 +32971,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -33009,7 +33009,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -33051,7 +33051,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33089,7 +33089,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33123,7 +33123,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33161,7 +33161,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33199,7 +33199,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33237,7 +33237,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33279,7 +33279,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33321,7 +33321,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33359,7 +33359,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33401,7 +33401,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33435,7 +33435,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33473,7 +33473,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">
@@ -33511,7 +33511,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -33549,7 +33549,7 @@
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-25T12:45:50+00:00</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-27 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4370,12 +4370,12 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T17:00:36+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr"/>
@@ -4386,7 +4386,7 @@
       </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
-          <t>3e628bd46fa1eba3663970d0d6089738eebe3de8d257c74485de94a1cd5bb1a1</t>
+          <t>e15296f609410ed4a8094e376dcf9867064dee0a605c3263efbe9c72b180870b</t>
         </is>
       </c>
     </row>
@@ -4438,7 +4438,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7042,7 +7042,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8090,12 +8090,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>314d94697a986595fdbf8d0bb82a3e25cfb4922fb569b6e071c0c6a39b745425</t>
+          <t>41bbd881fbd20444a279669b31593e8477217a5f65a7aefca6fb1a638879d3e0</t>
         </is>
       </c>
     </row>
@@ -8158,12 +8158,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>24f341f568ac9ca3318ce1223a5746e6c8b0c0e97827fe05bc7f9733aa1d9b4b</t>
+          <t>fa9e7ba536b7e04d96f24172a0040ae336d5b2d47332ba38a6e281b5520a2c59</t>
         </is>
       </c>
     </row>
@@ -8226,7 +8226,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8694,12 +8694,12 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L153" s="2" t="inlineStr">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="N153" s="2" t="inlineStr">
         <is>
-          <t>5cab8e3dfb94db05f3ad9ed1df3e4ddc7ae7073cbf100c264896a197ae26d3fc</t>
+          <t>fba58b08d22d8ee40c05053a6472d7422b7d98f169a5c8fdf319d117bb7ce36c</t>
         </is>
       </c>
     </row>
@@ -8766,7 +8766,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8894,7 +8894,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10910,7 +10910,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10978,7 +10978,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11050,12 +11050,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11070,7 +11070,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>4f48160ea80ed9cbd65523d833831cddc94e113c98709b1107b1c32da9f84fbd</t>
+          <t>7546f6a39a9936015d0581096b9f644bc959de6cdfa98a5bd988e2b39d67c4cb</t>
         </is>
       </c>
     </row>
@@ -11122,7 +11122,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11194,7 +11194,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11266,7 +11266,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11338,7 +11338,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11410,7 +11410,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11478,7 +11478,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11622,7 +11622,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11694,7 +11694,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11834,7 +11834,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11906,7 +11906,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12058,7 +12058,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>d9429ee44a65c1c084d33f4a7eb0abca1088557980e0d275d23636bbedce2a78</t>
+          <t>67c2ef387811b67cbd4867bcbeed952e154b8781d4706888ab7cb294ca15dd21</t>
         </is>
       </c>
     </row>
@@ -12110,7 +12110,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12202,7 +12202,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
+          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
         </is>
       </c>
     </row>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12550,7 +12550,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr">
@@ -12802,7 +12802,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12874,12 +12874,12 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L220" s="2" t="inlineStr">
@@ -12894,7 +12894,7 @@
       </c>
       <c r="N220" s="2" t="inlineStr">
         <is>
-          <t>f1c4839314c0da41158444ec5ba0b31e3d1ce38eeae9005241cc51079080ca32</t>
+          <t>7f14a0cded0b343fd970abf1ec0a46ca3c4cf69a99155ca9fecc8ebc4af9edeb</t>
         </is>
       </c>
     </row>
@@ -12946,7 +12946,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
@@ -13282,7 +13282,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13350,7 +13350,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13418,7 +13418,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13610,7 +13610,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13630,7 +13630,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>a55a21f9c39028df1294608bfa4eea59bcb8dbf9cd3fc8ac33b197e038e27e34</t>
+          <t>81b08ef2d60fd5a14fe13a16786dc2b851da61934465f87b3d10b7fd33adff32</t>
         </is>
       </c>
     </row>
@@ -13922,7 +13922,7 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
@@ -13942,7 +13942,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>e46a610694756c9ce72c5673c1e53b7f8db9ce7067f0be6ddb49559bda9705e9</t>
+          <t>c215cec8a9a3dd27da11e5e0a2ca791929570af6b530d22ef0f3f0f396d226c1</t>
         </is>
       </c>
     </row>
@@ -18194,12 +18194,12 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T12:54:41+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L312" s="2" t="inlineStr">
@@ -18214,7 +18214,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>0d0903557b20b250d77fe4717ab0e84fd0e6cf11f2c019013fb01d38eac5720f</t>
+          <t>6a564e4611aac05779e1c5027b4da05c2c9f2574f2e4385e052b1e2aa3d94f00</t>
         </is>
       </c>
     </row>
@@ -18266,7 +18266,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
@@ -18286,7 +18286,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>daf334636d5c335aebfb661951da905e75f609ba5ab5b0142c167945b98a44f0</t>
+          <t>a6f546c638009a6787e0d6bd369d8c11f02e293603056276224932d7a9f843a5</t>
         </is>
       </c>
     </row>
@@ -18338,7 +18338,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18410,7 +18410,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18478,7 +18478,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18546,7 +18546,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18670,7 +18670,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19098,7 +19098,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19166,7 +19166,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19234,7 +19234,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19302,12 +19302,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19322,7 +19322,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>d549fbf6112a74a7059c4ea5ae02a679f377a748052b878f9b08caa927e15f7e</t>
+          <t>9b684198cfc569af1019587c4aa34bb247b4cf9e90ff30676db10e73036ef711</t>
         </is>
       </c>
     </row>
@@ -19374,12 +19374,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T12:45:50+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19394,7 +19394,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>558a778e640ae7414537ae3735d447de7c176c2bff2792e39414893d928a4204</t>
+          <t>28488949ceb8403541b3a9ec878ffb7add38eda0d8ca3c60a36258cb40ab1107</t>
         </is>
       </c>
     </row>
@@ -19446,12 +19446,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19466,7 +19466,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>48426f9161a7bd5a93ff89b365170fe42e24825dda3fa3897df3ddaf83be23ac</t>
+          <t>2afe1a56676e3cb6be2eb0d02556f6ff1d3e4013cbd885e8cbb650c8b15784cd</t>
         </is>
       </c>
     </row>
@@ -19518,7 +19518,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr">
@@ -19646,7 +19646,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19714,7 +19714,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19782,7 +19782,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19850,7 +19850,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr">
@@ -19922,7 +19922,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
@@ -19994,7 +19994,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20062,7 +20062,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20130,7 +20130,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20198,12 +20198,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20218,7 +20218,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>a70e6bfe757d778dc36cbe864fc9d22b644bd49cba0174b6da9ee50278099dd8</t>
+          <t>50f90b6ed2da15ce202832d8ac1811a2a83a5948b8bcd2d522bf60a6d3ed68e5</t>
         </is>
       </c>
     </row>
@@ -20386,7 +20386,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
@@ -20458,7 +20458,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20526,7 +20526,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20594,7 +20594,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20662,7 +20662,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20730,7 +20730,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20798,7 +20798,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20866,7 +20866,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20934,7 +20934,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -21002,7 +21002,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21066,7 +21066,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21126,7 +21126,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21198,7 +21198,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21262,7 +21262,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21334,12 +21334,12 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
@@ -21354,7 +21354,7 @@
       </c>
       <c r="N359" s="2" t="inlineStr">
         <is>
-          <t>d080f4d6171318a1aca6606148bd9bda1b93193acf09291580d3911f802f28e0</t>
+          <t>d1b52e0f637ba877e4abd3cf8228dcfa776c9acf278e6ca8884ed370932f0483</t>
         </is>
       </c>
     </row>
@@ -21402,7 +21402,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr">
@@ -21474,7 +21474,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21534,7 +21534,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21598,7 +21598,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
@@ -21662,7 +21662,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21730,7 +21730,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr">
@@ -21802,12 +21802,12 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="L366" s="2" t="inlineStr">
@@ -21822,7 +21822,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>212251414afa7d6f44f6c16d1d1f37b7a00d19bc88f646a7998797b382877dae</t>
+          <t>789f2ac84c585c95cd5fb972deaa2f6dd02ec52575fb158573ee482c6bd4b929</t>
         </is>
       </c>
     </row>
@@ -21874,7 +21874,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21946,7 +21946,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -22074,7 +22074,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22551,7 +22551,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22593,7 +22593,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22627,7 +22627,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22669,7 +22669,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22707,7 +22707,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22745,7 +22745,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22783,7 +22783,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22821,7 +22821,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22859,7 +22859,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22901,7 +22901,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22939,7 +22939,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22981,7 +22981,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -23023,7 +23023,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23065,7 +23065,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23149,7 +23149,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23191,7 +23191,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23233,7 +23233,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23275,7 +23275,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23317,7 +23317,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23359,7 +23359,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23401,7 +23401,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23443,7 +23443,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23485,7 +23485,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23523,7 +23523,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23565,7 +23565,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23603,7 +23603,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23645,7 +23645,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23687,7 +23687,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23734,7 +23734,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -23771,7 +23771,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23813,7 +23813,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23851,7 +23851,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23889,7 +23889,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23927,7 +23927,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23969,7 +23969,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -24011,7 +24011,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24049,7 +24049,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24087,7 +24087,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24129,7 +24129,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24171,7 +24171,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24205,7 +24205,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24247,7 +24247,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24285,7 +24285,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24323,7 +24323,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24365,7 +24365,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24403,7 +24403,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24441,7 +24441,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24479,7 +24479,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24521,7 +24521,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24559,7 +24559,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24601,7 +24601,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24643,7 +24643,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24681,7 +24681,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24723,7 +24723,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24765,7 +24765,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24803,7 +24803,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24841,7 +24841,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24883,7 +24883,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24921,7 +24921,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24963,7 +24963,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -25005,7 +25005,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -25043,7 +25043,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25085,7 +25085,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25127,7 +25127,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25165,7 +25165,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25207,7 +25207,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25245,7 +25245,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25287,7 +25287,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25329,7 +25329,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25371,7 +25371,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25409,7 +25409,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25447,7 +25447,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25485,7 +25485,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25523,7 +25523,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25561,7 +25561,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25603,7 +25603,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25641,7 +25641,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25679,7 +25679,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25721,7 +25721,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25759,7 +25759,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25801,7 +25801,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25839,7 +25839,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25881,7 +25881,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25919,7 +25919,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25957,7 +25957,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25999,7 +25999,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26459,7 +26459,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26501,7 +26501,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26543,7 +26543,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26585,7 +26585,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26627,7 +26627,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26669,7 +26669,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26711,7 +26711,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26753,7 +26753,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26795,7 +26795,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26837,7 +26837,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26879,7 +26879,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26921,7 +26921,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26963,7 +26963,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -27005,7 +27005,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27047,7 +27047,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27089,7 +27089,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27131,7 +27131,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27173,7 +27173,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27215,7 +27215,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27257,7 +27257,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27299,7 +27299,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27341,7 +27341,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27383,7 +27383,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27425,7 +27425,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27467,7 +27467,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27509,7 +27509,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27551,12 +27551,12 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -27593,7 +27593,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27635,7 +27635,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27677,7 +27677,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27719,7 +27719,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27803,7 +27803,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27845,7 +27845,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27887,7 +27887,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27929,7 +27929,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27971,7 +27971,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -28013,7 +28013,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28051,7 +28051,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28093,7 +28093,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28135,7 +28135,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28177,7 +28177,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28219,7 +28219,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28261,7 +28261,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28303,7 +28303,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28345,7 +28345,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28387,7 +28387,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28429,7 +28429,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28471,7 +28471,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28513,7 +28513,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28555,7 +28555,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28597,7 +28597,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28639,7 +28639,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28681,7 +28681,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28723,7 +28723,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28770,7 +28770,7 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
@@ -28807,7 +28807,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28849,7 +28849,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28891,7 +28891,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28933,7 +28933,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28975,7 +28975,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -29017,7 +29017,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29059,7 +29059,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29101,7 +29101,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29143,7 +29143,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29185,7 +29185,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29227,7 +29227,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29269,7 +29269,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29311,7 +29311,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29353,7 +29353,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29395,7 +29395,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29437,7 +29437,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29479,7 +29479,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29521,7 +29521,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29563,7 +29563,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29605,7 +29605,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29647,7 +29647,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29689,7 +29689,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29731,7 +29731,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29773,7 +29773,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29815,7 +29815,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29857,7 +29857,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29899,7 +29899,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29941,7 +29941,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29983,7 +29983,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -30025,7 +30025,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30067,7 +30067,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30109,7 +30109,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30151,7 +30151,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30193,7 +30193,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30235,7 +30235,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30277,7 +30277,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30319,7 +30319,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30361,7 +30361,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30403,7 +30403,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30445,7 +30445,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30487,7 +30487,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30529,7 +30529,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30571,7 +30571,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30613,7 +30613,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30655,7 +30655,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30697,7 +30697,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30739,7 +30739,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30781,7 +30781,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30823,7 +30823,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30865,7 +30865,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -30907,7 +30907,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30954,7 +30954,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
@@ -30991,7 +30991,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -31033,7 +31033,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31075,7 +31075,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31117,7 +31117,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31159,7 +31159,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31201,7 +31201,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31243,7 +31243,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31285,7 +31285,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31327,7 +31327,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31369,7 +31369,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31411,7 +31411,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31453,7 +31453,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31495,7 +31495,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31537,7 +31537,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31579,7 +31579,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31621,7 +31621,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31663,7 +31663,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31705,7 +31705,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31747,7 +31747,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31789,7 +31789,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31831,7 +31831,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31873,7 +31873,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31915,7 +31915,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31957,7 +31957,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31999,7 +31999,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -32041,7 +32041,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32083,7 +32083,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32125,7 +32125,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32167,7 +32167,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32209,7 +32209,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32251,7 +32251,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32293,7 +32293,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32335,7 +32335,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32377,7 +32377,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32419,7 +32419,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32461,7 +32461,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32503,7 +32503,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32545,7 +32545,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32583,7 +32583,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32625,7 +32625,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32663,7 +32663,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32697,7 +32697,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32739,7 +32739,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32777,7 +32777,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32819,7 +32819,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32861,7 +32861,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32899,7 +32899,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32937,7 +32937,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32975,7 +32975,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -33013,7 +33013,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -33055,7 +33055,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33093,7 +33093,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33127,7 +33127,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33165,7 +33165,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33203,7 +33203,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33241,7 +33241,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33283,7 +33283,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33325,7 +33325,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33363,7 +33363,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33405,7 +33405,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33439,7 +33439,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33477,7 +33477,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">
@@ -33515,7 +33515,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -33553,7 +33553,7 @@
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-28 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5134,12 +5134,12 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L87" s="2" t="inlineStr"/>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>625e76ecfdad5d74642611ccbadcf8b5d220364b1268287f2eeacbc5d3cdafca</t>
+          <t>e24ed6242b99c0cd8efdb749e2e9e5c871d9f305b0561e7606a169c646688680</t>
         </is>
       </c>
     </row>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7042,7 +7042,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8090,12 +8090,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>41bbd881fbd20444a279669b31593e8477217a5f65a7aefca6fb1a638879d3e0</t>
+          <t>5cb393f25309756e3c3894ca7d0d9d52b9edaf5612da5e06e41c6e45b4c084c9</t>
         </is>
       </c>
     </row>
@@ -8158,7 +8158,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8226,7 +8226,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8694,7 +8694,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8766,7 +8766,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8894,7 +8894,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10910,7 +10910,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10978,7 +10978,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11050,12 +11050,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11070,7 +11070,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>7546f6a39a9936015d0581096b9f644bc959de6cdfa98a5bd988e2b39d67c4cb</t>
+          <t>d231c0279f7d536708aa62902fb48e54c65588e6f0ceefa4443bac430f38b156</t>
         </is>
       </c>
     </row>
@@ -11122,12 +11122,12 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>d61d4d289a2bf8129a529403eb6435c09ac7ad1141cce1b809d6ecee90342f05</t>
+          <t>51efa12106aa05172a702a81599a2a64c85ce5c863827c59cf87f49c377a6345</t>
         </is>
       </c>
     </row>
@@ -11194,12 +11194,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23T12:52:38+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>3184c99249877695e5c89421a1d59ab1f51f04c6ee87a489401c8d4f62ed7ef3</t>
+          <t>e0fd36d887acac7b270e3598b39b9f4f490ff550b61dca0650dbd209834c45d2</t>
         </is>
       </c>
     </row>
@@ -11266,7 +11266,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11338,7 +11338,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11410,7 +11410,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11478,7 +11478,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11622,7 +11622,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11694,7 +11694,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11762,12 +11762,12 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L203" s="2" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="N203" s="2" t="inlineStr">
         <is>
-          <t>7cf156acfa8cf7fd013d37471de6869ee4faa3c303815e72a9863af6079fa69f</t>
+          <t>806c4f3862ff5b209744ae0740c467cdcbdf8a3a657c768114eb1417e26ead33</t>
         </is>
       </c>
     </row>
@@ -11834,7 +11834,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11906,7 +11906,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12058,7 +12058,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>67c2ef387811b67cbd4867bcbeed952e154b8781d4706888ab7cb294ca15dd21</t>
+          <t>c19bf9561bb826e40743446c61c2095470d2e85f138c844831d1093305244fdd</t>
         </is>
       </c>
     </row>
@@ -12110,7 +12110,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr">
@@ -12182,12 +12182,12 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
@@ -12202,7 +12202,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
+          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
         </is>
       </c>
     </row>
@@ -12254,7 +12254,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12550,7 +12550,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr">
@@ -12802,7 +12802,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12874,7 +12874,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
@@ -12946,7 +12946,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
@@ -13282,7 +13282,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13350,7 +13350,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13418,7 +13418,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13486,7 +13486,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13610,7 +13610,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13630,7 +13630,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>81b08ef2d60fd5a14fe13a16786dc2b851da61934465f87b3d10b7fd33adff32</t>
+          <t>a55a21f9c39028df1294608bfa4eea59bcb8dbf9cd3fc8ac33b197e038e27e34</t>
         </is>
       </c>
     </row>
@@ -13922,7 +13922,7 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
@@ -18194,7 +18194,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18266,12 +18266,12 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20T12:58:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L313" s="2" t="inlineStr">
@@ -18286,7 +18286,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>a6f546c638009a6787e0d6bd369d8c11f02e293603056276224932d7a9f843a5</t>
+          <t>574614fd2266f5b64dd98441f469f25c1083046f394b41304bad2d486e8403d8</t>
         </is>
       </c>
     </row>
@@ -18338,7 +18338,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18410,7 +18410,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18478,7 +18478,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18546,7 +18546,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18670,7 +18670,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19098,7 +19098,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19166,7 +19166,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19234,7 +19234,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19302,12 +19302,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19322,7 +19322,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>9b684198cfc569af1019587c4aa34bb247b4cf9e90ff30676db10e73036ef711</t>
+          <t>255e3c60fc11d92af1f5da9cfd9b185d35d678e4bed8b55fbde4aca986af5bc9</t>
         </is>
       </c>
     </row>
@@ -19374,12 +19374,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19394,7 +19394,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>28488949ceb8403541b3a9ec878ffb7add38eda0d8ca3c60a36258cb40ab1107</t>
+          <t>654d2fae05243e8c663285119065c90da120b489490ba77e5129566823f55e8b</t>
         </is>
       </c>
     </row>
@@ -19446,12 +19446,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19466,7 +19466,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>2afe1a56676e3cb6be2eb0d02556f6ff1d3e4013cbd885e8cbb650c8b15784cd</t>
+          <t>fea00abbbc4148df3cefaf9b8c9b7038f097b4a05f45d3b83fe280d34c572e73</t>
         </is>
       </c>
     </row>
@@ -19518,7 +19518,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr">
@@ -19646,7 +19646,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19714,7 +19714,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19782,7 +19782,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19850,12 +19850,12 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T13:25:45+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L337" s="2" t="inlineStr">
@@ -19870,7 +19870,7 @@
       </c>
       <c r="N337" s="2" t="inlineStr">
         <is>
-          <t>43a402336a674da1b0b03d2040f92387ba0b1845d1c5c991801d8c0d99f9b67f</t>
+          <t>45f62bb98d58760c3c08ad7c5646813fbc454b8f4168d36e44ea545b8a115edc</t>
         </is>
       </c>
     </row>
@@ -19922,12 +19922,12 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L338" s="2" t="inlineStr">
@@ -19942,7 +19942,7 @@
       </c>
       <c r="N338" s="2" t="inlineStr">
         <is>
-          <t>36cfb98dd54f71e606063c0c528878f1c8de90a5438a168a9e85402351e78895</t>
+          <t>081a06496a9f2d956d351497c360c461bce278d62371b5ea0469baf0a6899b88</t>
         </is>
       </c>
     </row>
@@ -19994,7 +19994,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20062,7 +20062,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20130,7 +20130,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20198,12 +20198,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20218,7 +20218,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>50f90b6ed2da15ce202832d8ac1811a2a83a5948b8bcd2d522bf60a6d3ed68e5</t>
+          <t>a74f2430b67ce7fba5025f7cd3749aeb9fae367edb80b85543e8b5388ba290aa</t>
         </is>
       </c>
     </row>
@@ -20386,7 +20386,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
@@ -20458,7 +20458,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20526,10 +20526,14 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
-        </is>
-      </c>
-      <c r="K347" s="2" t="inlineStr"/>
+          <t>2026-10-28T14:21:26+00:00</t>
+        </is>
+      </c>
+      <c r="K347" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28T14:21:26+00:00</t>
+        </is>
+      </c>
       <c r="L347" s="2" t="inlineStr">
         <is>
           <t>2026-10-08</t>
@@ -20542,7 +20546,7 @@
       </c>
       <c r="N347" s="2" t="inlineStr">
         <is>
-          <t>a99f4492af7218450a406851894cfca0769c5478fffc760eb7fefd5656e32715</t>
+          <t>88052aa7aac873500adad400f63cc8b9468f260a7cdb2d82376366f2bb02d633</t>
         </is>
       </c>
     </row>
@@ -20594,7 +20598,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20662,7 +20666,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20730,7 +20734,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20798,7 +20802,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20866,7 +20870,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20934,7 +20938,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -21002,7 +21006,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21066,7 +21070,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21126,7 +21130,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21198,7 +21202,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21262,12 +21266,12 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26T14:23:43+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L358" s="2" t="inlineStr">
@@ -21282,7 +21286,7 @@
       </c>
       <c r="N358" s="2" t="inlineStr">
         <is>
-          <t>7073f1b7294b56fdccf6117e2f6be794214fcb824ac8379bbef00ee4f7420466</t>
+          <t>3d4820fdb45b2fffdfd789e97809b106421f81fb40c3f79744dede939398a8e5</t>
         </is>
       </c>
     </row>
@@ -21334,12 +21338,12 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
@@ -21354,7 +21358,7 @@
       </c>
       <c r="N359" s="2" t="inlineStr">
         <is>
-          <t>d1b52e0f637ba877e4abd3cf8228dcfa776c9acf278e6ca8884ed370932f0483</t>
+          <t>d6885681a201a6d997c84c467335622ed9421af02f6710c63beceecf221a9f30</t>
         </is>
       </c>
     </row>
@@ -21402,12 +21406,12 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T13:15:03+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L360" s="2" t="inlineStr">
@@ -21422,7 +21426,7 @@
       </c>
       <c r="N360" s="2" t="inlineStr">
         <is>
-          <t>122bca2d9362d91f97d56c159adf44dfbe6c85e6423e14cd3c8917eef16a12c0</t>
+          <t>a54d920afb677546fcf6794fbe91c3dfccd97acc90d33d30286f49a25165feca</t>
         </is>
       </c>
     </row>
@@ -21474,7 +21478,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21534,7 +21538,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21598,12 +21602,12 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:54:11+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="L363" s="2" t="inlineStr">
@@ -21618,7 +21622,7 @@
       </c>
       <c r="N363" s="2" t="inlineStr">
         <is>
-          <t>7b1f768edd0308f6c8f336441a21949bd99ec36f5cddddccb3f9198c3e4fd9a1</t>
+          <t>7ec3db99e6ad6f11d8c2ced072aaf23b7fbbeb405b4db04385e71dcf5864d5dd</t>
         </is>
       </c>
     </row>
@@ -21662,7 +21666,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21730,7 +21734,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr">
@@ -21750,7 +21754,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>45a79498aa39c0931a47d6ea55f86a7e5693cb49d5a537299ab5bf6be2143c8a</t>
+          <t>af9261098e89ea7c32af249b66204dd0966bcaf94a3862b9471a1b5a2ef76441</t>
         </is>
       </c>
     </row>
@@ -21802,14 +21806,14 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
+          <t>2026-10-28T14:21:26+00:00</t>
+        </is>
+      </c>
+      <c r="K366" s="2" t="inlineStr">
+        <is>
           <t>2026-10-27T13:29:58+00:00</t>
         </is>
       </c>
-      <c r="K366" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-27T13:29:58+00:00</t>
-        </is>
-      </c>
       <c r="L366" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21822,7 +21826,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>789f2ac84c585c95cd5fb972deaa2f6dd02ec52575fb158573ee482c6bd4b929</t>
+          <t>48987afc9d2a618b5b41a8ac1364e9673f19a6b8d8739b2b35b6e89f11a12c5d</t>
         </is>
       </c>
     </row>
@@ -21874,7 +21878,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21946,7 +21950,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -22074,7 +22078,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22551,7 +22555,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22593,7 +22597,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22627,7 +22631,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22669,7 +22673,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22707,7 +22711,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22745,7 +22749,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22783,7 +22787,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22821,7 +22825,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22859,7 +22863,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22901,7 +22905,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22939,7 +22943,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22981,7 +22985,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -23023,7 +23027,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23065,7 +23069,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23149,7 +23153,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23191,7 +23195,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23233,7 +23237,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23275,7 +23279,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23317,7 +23321,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23359,7 +23363,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23401,7 +23405,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23443,7 +23447,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23485,7 +23489,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23523,7 +23527,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23565,7 +23569,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23603,7 +23607,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23645,7 +23649,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23687,7 +23691,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23734,7 +23738,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -23771,7 +23775,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23813,7 +23817,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23851,7 +23855,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23889,7 +23893,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23927,7 +23931,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23969,7 +23973,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -24011,7 +24015,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24049,7 +24053,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24087,7 +24091,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24129,7 +24133,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24171,7 +24175,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24205,7 +24209,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24247,7 +24251,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24285,7 +24289,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24323,7 +24327,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24365,7 +24369,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24403,7 +24407,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24441,7 +24445,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24479,7 +24483,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24521,7 +24525,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24559,7 +24563,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24601,7 +24605,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24643,7 +24647,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24681,7 +24685,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24723,7 +24727,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24765,7 +24769,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24803,7 +24807,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24841,7 +24845,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24883,7 +24887,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24921,7 +24925,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24963,7 +24967,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -25005,7 +25009,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -25043,7 +25047,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25085,7 +25089,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25127,7 +25131,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25165,7 +25169,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25207,7 +25211,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25245,7 +25249,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25287,7 +25291,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25329,7 +25333,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25371,7 +25375,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25409,7 +25413,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25447,7 +25451,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25485,7 +25489,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25523,7 +25527,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25561,7 +25565,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25603,7 +25607,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25641,7 +25645,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25679,7 +25683,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25721,7 +25725,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25759,7 +25763,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25801,7 +25805,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25839,7 +25843,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25881,7 +25885,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25919,7 +25923,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25957,7 +25961,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -25999,7 +26003,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26459,7 +26463,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26501,7 +26505,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26543,7 +26547,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26585,7 +26589,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26627,7 +26631,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26669,7 +26673,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26711,7 +26715,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26753,7 +26757,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26795,7 +26799,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26837,7 +26841,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26879,7 +26883,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26921,7 +26925,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26963,7 +26967,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -27005,7 +27009,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27047,7 +27051,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27089,7 +27093,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27131,7 +27135,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27173,7 +27177,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27215,7 +27219,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27257,7 +27261,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27299,7 +27303,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27341,7 +27345,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27383,7 +27387,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27425,7 +27429,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27467,7 +27471,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27509,7 +27513,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27551,7 +27555,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27593,7 +27597,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27635,7 +27639,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27677,7 +27681,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27719,7 +27723,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27766,7 +27770,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -27803,7 +27807,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27845,7 +27849,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27887,7 +27891,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27929,7 +27933,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27971,7 +27975,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -28013,7 +28017,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28051,7 +28055,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28093,7 +28097,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28135,7 +28139,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28177,7 +28181,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28219,7 +28223,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28261,7 +28265,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28303,7 +28307,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28345,7 +28349,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28387,7 +28391,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28429,7 +28433,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28471,7 +28475,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28513,7 +28517,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28555,7 +28559,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28597,7 +28601,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28639,7 +28643,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28681,7 +28685,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28723,7 +28727,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28770,7 +28774,7 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
@@ -28807,7 +28811,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28849,7 +28853,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28891,7 +28895,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28933,7 +28937,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28975,7 +28979,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -29017,7 +29021,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29059,7 +29063,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29101,7 +29105,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29143,7 +29147,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29185,7 +29189,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29227,7 +29231,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29269,7 +29273,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29311,7 +29315,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29353,7 +29357,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29395,7 +29399,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29437,7 +29441,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29479,7 +29483,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29521,7 +29525,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29563,7 +29567,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29605,7 +29609,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29647,7 +29651,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29689,7 +29693,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29731,7 +29735,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -29773,7 +29777,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29815,7 +29819,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29857,7 +29861,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29899,7 +29903,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29941,7 +29945,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29983,7 +29987,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -30025,7 +30029,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30067,7 +30071,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30109,7 +30113,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30151,7 +30155,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30193,7 +30197,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30235,7 +30239,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30277,7 +30281,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30319,7 +30323,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30361,7 +30365,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30403,7 +30407,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30445,7 +30449,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30487,7 +30491,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30529,7 +30533,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30571,7 +30575,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30613,7 +30617,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30655,7 +30659,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30697,7 +30701,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30739,7 +30743,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30781,7 +30785,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30823,7 +30827,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30865,7 +30869,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -30907,7 +30911,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30954,7 +30958,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
@@ -30991,7 +30995,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -31033,7 +31037,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31075,7 +31079,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31117,7 +31121,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31159,7 +31163,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31201,7 +31205,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31243,7 +31247,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31285,7 +31289,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31327,7 +31331,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31369,7 +31373,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31411,7 +31415,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31453,7 +31457,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31495,7 +31499,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31537,7 +31541,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31579,7 +31583,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31621,7 +31625,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31663,7 +31667,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31705,7 +31709,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31747,7 +31751,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31789,7 +31793,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31831,7 +31835,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31873,7 +31877,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31915,7 +31919,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31957,7 +31961,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -31999,7 +32003,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -32041,7 +32045,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32083,7 +32087,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32125,7 +32129,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32167,7 +32171,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32209,7 +32213,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32251,7 +32255,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32293,7 +32297,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32335,7 +32339,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32377,7 +32381,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32419,7 +32423,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32461,7 +32465,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32503,7 +32507,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32545,7 +32549,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32583,7 +32587,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32625,7 +32629,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32663,7 +32667,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32697,7 +32701,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32739,7 +32743,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32777,7 +32781,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32819,7 +32823,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32861,7 +32865,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32899,7 +32903,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32937,7 +32941,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32975,7 +32979,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -33013,7 +33017,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -33055,7 +33059,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33093,7 +33097,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33127,7 +33131,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33165,7 +33169,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33203,7 +33207,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33241,7 +33245,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33283,7 +33287,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33325,7 +33329,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33363,7 +33367,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33405,7 +33409,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33439,7 +33443,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33477,7 +33481,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">
@@ -33515,7 +33519,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -33553,7 +33557,7 @@
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-29 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7042,7 +7042,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8090,12 +8090,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>5cb393f25309756e3c3894ca7d0d9d52b9edaf5612da5e06e41c6e45b4c084c9</t>
+          <t>03badc26d23332eddcede7a6268a106f56f04f08c2035bd0c52f7ace892c8828</t>
         </is>
       </c>
     </row>
@@ -8158,12 +8158,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>fa9e7ba536b7e04d96f24172a0040ae336d5b2d47332ba38a6e281b5520a2c59</t>
+          <t>178ebd8f760edfbb4d15364b0a47e22f57fb0cba6c36107801788cbc03178169</t>
         </is>
       </c>
     </row>
@@ -8226,7 +8226,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8694,7 +8694,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8766,7 +8766,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8894,7 +8894,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10910,7 +10910,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10978,7 +10978,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -10998,7 +10998,7 @@
       </c>
       <c r="N192" s="2" t="inlineStr">
         <is>
-          <t>aaf27aac7cfbdfd186ccb80f279814b64890cc27087b3bd14d80bfa6640f06a7</t>
+          <t>efae0dae52d3959e219660f18fa173fb3ba9d3f86925d83d11a416724271b032</t>
         </is>
       </c>
     </row>
@@ -11050,12 +11050,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11070,7 +11070,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>d231c0279f7d536708aa62902fb48e54c65588e6f0ceefa4443bac430f38b156</t>
+          <t>cb6adaab7878572b60a4a8aae6c9bcd601a4e59bda9e47559103adfcd0724b07</t>
         </is>
       </c>
     </row>
@@ -11122,12 +11122,12 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
@@ -11142,7 +11142,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>51efa12106aa05172a702a81599a2a64c85ce5c863827c59cf87f49c377a6345</t>
+          <t>0b27eab5cd95f98e30b49b2e885b954039e0948f2a1e4e57f399e6f4bdfa9ac3</t>
         </is>
       </c>
     </row>
@@ -11194,14 +11194,14 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
+          <t>2026-10-29T14:26:50+00:00</t>
+        </is>
+      </c>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
           <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
-      <c r="K195" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-28T14:21:26+00:00</t>
-        </is>
-      </c>
       <c r="L195" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11214,7 +11214,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>e0fd36d887acac7b270e3598b39b9f4f490ff550b61dca0650dbd209834c45d2</t>
+          <t>7856641f8326bdd8b90a856d2361d918eb5c404d78e2d63f06c2b8a8f3b57bac</t>
         </is>
       </c>
     </row>
@@ -11266,7 +11266,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11338,7 +11338,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11410,7 +11410,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11478,7 +11478,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11622,12 +11622,12 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T12:17:25+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="L201" s="2" t="inlineStr">
@@ -11642,7 +11642,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>39a5b5aec077f70883b6209af0e2f1382a8234a06b7bd7fe7ca93e263a5fa4dd</t>
+          <t>d97c5d2cdead707e1eb4f0b0de08498e8de550425fbaea21dd19993937be60aa</t>
         </is>
       </c>
     </row>
@@ -11694,7 +11694,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11834,7 +11834,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11906,7 +11906,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12058,7 +12058,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>c19bf9561bb826e40743446c61c2095470d2e85f138c844831d1093305244fdd</t>
+          <t>b8b0809430253e08f5237a8befd2537454a10d56d9f2ff70cbd1221d28e886f3</t>
         </is>
       </c>
     </row>
@@ -12110,7 +12110,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12254,7 +12254,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12550,7 +12550,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr">
@@ -12802,7 +12802,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12874,7 +12874,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
@@ -12946,7 +12946,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13138,7 +13138,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
@@ -13282,7 +13282,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13350,7 +13350,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13418,10 +13418,14 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
-        </is>
-      </c>
-      <c r="K228" s="2" t="inlineStr"/>
+          <t>2026-10-29T14:26:50+00:00</t>
+        </is>
+      </c>
+      <c r="K228" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29T14:26:50+00:00</t>
+        </is>
+      </c>
       <c r="L228" s="2" t="inlineStr">
         <is>
           <t>2026-10-08</t>
@@ -13434,7 +13438,7 @@
       </c>
       <c r="N228" s="2" t="inlineStr">
         <is>
-          <t>9ad1b81208e9662d9d0b011457b245be0df7486d3a66e613119d2e03034a8099</t>
+          <t>3c5c5a5186f1407095a781593880d3da8caf970f46480f15754441563af8dfbe</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13490,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13610,7 +13614,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13922,7 +13926,7 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
@@ -18194,7 +18198,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18214,7 +18218,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>6a564e4611aac05779e1c5027b4da05c2c9f2574f2e4385e052b1e2aa3d94f00</t>
+          <t>5ba9f3e088e5fde0df07eeb540628f48fc0d0fa712560e89a326c25339b1173b</t>
         </is>
       </c>
     </row>
@@ -18266,14 +18270,14 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
+          <t>2026-10-29T14:26:50+00:00</t>
+        </is>
+      </c>
+      <c r="K313" s="2" t="inlineStr">
+        <is>
           <t>2026-10-28T14:21:26+00:00</t>
         </is>
       </c>
-      <c r="K313" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-28T14:21:26+00:00</t>
-        </is>
-      </c>
       <c r="L313" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -18286,7 +18290,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>574614fd2266f5b64dd98441f469f25c1083046f394b41304bad2d486e8403d8</t>
+          <t>501483015645273acb71f5c24f1b7a293ba100e50c72e890b1ade6d9e5e38a8c</t>
         </is>
       </c>
     </row>
@@ -18338,7 +18342,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18410,7 +18414,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18478,7 +18482,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18546,7 +18550,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18670,7 +18674,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19098,7 +19102,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19166,7 +19170,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19234,7 +19238,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19302,12 +19306,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19322,7 +19326,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>255e3c60fc11d92af1f5da9cfd9b185d35d678e4bed8b55fbde4aca986af5bc9</t>
+          <t>c3f025bb73b38c43041e86e2f2f9ec3d376b1b4cee2171b25dce0f67f984de81</t>
         </is>
       </c>
     </row>
@@ -19374,12 +19378,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19394,7 +19398,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>654d2fae05243e8c663285119065c90da120b489490ba77e5129566823f55e8b</t>
+          <t>b230bdfa36da8b0649a4122b46e5a2605c9e992087229932fb9517617b7fae12</t>
         </is>
       </c>
     </row>
@@ -19446,12 +19450,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19466,7 +19470,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>fea00abbbc4148df3cefaf9b8c9b7038f097b4a05f45d3b83fe280d34c572e73</t>
+          <t>5fdbc0941ad37909789f155f3d580ceb55335fc57e33628f1383d3db23de2f75</t>
         </is>
       </c>
     </row>
@@ -19518,7 +19522,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr">
@@ -19646,7 +19650,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19714,7 +19718,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19782,7 +19786,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19850,7 +19854,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr">
@@ -19922,7 +19926,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
@@ -19994,7 +19998,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20062,7 +20066,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20130,7 +20134,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20198,12 +20202,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20218,7 +20222,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>a74f2430b67ce7fba5025f7cd3749aeb9fae367edb80b85543e8b5388ba290aa</t>
+          <t>4e485c638b005f9fd42d1223f09bf21bf9154d71ef6e1ebaebf0c7657cdf15bb</t>
         </is>
       </c>
     </row>
@@ -20386,7 +20390,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
@@ -20458,7 +20462,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20526,7 +20530,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr">
@@ -20598,7 +20602,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20666,7 +20670,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20734,7 +20738,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20802,7 +20806,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20870,7 +20874,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20938,7 +20942,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -21006,7 +21010,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21070,7 +21074,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21130,7 +21134,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21202,7 +21206,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21266,7 +21270,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21338,7 +21342,7 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
@@ -21406,7 +21410,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr">
@@ -21478,7 +21482,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21538,7 +21542,7 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr"/>
@@ -21602,7 +21606,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
@@ -21666,7 +21670,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21734,7 +21738,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr">
@@ -21754,7 +21758,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>af9261098e89ea7c32af249b66204dd0966bcaf94a3862b9471a1b5a2ef76441</t>
+          <t>d2479ab9a508b24937d3e3e6b1ee1b58965ae1a2f2a172a0c0945f68712b9747</t>
         </is>
       </c>
     </row>
@@ -21806,7 +21810,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr">
@@ -21826,7 +21830,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>48987afc9d2a618b5b41a8ac1364e9673f19a6b8d8739b2b35b6e89f11a12c5d</t>
+          <t>f17837075b6cd3332572234e587e919d400a8d55980277a4382ace1fe382747a</t>
         </is>
       </c>
     </row>
@@ -21878,7 +21882,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21950,7 +21954,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -22078,7 +22082,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22555,7 +22559,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22597,7 +22601,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22631,7 +22635,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22673,7 +22677,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22711,7 +22715,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22749,7 +22753,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22787,7 +22791,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22825,7 +22829,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22863,7 +22867,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22905,7 +22909,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22943,7 +22947,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22985,7 +22989,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -23027,7 +23031,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23069,7 +23073,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23116,7 +23120,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -23153,7 +23157,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23195,7 +23199,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23237,7 +23241,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23279,7 +23283,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23321,7 +23325,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23363,7 +23367,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23405,7 +23409,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23447,7 +23451,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23489,7 +23493,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23527,7 +23531,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23569,7 +23573,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23607,7 +23611,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23649,7 +23653,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23691,7 +23695,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23775,7 +23779,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23817,7 +23821,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23855,7 +23859,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23893,7 +23897,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23931,7 +23935,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23973,7 +23977,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -24015,7 +24019,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24053,7 +24057,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24091,7 +24095,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24133,7 +24137,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24175,7 +24179,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24209,7 +24213,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24251,7 +24255,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24289,7 +24293,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24327,7 +24331,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24369,7 +24373,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24407,7 +24411,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24445,7 +24449,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24483,7 +24487,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24525,7 +24529,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24563,7 +24567,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24605,7 +24609,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24647,7 +24651,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24685,7 +24689,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24727,7 +24731,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24769,7 +24773,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24807,7 +24811,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24845,7 +24849,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24887,7 +24891,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24925,7 +24929,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24967,7 +24971,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -25009,7 +25013,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -25047,7 +25051,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25089,7 +25093,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25131,7 +25135,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25169,7 +25173,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25211,7 +25215,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25249,7 +25253,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25291,7 +25295,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25333,7 +25337,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25375,7 +25379,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25413,7 +25417,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25451,7 +25455,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25489,7 +25493,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25527,7 +25531,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25565,7 +25569,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25607,7 +25611,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25645,7 +25649,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25683,7 +25687,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25725,7 +25729,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25763,7 +25767,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25805,7 +25809,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25843,7 +25847,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25885,7 +25889,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25923,7 +25927,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25961,7 +25965,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -26003,7 +26007,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26463,7 +26467,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26505,7 +26509,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26547,7 +26551,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26589,7 +26593,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26631,7 +26635,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26673,7 +26677,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26715,7 +26719,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26757,7 +26761,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26799,7 +26803,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26841,7 +26845,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26883,7 +26887,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26925,7 +26929,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26967,7 +26971,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -27009,7 +27013,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27051,7 +27055,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27093,7 +27097,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27135,7 +27139,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27177,7 +27181,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27219,7 +27223,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27261,7 +27265,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27303,7 +27307,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27345,7 +27349,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27387,7 +27391,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27429,7 +27433,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27471,7 +27475,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27513,7 +27517,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27555,7 +27559,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27597,7 +27601,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27639,7 +27643,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27681,7 +27685,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27723,7 +27727,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27807,7 +27811,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27849,7 +27853,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27891,7 +27895,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27933,7 +27937,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27975,7 +27979,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -28017,7 +28021,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28055,7 +28059,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28097,7 +28101,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28139,7 +28143,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28181,7 +28185,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28223,7 +28227,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28265,7 +28269,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28307,7 +28311,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28349,7 +28353,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28391,7 +28395,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28433,7 +28437,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28475,7 +28479,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28517,7 +28521,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28559,7 +28563,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28601,7 +28605,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28643,7 +28647,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28685,7 +28689,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28727,7 +28731,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28769,12 +28773,12 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
@@ -28811,7 +28815,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28853,7 +28857,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28895,7 +28899,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28937,7 +28941,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28979,7 +28983,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -29021,7 +29025,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29063,7 +29067,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29105,7 +29109,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29147,7 +29151,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29189,7 +29193,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29231,7 +29235,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29273,7 +29277,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29315,7 +29319,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29357,7 +29361,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29399,7 +29403,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29441,7 +29445,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29483,7 +29487,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29525,7 +29529,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29567,7 +29571,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29609,7 +29613,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29651,7 +29655,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29693,7 +29697,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29740,7 +29744,7 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H178" s="2" t="inlineStr">
@@ -29777,7 +29781,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29819,7 +29823,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29861,7 +29865,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29903,7 +29907,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29945,7 +29949,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29987,7 +29991,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -30029,7 +30033,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30071,7 +30075,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30113,7 +30117,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30155,7 +30159,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30197,7 +30201,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30239,7 +30243,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30281,7 +30285,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30323,7 +30327,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30365,7 +30369,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30407,7 +30411,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30449,7 +30453,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30491,7 +30495,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30533,7 +30537,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30575,7 +30579,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30617,7 +30621,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30659,7 +30663,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30701,7 +30705,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -30743,7 +30747,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30785,7 +30789,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30827,7 +30831,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30869,7 +30873,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -30911,7 +30915,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30995,7 +30999,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -31037,7 +31041,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31079,7 +31083,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31126,7 +31130,7 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr">
@@ -31163,7 +31167,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31205,7 +31209,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31247,7 +31251,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31289,7 +31293,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31331,7 +31335,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31373,7 +31377,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31415,7 +31419,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31457,7 +31461,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31499,7 +31503,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31541,7 +31545,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31583,7 +31587,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31625,7 +31629,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31667,7 +31671,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31709,7 +31713,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31751,7 +31755,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31793,7 +31797,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31835,7 +31839,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31877,7 +31881,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31919,7 +31923,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31961,7 +31965,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -32003,7 +32007,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -32045,7 +32049,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32087,7 +32091,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32129,7 +32133,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32171,7 +32175,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32213,7 +32217,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32255,7 +32259,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32297,7 +32301,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32339,7 +32343,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32381,7 +32385,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32423,7 +32427,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32465,7 +32469,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32507,7 +32511,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32549,7 +32553,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32587,7 +32591,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32629,7 +32633,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32667,7 +32671,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32701,7 +32705,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32743,7 +32747,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32781,7 +32785,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32823,7 +32827,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32865,7 +32869,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32903,7 +32907,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32941,7 +32945,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32979,7 +32983,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -33017,7 +33021,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -33059,7 +33063,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33097,7 +33101,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33131,7 +33135,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33169,7 +33173,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33207,7 +33211,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33245,7 +33249,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33287,7 +33291,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33329,7 +33333,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33367,7 +33371,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33409,7 +33413,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33443,7 +33447,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33481,7 +33485,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">
@@ -33519,7 +33523,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -33557,7 +33561,7 @@
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-29T14:26:50+00:00</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-30 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7042,7 +7042,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8090,12 +8090,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>03badc26d23332eddcede7a6268a106f56f04f08c2035bd0c52f7ace892c8828</t>
+          <t>29aa8ba63351c70d3128b49fc86c53835f995f3314d1d982085d8d53344113d7</t>
         </is>
       </c>
     </row>
@@ -8158,12 +8158,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>178ebd8f760edfbb4d15364b0a47e22f57fb0cba6c36107801788cbc03178169</t>
+          <t>c4b83f4a527a0536b4aba8fe75af68b403c126fefac9f77ae5ff060670ecd119</t>
         </is>
       </c>
     </row>
@@ -8226,7 +8226,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8694,7 +8694,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8766,7 +8766,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8894,7 +8894,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10730,10 +10730,14 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
-        </is>
-      </c>
-      <c r="K188" s="2" t="inlineStr"/>
+          <t>2026-10-30T14:18:21+00:00</t>
+        </is>
+      </c>
+      <c r="K188" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30T14:18:21+00:00</t>
+        </is>
+      </c>
       <c r="L188" s="2" t="inlineStr">
         <is>
           <t>2026-09-06</t>
@@ -10746,7 +10750,7 @@
       </c>
       <c r="N188" s="2" t="inlineStr">
         <is>
-          <t>3124fc1887303e571edec4a48ff382f81bc987eee7f99c2c2a097ba5bbc79ba4</t>
+          <t>d3927702d2f17dd33b7ce51569545313f21325ab845e3fd4c9f11b7e1f582841</t>
         </is>
       </c>
     </row>
@@ -10910,7 +10914,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10978,7 +10982,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11050,12 +11054,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11070,7 +11074,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>cb6adaab7878572b60a4a8aae6c9bcd601a4e59bda9e47559103adfcd0724b07</t>
+          <t>9e47a91c0d02bc3a7bf6a09842aaeb276a72799461c423baa98728be144d382d</t>
         </is>
       </c>
     </row>
@@ -11122,7 +11126,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11194,7 +11198,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11214,7 +11218,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>7856641f8326bdd8b90a856d2361d918eb5c404d78e2d63f06c2b8a8f3b57bac</t>
+          <t>b3a7b5eef98aea72336e8049c2e915c58b9e298f24cfe4e08a2c5d8f4c0c14dc</t>
         </is>
       </c>
     </row>
@@ -11266,7 +11270,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11338,7 +11342,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11410,7 +11414,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11478,7 +11482,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11550,7 +11554,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11622,7 +11626,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11694,7 +11698,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11762,12 +11766,12 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L203" s="2" t="inlineStr">
@@ -11782,7 +11786,7 @@
       </c>
       <c r="N203" s="2" t="inlineStr">
         <is>
-          <t>806c4f3862ff5b209744ae0740c467cdcbdf8a3a657c768114eb1417e26ead33</t>
+          <t>eb257a214686fc575ab4ae8466458a265ea20ee07e69bd05127ec84deb8f1863</t>
         </is>
       </c>
     </row>
@@ -11834,7 +11838,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11906,7 +11910,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12038,7 +12042,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12058,7 +12062,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>b8b0809430253e08f5237a8befd2537454a10d56d9f2ff70cbd1221d28e886f3</t>
+          <t>d9429ee44a65c1c084d33f4a7eb0abca1088557980e0d275d23636bbedce2a78</t>
         </is>
       </c>
     </row>
@@ -12110,7 +12114,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr">
@@ -12182,7 +12186,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12254,7 +12258,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12550,7 +12554,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr">
@@ -12802,7 +12806,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12874,7 +12878,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
@@ -12946,7 +12950,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13138,7 +13142,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
@@ -13210,7 +13214,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
@@ -13282,7 +13286,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13298,7 +13302,7 @@
       </c>
       <c r="N226" s="2" t="inlineStr">
         <is>
-          <t>81a8cc3894d31d1c48ec96e11198fcb9bc26f93e549242b13ab98d9048060022</t>
+          <t>8be740f8b0db7138ad012021690ac0bbe154447e196130326bc4324193cf4b02</t>
         </is>
       </c>
     </row>
@@ -13350,7 +13354,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13418,7 +13422,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr">
@@ -13490,7 +13494,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13614,7 +13618,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13634,7 +13638,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>a55a21f9c39028df1294608bfa4eea59bcb8dbf9cd3fc8ac33b197e038e27e34</t>
+          <t>10187e2645e74fa6a90a91f3625421ff2226d62b8e099abef1c61079bc7d39e6</t>
         </is>
       </c>
     </row>
@@ -13926,7 +13930,7 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
@@ -13946,7 +13950,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>c215cec8a9a3dd27da11e5e0a2ca791929570af6b530d22ef0f3f0f396d226c1</t>
+          <t>36b31a1bd169fa9113fae02c81edebdb03fab441a0bf7f5225528a0e631b5016</t>
         </is>
       </c>
     </row>
@@ -18198,7 +18202,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18270,7 +18274,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
@@ -18290,7 +18294,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>501483015645273acb71f5c24f1b7a293ba100e50c72e890b1ade6d9e5e38a8c</t>
+          <t>d0cb4d634dc4a4074c1a3223444aa0ac73139127ec8173f41209867262bc9518</t>
         </is>
       </c>
     </row>
@@ -18342,7 +18346,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18414,7 +18418,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18482,7 +18486,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18550,7 +18554,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18674,7 +18678,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19102,7 +19106,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19170,7 +19174,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19238,7 +19242,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19306,12 +19310,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19326,7 +19330,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>c3f025bb73b38c43041e86e2f2f9ec3d376b1b4cee2171b25dce0f67f984de81</t>
+          <t>094d60c2f2d91adab4bd5a24a4c8887a2d7eef6377cda0a6414a6a34491595da</t>
         </is>
       </c>
     </row>
@@ -19378,12 +19382,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19398,7 +19402,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>b230bdfa36da8b0649a4122b46e5a2605c9e992087229932fb9517617b7fae12</t>
+          <t>8f672a740539545631b6777adeb40e522564d65b619f6f071cd8e4bf0093c3da</t>
         </is>
       </c>
     </row>
@@ -19450,12 +19454,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19470,7 +19474,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>5fdbc0941ad37909789f155f3d580ceb55335fc57e33628f1383d3db23de2f75</t>
+          <t>0c5c14f30a47ec829ae8873cb4a59a8eb00847a3603090389040a1ea7bf76f64</t>
         </is>
       </c>
     </row>
@@ -19522,7 +19526,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr">
@@ -19650,7 +19654,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19718,7 +19722,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19786,7 +19790,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19854,12 +19858,12 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L337" s="2" t="inlineStr">
@@ -19874,7 +19878,7 @@
       </c>
       <c r="N337" s="2" t="inlineStr">
         <is>
-          <t>45f62bb98d58760c3c08ad7c5646813fbc454b8f4168d36e44ea545b8a115edc</t>
+          <t>90af8db1f07270d3533224010d8754c48135c686326275d5420f4ca2999aa599</t>
         </is>
       </c>
     </row>
@@ -19926,7 +19930,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
@@ -19998,7 +20002,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20066,7 +20070,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20134,7 +20138,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20202,12 +20206,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20222,7 +20226,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>4e485c638b005f9fd42d1223f09bf21bf9154d71ef6e1ebaebf0c7657cdf15bb</t>
+          <t>f7e305ef5570a9ed6583ce21701363c1a89a20af557324ba852b4eddcbffa04c</t>
         </is>
       </c>
     </row>
@@ -20390,7 +20394,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
@@ -20462,7 +20466,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20530,7 +20534,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr">
@@ -20602,7 +20606,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20670,7 +20674,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20738,7 +20742,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20806,7 +20810,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20874,7 +20878,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20942,7 +20946,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -21010,7 +21014,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21074,7 +21078,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21134,7 +21138,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21206,7 +21210,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21270,7 +21274,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21342,12 +21346,12 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
@@ -21362,7 +21366,7 @@
       </c>
       <c r="N359" s="2" t="inlineStr">
         <is>
-          <t>d6885681a201a6d997c84c467335622ed9421af02f6710c63beceecf221a9f30</t>
+          <t>7f22cc067a9b150fc82602b44cf1d952fae7e4d66b013cdbe69b83a14239654e</t>
         </is>
       </c>
     </row>
@@ -21410,7 +21414,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr">
@@ -21482,7 +21486,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21542,10 +21546,14 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
-        </is>
-      </c>
-      <c r="K362" s="2" t="inlineStr"/>
+          <t>2026-10-30T14:18:21+00:00</t>
+        </is>
+      </c>
+      <c r="K362" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30T14:18:21+00:00</t>
+        </is>
+      </c>
       <c r="L362" s="2" t="inlineStr">
         <is>
           <t>2026-10-12</t>
@@ -21558,7 +21566,7 @@
       </c>
       <c r="N362" s="2" t="inlineStr">
         <is>
-          <t>38335dbc5776bfd9f31db210baa2292f7f13d03cfca5b3d2260489a02c87ded9</t>
+          <t>67adbe5d49d0a8401d9f84b27f1ad05c3ff4341dc5b787b555f7ae45bab8e446</t>
         </is>
       </c>
     </row>
@@ -21606,12 +21614,12 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="L363" s="2" t="inlineStr">
@@ -21626,7 +21634,7 @@
       </c>
       <c r="N363" s="2" t="inlineStr">
         <is>
-          <t>7ec3db99e6ad6f11d8c2ced072aaf23b7fbbeb405b4db04385e71dcf5864d5dd</t>
+          <t>5835651e6f3855dd70cc765d964ebe48165c31a76d791d120e1520e494a35f2b</t>
         </is>
       </c>
     </row>
@@ -21670,7 +21678,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21738,7 +21746,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr">
@@ -21758,7 +21766,7 @@
       </c>
       <c r="N365" s="2" t="inlineStr">
         <is>
-          <t>d2479ab9a508b24937d3e3e6b1ee1b58965ae1a2f2a172a0c0945f68712b9747</t>
+          <t>2bcaf2437099b8c982594abbd0cf554ba6142f4bc4f6a7531076188e650998c9</t>
         </is>
       </c>
     </row>
@@ -21810,7 +21818,7 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr">
@@ -21830,7 +21838,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>f17837075b6cd3332572234e587e919d400a8d55980277a4382ace1fe382747a</t>
+          <t>3c194867f74d55c41aa2262384a81c262b93ced4b40d2b2e6ff6724453e697be</t>
         </is>
       </c>
     </row>
@@ -21882,7 +21890,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21954,7 +21962,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -22082,7 +22090,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22559,7 +22567,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22601,7 +22609,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22635,7 +22643,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22677,7 +22685,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22715,7 +22723,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22753,7 +22761,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22791,7 +22799,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22829,7 +22837,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22867,7 +22875,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22909,7 +22917,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22947,7 +22955,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22989,7 +22997,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -23031,7 +23039,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23073,7 +23081,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23157,7 +23165,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23199,7 +23207,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23241,7 +23249,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23283,7 +23291,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23325,7 +23333,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23367,7 +23375,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23409,7 +23417,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23451,7 +23459,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23493,7 +23501,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23531,7 +23539,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23573,7 +23581,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23611,7 +23619,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23653,7 +23661,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23695,7 +23703,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23742,7 +23750,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -23779,7 +23787,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23821,7 +23829,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23859,7 +23867,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23897,7 +23905,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23935,7 +23943,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23977,7 +23985,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -24019,7 +24027,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24057,7 +24065,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24095,7 +24103,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24137,7 +24145,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24179,7 +24187,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24213,7 +24221,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24255,7 +24263,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24293,7 +24301,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24331,7 +24339,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24373,7 +24381,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24411,7 +24419,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24449,7 +24457,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24487,7 +24495,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24529,7 +24537,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24567,7 +24575,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24609,7 +24617,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24651,7 +24659,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24689,7 +24697,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24731,7 +24739,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24773,7 +24781,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24811,7 +24819,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24849,7 +24857,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24891,7 +24899,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24929,7 +24937,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24971,7 +24979,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -25013,7 +25021,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -25051,7 +25059,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25093,7 +25101,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25135,7 +25143,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25173,7 +25181,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25215,7 +25223,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25253,7 +25261,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25295,7 +25303,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25337,7 +25345,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25379,7 +25387,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25417,7 +25425,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25455,7 +25463,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25493,7 +25501,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25531,7 +25539,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25569,7 +25577,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25611,7 +25619,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25649,7 +25657,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25687,7 +25695,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25729,7 +25737,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25767,7 +25775,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25809,7 +25817,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25847,7 +25855,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25889,7 +25897,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25927,7 +25935,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25965,7 +25973,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -26007,7 +26015,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26467,7 +26475,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26509,7 +26517,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26551,7 +26559,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26593,7 +26601,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26635,7 +26643,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26677,7 +26685,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26719,7 +26727,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26761,7 +26769,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26803,7 +26811,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26845,7 +26853,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26887,7 +26895,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26929,7 +26937,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26971,7 +26979,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -27013,7 +27021,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27055,7 +27063,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27097,7 +27105,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27139,7 +27147,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27181,7 +27189,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27223,7 +27231,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27265,7 +27273,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27307,7 +27315,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27349,7 +27357,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27391,7 +27399,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27433,7 +27441,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27475,7 +27483,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27517,7 +27525,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27559,7 +27567,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27601,7 +27609,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27643,7 +27651,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27685,7 +27693,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27727,7 +27735,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27811,7 +27819,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27853,7 +27861,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27895,7 +27903,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27937,7 +27945,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27979,7 +27987,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -28021,7 +28029,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28059,7 +28067,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28101,7 +28109,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28143,7 +28151,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28185,7 +28193,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28227,7 +28235,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28269,7 +28277,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28311,7 +28319,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28353,7 +28361,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28395,7 +28403,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28437,7 +28445,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28479,7 +28487,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28521,7 +28529,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28563,7 +28571,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28605,7 +28613,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28647,7 +28655,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28689,7 +28697,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28731,7 +28739,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28773,7 +28781,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28815,7 +28823,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28857,7 +28865,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28899,7 +28907,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28941,7 +28949,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28983,7 +28991,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -29025,7 +29033,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29067,7 +29075,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29109,7 +29117,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29151,7 +29159,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29193,7 +29201,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29235,7 +29243,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29277,7 +29285,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29319,7 +29327,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29361,7 +29369,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29403,7 +29411,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29445,7 +29453,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29487,7 +29495,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29529,7 +29537,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29571,7 +29579,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29613,7 +29621,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29655,7 +29663,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29697,7 +29705,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29744,7 +29752,7 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H178" s="2" t="inlineStr">
@@ -29781,7 +29789,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29823,7 +29831,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29865,7 +29873,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29907,7 +29915,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29949,7 +29957,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29991,7 +29999,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -30033,7 +30041,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30075,7 +30083,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30117,7 +30125,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30159,7 +30167,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30201,7 +30209,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30243,7 +30251,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30285,7 +30293,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30327,7 +30335,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30369,7 +30377,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30411,7 +30419,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30453,7 +30461,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30495,7 +30503,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30537,7 +30545,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30579,7 +30587,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30621,7 +30629,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30663,7 +30671,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30710,7 +30718,7 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr">
@@ -30747,7 +30755,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30789,7 +30797,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30831,7 +30839,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30873,7 +30881,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -30915,7 +30923,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30999,7 +31007,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -31041,7 +31049,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31083,7 +31091,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31125,12 +31133,12 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:21:26+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr">
@@ -31167,7 +31175,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31209,7 +31217,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31251,7 +31259,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31293,7 +31301,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31335,7 +31343,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31377,7 +31385,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31419,7 +31427,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31461,7 +31469,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31503,7 +31511,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31545,7 +31553,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31587,7 +31595,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31629,7 +31637,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31671,7 +31679,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31713,7 +31721,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31755,7 +31763,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31797,7 +31805,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31839,7 +31847,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31881,7 +31889,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31923,7 +31931,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31965,7 +31973,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -32007,7 +32015,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -32049,7 +32057,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -32091,7 +32099,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32133,7 +32141,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32175,7 +32183,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32217,7 +32225,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32259,7 +32267,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32301,7 +32309,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32343,7 +32351,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32385,7 +32393,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32427,7 +32435,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32469,7 +32477,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32511,7 +32519,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32553,7 +32561,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32591,7 +32599,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32633,7 +32641,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32671,7 +32679,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32705,7 +32713,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32747,7 +32755,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32785,7 +32793,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32827,7 +32835,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32869,7 +32877,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32907,7 +32915,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32945,7 +32953,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32983,7 +32991,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -33021,7 +33029,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -33063,7 +33071,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33101,7 +33109,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33135,7 +33143,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33173,7 +33181,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33211,7 +33219,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33249,7 +33257,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33291,7 +33299,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33333,7 +33341,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33371,7 +33379,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33413,7 +33421,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33447,7 +33455,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33485,7 +33493,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">
@@ -33523,7 +33531,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -33561,7 +33569,7 @@
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:26:50+00:00</t>
+          <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-31 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -4438,7 +4438,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6822,7 +6822,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7042,7 +7042,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8090,12 +8090,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>29aa8ba63351c70d3128b49fc86c53835f995f3314d1d982085d8d53344113d7</t>
+          <t>16530dddcfdbff9983593de1292f82a1a1c416e495561142317fe29f3b900741</t>
         </is>
       </c>
     </row>
@@ -8158,7 +8158,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8226,7 +8226,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8694,7 +8694,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8766,7 +8766,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8894,7 +8894,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr">
@@ -10914,7 +10914,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10982,7 +10982,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11054,12 +11054,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>9e47a91c0d02bc3a7bf6a09842aaeb276a72799461c423baa98728be144d382d</t>
+          <t>c2b08f58b3f6dc4e15db00ed73546be7db417e03c52abecd43190f8cbfc97c2f</t>
         </is>
       </c>
     </row>
@@ -11126,7 +11126,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>0b27eab5cd95f98e30b49b2e885b954039e0948f2a1e4e57f399e6f4bdfa9ac3</t>
+          <t>cc90100297aaa424969f5887fad8c946215ff942e513fb9da3277ef17c4e46f7</t>
         </is>
       </c>
     </row>
@@ -11198,7 +11198,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11270,7 +11270,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11342,7 +11342,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11414,7 +11414,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11482,7 +11482,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr">
@@ -11554,7 +11554,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr">
@@ -11626,7 +11626,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>d97c5d2cdead707e1eb4f0b0de08498e8de550425fbaea21dd19993937be60aa</t>
+          <t>380bd977f4a44274a8557c0bccba1af34c7a0bf55e8c77f3ca9d3c220eae7353</t>
         </is>
       </c>
     </row>
@@ -11698,7 +11698,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11766,7 +11766,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11838,7 +11838,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11910,7 +11910,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12042,7 +12042,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12062,7 +12062,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>d9429ee44a65c1c084d33f4a7eb0abca1088557980e0d275d23636bbedce2a78</t>
+          <t>b8b0809430253e08f5237a8befd2537454a10d56d9f2ff70cbd1221d28e886f3</t>
         </is>
       </c>
     </row>
@@ -12114,7 +12114,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr">
@@ -12186,7 +12186,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12258,7 +12258,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12554,7 +12554,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr">
@@ -12878,7 +12878,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr">
@@ -12950,7 +12950,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13142,7 +13142,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr">
@@ -13214,7 +13214,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13354,7 +13354,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13422,7 +13422,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr">
@@ -13494,7 +13494,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13618,7 +13618,7 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K231" s="2" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>10187e2645e74fa6a90a91f3625421ff2226d62b8e099abef1c61079bc7d39e6</t>
+          <t>0dbd8d6f9d24151e4bbd9e79b809f9b97a33d5ba0ab4cf2d7bddc887361154ad</t>
         </is>
       </c>
     </row>
@@ -13930,12 +13930,12 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T12:15:32+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="L236" s="2" t="inlineStr">
@@ -13950,7 +13950,7 @@
       </c>
       <c r="N236" s="2" t="inlineStr">
         <is>
-          <t>36b31a1bd169fa9113fae02c81edebdb03fab441a0bf7f5225528a0e631b5016</t>
+          <t>d3b00c1ee345b9c0791a959af6bb3c1b26de3c883b5961b88fe9610063ff91ae</t>
         </is>
       </c>
     </row>
@@ -18202,7 +18202,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18274,7 +18274,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr">
@@ -18294,7 +18294,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>d0cb4d634dc4a4074c1a3223444aa0ac73139127ec8173f41209867262bc9518</t>
+          <t>b0d5efd5ac3ad526696e229e71f1ecf5c20fcebe74c85d09923f5abede5cc75d</t>
         </is>
       </c>
     </row>
@@ -18346,7 +18346,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18418,7 +18418,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18486,7 +18486,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18554,7 +18554,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18678,7 +18678,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19106,7 +19106,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19174,7 +19174,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19242,7 +19242,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19310,12 +19310,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19330,7 +19330,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>094d60c2f2d91adab4bd5a24a4c8887a2d7eef6377cda0a6414a6a34491595da</t>
+          <t>bcdc19862c8f34945bc8a7fd2c3b2f43c611d7b53ba099f43d055fd9d052e866</t>
         </is>
       </c>
     </row>
@@ -19382,14 +19382,14 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
+          <t>2026-10-31T13:50:35+00:00</t>
+        </is>
+      </c>
+      <c r="K330" s="2" t="inlineStr">
+        <is>
           <t>2026-10-30T14:18:21+00:00</t>
         </is>
       </c>
-      <c r="K330" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-30T14:18:21+00:00</t>
-        </is>
-      </c>
       <c r="L330" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -19402,7 +19402,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>8f672a740539545631b6777adeb40e522564d65b619f6f071cd8e4bf0093c3da</t>
+          <t>bb9a617c19534fbe4933632469d9c3893c96a541ae1c8119685c1058def4ce22</t>
         </is>
       </c>
     </row>
@@ -19454,12 +19454,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19474,7 +19474,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>0c5c14f30a47ec829ae8873cb4a59a8eb00847a3603090389040a1ea7bf76f64</t>
+          <t>c1e0e051aa9a3fcb8dbe35e2db1c623443444cd9adb1bfd949fe81532e39fa60</t>
         </is>
       </c>
     </row>
@@ -19526,7 +19526,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr">
@@ -19654,7 +19654,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19722,7 +19722,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19790,7 +19790,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19858,7 +19858,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr">
@@ -19930,7 +19930,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr">
@@ -20002,7 +20002,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -20070,7 +20070,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20138,7 +20138,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20206,12 +20206,12 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -20226,7 +20226,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>f7e305ef5570a9ed6583ce21701363c1a89a20af557324ba852b4eddcbffa04c</t>
+          <t>4fce2fb029a4fdf591ad472b379f8041049b39fb25ae15bc6e56c92dbe15d432</t>
         </is>
       </c>
     </row>
@@ -20394,7 +20394,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr">
@@ -20466,7 +20466,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20534,7 +20534,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr">
@@ -20606,7 +20606,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20674,7 +20674,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20742,7 +20742,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20810,7 +20810,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20878,7 +20878,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -20946,7 +20946,7 @@
       </c>
       <c r="J353" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K353" s="2" t="inlineStr"/>
@@ -21014,7 +21014,7 @@
       </c>
       <c r="J354" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K354" s="2" t="inlineStr">
@@ -21078,7 +21078,7 @@
       </c>
       <c r="J355" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K355" s="2" t="inlineStr"/>
@@ -21138,7 +21138,7 @@
       </c>
       <c r="J356" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K356" s="2" t="inlineStr">
@@ -21210,7 +21210,7 @@
       </c>
       <c r="J357" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K357" s="2" t="inlineStr">
@@ -21274,7 +21274,7 @@
       </c>
       <c r="J358" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K358" s="2" t="inlineStr">
@@ -21346,12 +21346,12 @@
       </c>
       <c r="J359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K359" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
@@ -21366,7 +21366,7 @@
       </c>
       <c r="N359" s="2" t="inlineStr">
         <is>
-          <t>7f22cc067a9b150fc82602b44cf1d952fae7e4d66b013cdbe69b83a14239654e</t>
+          <t>60e9674292b80b5b4b50a854c4c091e1ad146b3d4cc4cbd121fecfb40a014e37</t>
         </is>
       </c>
     </row>
@@ -21414,7 +21414,7 @@
       </c>
       <c r="J360" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K360" s="2" t="inlineStr">
@@ -21486,7 +21486,7 @@
       </c>
       <c r="J361" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K361" s="2" t="inlineStr"/>
@@ -21546,12 +21546,12 @@
       </c>
       <c r="J362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K362" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="L362" s="2" t="inlineStr">
@@ -21566,7 +21566,7 @@
       </c>
       <c r="N362" s="2" t="inlineStr">
         <is>
-          <t>67adbe5d49d0a8401d9f84b27f1ad05c3ff4341dc5b787b555f7ae45bab8e446</t>
+          <t>38335dbc5776bfd9f31db210baa2292f7f13d03cfca5b3d2260489a02c87ded9</t>
         </is>
       </c>
     </row>
@@ -21614,7 +21614,7 @@
       </c>
       <c r="J363" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K363" s="2" t="inlineStr">
@@ -21678,7 +21678,7 @@
       </c>
       <c r="J364" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K364" s="2" t="inlineStr"/>
@@ -21746,7 +21746,7 @@
       </c>
       <c r="J365" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K365" s="2" t="inlineStr">
@@ -21818,12 +21818,12 @@
       </c>
       <c r="J366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K366" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T13:29:58+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="L366" s="2" t="inlineStr">
@@ -21838,7 +21838,7 @@
       </c>
       <c r="N366" s="2" t="inlineStr">
         <is>
-          <t>3c194867f74d55c41aa2262384a81c262b93ced4b40d2b2e6ff6724453e697be</t>
+          <t>94a6656e92f89188621dfe13ca9bf05cff68c855fe69fd2068ce016b040550f2</t>
         </is>
       </c>
     </row>
@@ -21890,7 +21890,7 @@
       </c>
       <c r="J367" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K367" s="2" t="inlineStr">
@@ -21962,7 +21962,7 @@
       </c>
       <c r="J368" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K368" s="2" t="inlineStr"/>
@@ -22090,7 +22090,7 @@
       </c>
       <c r="J370" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="K370" s="2" t="inlineStr"/>
@@ -22567,7 +22567,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -22609,7 +22609,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -22643,7 +22643,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -22685,7 +22685,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -22723,7 +22723,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -22761,7 +22761,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -22799,7 +22799,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -22837,7 +22837,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -22875,7 +22875,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -22917,7 +22917,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -22955,7 +22955,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -22997,7 +22997,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -23039,7 +23039,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -23081,7 +23081,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -23165,7 +23165,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -23207,7 +23207,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -23249,7 +23249,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -23291,7 +23291,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -23333,7 +23333,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -23375,7 +23375,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -23417,7 +23417,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -23459,7 +23459,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -23501,7 +23501,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -23539,7 +23539,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -23581,7 +23581,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -23619,7 +23619,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -23661,7 +23661,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -23703,7 +23703,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -23787,7 +23787,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -23829,7 +23829,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -23867,7 +23867,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -23905,7 +23905,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -23943,7 +23943,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -23985,7 +23985,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -24027,7 +24027,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -24065,7 +24065,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -24103,7 +24103,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -24145,7 +24145,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -24187,7 +24187,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -24221,7 +24221,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -24263,7 +24263,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -24301,7 +24301,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -24339,7 +24339,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -24381,7 +24381,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -24419,7 +24419,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -24457,7 +24457,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -24495,7 +24495,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -24537,7 +24537,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -24575,7 +24575,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -24617,7 +24617,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -24659,7 +24659,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -24697,7 +24697,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -24739,7 +24739,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -24781,7 +24781,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -24819,7 +24819,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -24857,7 +24857,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -24899,7 +24899,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -24937,7 +24937,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -24979,7 +24979,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -25021,7 +25021,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -25059,7 +25059,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -25101,7 +25101,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -25143,7 +25143,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -25181,7 +25181,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -25223,7 +25223,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -25261,7 +25261,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -25303,7 +25303,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -25345,7 +25345,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -25387,7 +25387,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -25425,7 +25425,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -25463,7 +25463,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -25501,7 +25501,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -25539,7 +25539,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -25577,7 +25577,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -25619,7 +25619,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -25657,7 +25657,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -25695,7 +25695,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -25737,7 +25737,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -25775,7 +25775,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -25817,7 +25817,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -25855,7 +25855,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -25897,7 +25897,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -25935,7 +25935,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -25973,7 +25973,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -26015,7 +26015,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -26475,7 +26475,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -26517,7 +26517,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -26559,7 +26559,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -26601,7 +26601,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -26643,7 +26643,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -26727,7 +26727,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -26769,7 +26769,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -26811,7 +26811,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -26853,7 +26853,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -26895,7 +26895,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -26937,7 +26937,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -26979,7 +26979,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -27021,7 +27021,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -27063,7 +27063,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -27105,7 +27105,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -27147,7 +27147,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -27189,7 +27189,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -27231,7 +27231,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -27273,7 +27273,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -27315,7 +27315,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -27357,7 +27357,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -27399,7 +27399,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -27441,7 +27441,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -27525,7 +27525,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -27567,7 +27567,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -27609,7 +27609,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -27651,7 +27651,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -27693,7 +27693,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -27735,7 +27735,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -27782,7 +27782,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -27819,7 +27819,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -27861,7 +27861,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -27903,7 +27903,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -27945,7 +27945,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -27987,7 +27987,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -28029,7 +28029,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -28067,7 +28067,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -28109,7 +28109,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -28151,7 +28151,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -28193,7 +28193,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -28235,7 +28235,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -28277,7 +28277,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -28319,7 +28319,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -28361,7 +28361,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -28403,7 +28403,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -28445,7 +28445,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -28487,7 +28487,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -28529,7 +28529,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -28571,7 +28571,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -28613,7 +28613,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -28655,7 +28655,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -28697,7 +28697,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -28739,7 +28739,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -28781,7 +28781,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -28823,7 +28823,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -28865,7 +28865,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -28907,7 +28907,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -28949,7 +28949,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -28991,7 +28991,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -29033,7 +29033,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -29075,7 +29075,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -29117,7 +29117,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -29159,7 +29159,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -29201,7 +29201,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -29243,7 +29243,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -29285,7 +29285,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -29327,7 +29327,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -29369,7 +29369,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -29411,7 +29411,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -29453,7 +29453,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -29495,7 +29495,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -29537,7 +29537,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -29579,7 +29579,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -29621,7 +29621,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -29663,7 +29663,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -29705,7 +29705,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -29752,7 +29752,7 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H178" s="2" t="inlineStr">
@@ -29789,7 +29789,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -29831,7 +29831,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -29873,7 +29873,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -29915,7 +29915,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -29957,7 +29957,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -29999,7 +29999,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -30041,7 +30041,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -30083,7 +30083,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -30125,7 +30125,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -30167,7 +30167,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -30209,7 +30209,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -30251,7 +30251,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -30293,7 +30293,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -30335,7 +30335,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -30377,7 +30377,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -30419,7 +30419,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -30461,7 +30461,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -30503,7 +30503,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -30545,7 +30545,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -30587,7 +30587,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -30629,7 +30629,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -30671,7 +30671,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -30718,7 +30718,7 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H201" s="2" t="inlineStr">
@@ -30755,7 +30755,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -30797,7 +30797,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -30839,7 +30839,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -30881,7 +30881,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -30923,7 +30923,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -30970,7 +30970,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
@@ -31007,7 +31007,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -31049,7 +31049,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -31091,7 +31091,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -31133,7 +31133,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -31175,7 +31175,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -31217,7 +31217,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -31259,7 +31259,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -31301,7 +31301,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -31343,7 +31343,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -31385,7 +31385,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -31427,7 +31427,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -31469,7 +31469,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -31511,7 +31511,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -31553,7 +31553,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -31595,7 +31595,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -31637,7 +31637,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -31679,7 +31679,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -31721,7 +31721,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -31763,7 +31763,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -31805,7 +31805,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -31847,7 +31847,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -31889,7 +31889,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -31931,7 +31931,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -31973,7 +31973,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -32015,7 +32015,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -32062,7 +32062,7 @@
       </c>
       <c r="G233" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H233" s="2" t="inlineStr">
@@ -32099,7 +32099,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -32141,7 +32141,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -32183,7 +32183,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -32225,7 +32225,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -32267,7 +32267,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -32309,7 +32309,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -32351,7 +32351,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -32393,7 +32393,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -32435,7 +32435,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -32477,7 +32477,7 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
@@ -32519,7 +32519,7 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
@@ -32561,7 +32561,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -32599,7 +32599,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -32641,7 +32641,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -32679,7 +32679,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -32713,7 +32713,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -32755,7 +32755,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -32793,7 +32793,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
@@ -32835,7 +32835,7 @@
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
@@ -32877,7 +32877,7 @@
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G253" s="2" t="inlineStr">
@@ -32915,7 +32915,7 @@
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G254" s="2" t="inlineStr">
@@ -32953,7 +32953,7 @@
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
@@ -32991,7 +32991,7 @@
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G256" s="2" t="inlineStr">
@@ -33029,7 +33029,7 @@
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
@@ -33071,7 +33071,7 @@
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
@@ -33109,7 +33109,7 @@
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
@@ -33143,7 +33143,7 @@
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
@@ -33181,7 +33181,7 @@
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
@@ -33219,7 +33219,7 @@
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
@@ -33257,7 +33257,7 @@
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
@@ -33299,7 +33299,7 @@
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G264" s="2" t="inlineStr">
@@ -33341,7 +33341,7 @@
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
@@ -33379,7 +33379,7 @@
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G266" s="2" t="inlineStr">
@@ -33421,7 +33421,7 @@
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G267" s="2" t="inlineStr">
@@ -33455,7 +33455,7 @@
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G268" s="2" t="inlineStr">
@@ -33493,7 +33493,7 @@
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G269" s="2" t="inlineStr">
@@ -33531,7 +33531,7 @@
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G270" s="2" t="inlineStr">
@@ -33569,7 +33569,7 @@
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30T14:18:21+00:00</t>
+          <t>2026-10-31T13:50:35+00:00</t>
         </is>
       </c>
       <c r="G271" s="2" t="inlineStr">

</xml_diff>